<commit_message>
CAS outstanding items: restart behaviour per FD rev B
IN-21 restart after power failure is now a PLC gap (FD Motor-Forrigling:
retained run state, sequence 1/2a-c/3). IN-27 restart after trip decided
by the FD (LOCKDOWN, operator Reset). IN-28 new decision: emergency stop
listed as an interlock with automatic restart.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAS/Outstanding items.xlsx
+++ b/CAS/Outstanding items.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Outstanding items'!$A$1:$O$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Outstanding items'!$A$1:$O$84</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O82"/>
+  <dimension ref="A1:O84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2287,7 +2287,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>PLC gap</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -2297,19 +2297,15 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>No auto-restart or staggered start; Pen Start starts all pumps at once.</t>
+          <t>FD 'Motor-Forrigling' + motor table T3/T4: motors that were running restart after a power cut, larger ones in sequence (1 hydraulic pump, 2a/2b/2c inlet pumps, 3 oxygenator pumps; vacuum J01A-C auto-restart). PLC: PenStart is not retained, so after a PLC power loss nothing restarts; if only the Framo cabinets lose power, all pumps restart together once Available. Needs a retained 'was running' state per motor and the restart sequence with delays.</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Inlet OI16</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>Auto-restart / staggered start / manual only</t>
-        </is>
-      </c>
+          <t>FD rev B 'Motor-Forrigling', Tabell T3/T4; CAS FD Inlet OI16; FB.Inlet.InletSupervisor (PenStart)</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr"/>
       <c r="I27" s="2" t="inlineStr">
         <is>
           <t>Internal</t>
@@ -2317,7 +2313,7 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>Project</t>
+          <t>Sigurd</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -2536,17 +2532,17 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>OX-01</t>
+          <t>IN-27</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Oxygen</t>
+          <t>Inlet</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Physical</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -2556,17 +2552,17 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Oxygen supplier</t>
+          <t>Restart after a pump trip</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Supplier for oxygen chosen.</t>
+          <t>Should a tripped inlet pump restart by itself?</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Project meeting 2026-10-21</t>
+          <t>FD rev B §3.2.1, Tabell 6 (LOCKDOWN), 'Motor-Forrigling'</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
@@ -2582,7 +2578,7 @@
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
@@ -2597,7 +2593,7 @@
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>Normex</t>
+          <t>Given by FD rev B: a fault gives LOCKDOWN; the operator sends Reset after fixing it; the pump then restarts while group start (Pen Start) is active. PLC complies (start request stays latched; seen in sim 2026-10-21).</t>
         </is>
       </c>
       <c r="O31" s="2" t="inlineStr">
@@ -2609,48 +2605,52 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>OX-02</t>
+          <t>IN-28</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Oxygen</t>
+          <t>Inlet</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Physical</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Missing info</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Oxygen supply and safety interface (Normex)</t>
+          <t>Emergency stop as interlock with auto-restart</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Supply type (LOX / generator / valve panel), normal and minimum supply pressure, low-supply-pressure signal, PLC-controlled master shut-off valve, non-return protection (HAZID: water back into oxygenator and O2 tank). Supply pressure is display-only in the PLC.</t>
+          <t>FD motor table lists emergency stop as the interlock for PM01-03, PU01-03 and XV01-M01, and 'Motor-Forrigling' says a motor stopped by an interlock in auto restarts automatically when the interlock clears (group start still active). Read literally, pumps restart when the E-stop is released — normally an E-stop reset requires a deliberate restart. Framo E-stops are in series across all lines.</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>HAZID oksygen; PenControl O2InjectionPressureSensor</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr"/>
+          <t>FD rev B 'Motor-Forrigling', Tabell T3; Aksjonsliste #16</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>E-stop release requires operator restart (recommended) / auto-restart as FD</t>
+        </is>
+      </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>Normex</t>
+          <t>Internal / Framo</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>Sigurd</t>
+          <t>Project</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
@@ -2674,7 +2674,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>OX-03</t>
+          <t>OX-01</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -2684,62 +2684,70 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Physical</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Inconsistency</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>O2 control valve type</t>
+          <t>Oxygen supplier</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>FD: PWM solenoid valve 'via 4-20 mA'. PLC: proportional valve 4-20 mA, 4 mA = closed, 2 s ramp. Linde photos show 'pwm_ventil'; Normex sketch (15.10.26) shows a motorised valve. Signal, stroke time, fail position, position feedback unknown.</t>
+          <t>Supplier for oxygen chosen.</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>FD §3.2.4; FB.OxySystem.OxyControl</t>
+          <t>Project meeting 2026-10-21</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr"/>
       <c r="I33" s="2" t="inlineStr">
         <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
           <t>Normex</t>
         </is>
       </c>
-      <c r="J33" s="2" t="inlineStr">
-        <is>
-          <t>Sigurd</t>
-        </is>
-      </c>
-      <c r="K33" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="L33" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M33" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="N33" s="2" t="inlineStr"/>
-      <c r="O33" s="2" t="inlineStr"/>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>OX-04</t>
+          <t>OX-02</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -2749,7 +2757,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Physical</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -2759,17 +2767,17 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>O2 flow meter</t>
+          <t>Oxygen supply and safety interface (Normex)</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Unit (kg/h or Nl/min), range and signal type. PLC and FIC work in kg/h; FD FIC in l/min.</t>
+          <t>Supply type (LOX / generator / valve panel), normal and minimum supply pressure, low-supply-pressure signal, PLC-controlled master shut-off valve, non-return protection (HAZID: water back into oxygenator and O2 tank). Supply pressure is display-only in the PLC.</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>FD Tabell 14; ConfigValues</t>
+          <t>HAZID oksygen; PenControl O2InjectionPressureSensor</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
@@ -2785,7 +2793,7 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
@@ -2804,7 +2812,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>OX-05</t>
+          <t>OX-03</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -2814,33 +2822,33 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Physical</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Missing info</t>
+          <t>Inconsistency</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Injector model and gas ratio</t>
+          <t>O2 control valve type</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>FlowMax 104.2 kg/h = Chucaotech at 15 % v/v; same model 34.7 kg/h at 5 %. Confirm model, allowed ratio, valve and flow meter range.</t>
+          <t>FD: PWM solenoid valve 'via 4-20 mA'. PLC: proportional valve 4-20 mA, 4 mA = closed, 2 s ramp. Linde photos show 'pwm_ventil'; Normex sketch (15.10.26) shows a motorised valve. Signal, stroke time, fail position, position feedback unknown.</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Oppsett innløsere CT.xlsx; ConfigValues OxySystemConfig</t>
+          <t>FD §3.2.4; FB.OxySystem.OxyControl</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr"/>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>Normex / Chucaotech</t>
+          <t>Normex</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
@@ -2850,7 +2858,7 @@
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
@@ -2869,7 +2877,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>OX-06</t>
+          <t>OX-04</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -2879,37 +2887,33 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>PLC gap</t>
+          <t>Missing info</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>High-high O2 / supersaturation shut-off</t>
+          <t>O2 flow meter</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>FD (HOLD) asks oxygenation to close on high-high O2 near the inlet. No HH or TDGP shut-off in OxyControl/InletSupervisor.</t>
+          <t>Unit (kg/h or Nl/min), range and signal type. PLC and FIC work in kg/h; FD FIC in l/min.</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>FD §3.2.4</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t>Decide limits, sensors, latching</t>
-        </is>
-      </c>
+          <t>FD Tabell 14; ConfigValues</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr"/>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>Internal</t>
+          <t>Normex</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -2919,7 +2923,7 @@
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr">
@@ -2938,7 +2942,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>OX-07</t>
+          <t>OX-05</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -2948,47 +2952,43 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Physical</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Missing info</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>O2 setpoint and unit</t>
+          <t>Injector model and gas ratio</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>8.0 mg/L is a placeholder. FD asks '% or g/l?'. Sizing sheet uses % saturation (≥80 %, 90 % at 16 °C).</t>
+          <t>FlowMax 104.2 kg/h = Chucaotech at 15 % v/v; same model 34.7 kg/h at 5 %. Confirm model, allowed ratio, valve and flow meter range.</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>FD §3.2.4; Beregningsark dimensjonering 17mars26.xlsx</t>
-        </is>
-      </c>
-      <c r="H37" s="2" t="inlineStr">
-        <is>
-          <t>mg/L vs % saturation (with temperature/salinity)</t>
-        </is>
-      </c>
+          <t>Oppsett innløsere CT.xlsx; ConfigValues OxySystemConfig</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr"/>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>Customer / biologist</t>
+          <t>Normex / Chucaotech</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>Project</t>
+          <t>Sigurd</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
@@ -3007,7 +3007,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>OX-08</t>
+          <t>OX-06</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -3022,27 +3022,27 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>PLC gap</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Loss of pen O2 measurement</t>
+          <t>High-high O2 / supersaturation shut-off</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>OIC01 holds its output indefinitely. FD sentence unfinished ('skal regulatoren…').</t>
+          <t>FD (HOLD) asks oxygenation to close on high-high O2 near the inlet. No HH or TDGP shut-off in OxyControl/InletSupervisor.</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>FD §3.2.4; FB.Inlet.InletSupervisor</t>
+          <t>FD §3.2.4</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Hold / fixed fallback flow / hold for limited time then alarm</t>
+          <t>Decide limits, sensors, latching</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -3052,7 +3052,7 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>Project</t>
+          <t>Sigurd</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
@@ -3076,7 +3076,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>OX-09</t>
+          <t>OX-07</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -3096,27 +3096,27 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Loss of line flow measurement</t>
+          <t>O2 setpoint and unit</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Line leaves auto and holds its last valve position open-loop.</t>
+          <t>8.0 mg/L is a placeholder. FD asks '% or g/l?'. Sizing sheet uses % saturation (≥80 %, 90 % at 16 °C).</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>FB.OxySystem.OxyControl</t>
+          <t>FD §3.2.4; Beregningsark dimensjonering 17mars26.xlsx</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Hold vs close valve</t>
+          <t>mg/L vs % saturation (with temperature/salinity)</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>Internal</t>
+          <t>Customer / biologist</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
@@ -3126,7 +3126,7 @@
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr">
@@ -3145,7 +3145,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>OX-10</t>
+          <t>OX-08</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -3155,43 +3155,47 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Missing info</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Pressure transmitters absolute or gauge</t>
+          <t>Loss of pen O2 measurement</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>PressureSetpoint 4.0 bar assumes absolute; ValveOpenPressure 3.0 must change together with it. Range assumed 0-10 bar. Chucaotech required inlet pressure needed.</t>
+          <t>OIC01 holds its output indefinitely. FD sentence unfinished ('skal regulatoren…').</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>OxySystemConfigDUT; ConfigValues</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="inlineStr"/>
+          <t>FD §3.2.4; FB.Inlet.InletSupervisor</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Hold / fixed fallback flow / hold for limited time then alarm</t>
+        </is>
+      </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>Normex / Chucaotech</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>Sigurd</t>
+          <t>Project</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
@@ -3210,7 +3214,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>OX-11</t>
+          <t>OX-09</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -3220,30 +3224,34 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Missing info</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>ATV650 settings</t>
+          <t>Loss of line flow measurement</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Unit id, comm-loss behaviour (FD expects hold at preset speed), 20-50 Hz and preset 40 Hz vs NX 3153 pump curve. Fault codes in PLC came from ATV320 list (NVE41316) — re-check for ATV650.</t>
+          <t>Line leaves auto and holds its last valve position open-loop.</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>ATV600-Communication-parameters-EAV64332; FB.OxySystem.OxyPumpATV650</t>
-        </is>
-      </c>
-      <c r="H41" s="2" t="inlineStr"/>
+          <t>FB.OxySystem.OxyControl</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>Hold vs close valve</t>
+        </is>
+      </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
           <t>Internal</t>
@@ -3251,7 +3259,7 @@
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>Sigurd</t>
+          <t>Project</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
@@ -3275,7 +3283,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>OX-12</t>
+          <t>OX-10</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -3285,7 +3293,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Physical</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -3295,33 +3303,33 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Ethernet to oxy pump drive cabinet</t>
+          <t>Pressure transmitters absolute or gauge</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Ethernet not drawn in 15169-874.004-DriveCabinet. DIN RJ45 socket (Bjørn) vs build into cabinets (JP).</t>
+          <t>PressureSetpoint 4.0 bar assumes absolute; ValveOpenPressure 3.0 must change together with it. Range assumed 0-10 bar. Chucaotech required inlet pressure needed.</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Mail 2026-10-16 'Drive cobinet for sideløpspumpen'</t>
+          <t>OxySystemConfigDUT; ConfigValues</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>Internal</t>
+          <t>Normex / Chucaotech</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>Project</t>
+          <t>Sigurd</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr">
@@ -3340,7 +3348,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>OX-13</t>
+          <t>OX-11</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -3350,27 +3358,27 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>PLC gap</t>
+          <t>Missing info</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>OIC01 and O2 sensor alarms</t>
+          <t>ATV650 settings</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>FD Tabell 15: OIC01 deviation from setpoint and deviation between O2 sensors — not implemented.</t>
+          <t>Unit id, comm-loss behaviour (FD expects hold at preset speed), 20-50 Hz and preset 40 Hz vs NX 3153 pump curve. Fault codes in PLC came from ATV320 list (NVE41316) — re-check for ATV650.</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>FD Tabell 15</t>
+          <t>ATV600-Communication-parameters-EAV64332; FB.OxySystem.OxyPumpATV650</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
@@ -3386,7 +3394,7 @@
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr">
@@ -3405,7 +3413,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>OX-14</t>
+          <t>OX-12</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -3415,27 +3423,27 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Physical</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Inconsistency</t>
+          <t>Missing info</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Controller units vs FD</t>
+          <t>Ethernet to oxy pump drive cabinet</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>FD: OIC01 0-100 %, three parameter sets; FIC in l/min. PLC: OIC01 total kg/h shared over lines, one set (Kp 50, Ti 1800). Deliberate — add to FD deviation list.</t>
+          <t>Ethernet not drawn in 15169-874.004-DriveCabinet. DIN RJ45 socket (Bjørn) vs build into cabinets (JP).</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>FD Tabell 13/14; FB.Inlet.InletSupervisor</t>
+          <t>Mail 2026-10-16 'Drive cobinet for sideløpspumpen'</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr"/>
@@ -3446,7 +3454,7 @@
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>Sigurd</t>
+          <t>Project</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
@@ -3470,7 +3478,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>OX-15</t>
+          <t>OX-13</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -3480,27 +3488,27 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Physical</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Missing info</t>
+          <t>PLC gap</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Orbit 864 Modbus noise / hub</t>
+          <t>OIC01 and O2 sensor alarms</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Mechatronic recommends a hub on the Orbit 864 RTU line. Hub ordered for Bergen lab?</t>
+          <t>FD Tabell 15: OIC01 deviation from setpoint and deviation between O2 sensors — not implemented.</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Mail 2026-09-21/30 'Bestilling av komponent til Lab i Bergen'</t>
+          <t>FD Tabell 15</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr"/>
@@ -3511,7 +3519,7 @@
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>Bjørn</t>
+          <t>Sigurd</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
@@ -3535,7 +3543,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>OX-16</t>
+          <t>OX-14</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -3550,22 +3558,22 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Code bug</t>
+          <t>Inconsistency</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Drive IP in ConfigValues</t>
+          <t>Controller units vs FD</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>InletRIOConfig DriveIP still 10.1.2.101; CAS simulator pod is at 10.1.2.150.</t>
+          <t>FD: OIC01 0-100 %, three parameter sets; FIC in l/min. PLC: OIC01 total kg/h shared over lines, one set (Kp 50, Ti 1800). Deliberate — add to FD deviation list.</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>PFC200_Sim ConfigValues</t>
+          <t>FD Tabell 13/14; FB.Inlet.InletSupervisor</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
@@ -3600,7 +3608,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>OX-17</t>
+          <t>OX-15</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -3615,38 +3623,38 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Missing hardware</t>
+          <t>Missing info</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Low O2 supply pressure switch / master shut-off valve</t>
+          <t>Orbit 864 Modbus noise / hub</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>No PLC input for low supply pressure and no PLC-controlled master shut-off valve on P&amp;ID or in PLC (HAZID backflow risk).</t>
+          <t>Mechatronic recommends a hub on the Orbit 864 RTU line. Hub ordered for Bergen lab?</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>HAZID oksygen; P&amp;ID rev A</t>
+          <t>Mail 2026-09-21/30 'Bestilling av komponent til Lab i Bergen'</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr"/>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>Normex</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>Sigurd</t>
+          <t>Bjørn</t>
         </is>
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="L47" s="2" t="inlineStr">
@@ -3665,7 +3673,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>OX-18</t>
+          <t>OX-16</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -3685,17 +3693,17 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>ATV650 fault codes from ATV320 list</t>
+          <t>Drive IP in ConfigValues</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>OxyPumpATV650 decodes LFT with ATV320 (NVE41316) codes (e.g. 16 OHF, 17 OLF, 22 USF). Verify against ATV600 list EAV64332.</t>
+          <t>InletRIOConfig DriveIP still 10.1.2.101; CAS simulator pod is at 10.1.2.150.</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>FB.OxySystem.OxyPumpATV650</t>
+          <t>PFC200_Sim ConfigValues</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -3711,12 +3719,12 @@
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="M48" s="2" t="inlineStr">
@@ -3724,21 +3732,13 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="N48" s="2" t="inlineStr">
-        <is>
-          <t>Checked 2026-10-21 (CAS FD Oxygen): register addresses and fault codes match ATV600 EAV64332. Verify on the real drive at commissioning; program design/design basis still say ATV320.</t>
-        </is>
-      </c>
-      <c r="O48" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
+      <c r="N48" s="2" t="inlineStr"/>
+      <c r="O48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>OX-19</t>
+          <t>OX-17</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -3753,32 +3753,28 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Inconsistency</t>
+          <t>Missing hardware</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Side-stream pump head vs 4 bar setpoint</t>
+          <t>Low O2 supply pressure switch / master shut-off valve</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Flygt NX 3153 datasheet: 10.2 m head at duty point, 18.3 m at shut-off (≈1-1.8 bar) — cannot give 4.0 bar after the pump. Simulator assumes 4.5 bar rise.</t>
+          <t>No PLC input for low supply pressure and no PLC-controlled master shut-off valve on P&amp;ID or in PLC (HAZID backflow risk).</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Oxygen OI18; NX 3153 datasheet; design_basis.toml</t>
-        </is>
-      </c>
-      <c r="H49" s="2" t="inlineStr">
-        <is>
-          <t>Confirm pump, injector inlet pressure and setpoint</t>
-        </is>
-      </c>
+          <t>HAZID oksygen; P&amp;ID rev A</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr"/>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>Normex / Chucaotech</t>
+          <t>Normex</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
@@ -3807,7 +3803,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>OX-20</t>
+          <t>OX-18</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -3827,24 +3823,20 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Bad flow measurement causes over-dosing</t>
+          <t>ATV650 fault codes from ATV320 list</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>When a line's flow measurement is bad its flow counts as 0 in the sharing while its valve stays where it was — other lines add the same flow again.</t>
+          <t>OxyPumpATV650 decodes LFT with ATV320 (NVE41316) codes (e.g. 16 OHF, 17 OLF, 22 USF). Verify against ATV600 list EAV64332.</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Oxygen OI15; FB.Inlet.InletSupervisor</t>
-        </is>
-      </c>
-      <c r="H50" s="2" t="inlineStr">
-        <is>
-          <t>Use last good flow or close the valve</t>
-        </is>
-      </c>
+          <t>FB.OxySystem.OxyPumpATV650</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr"/>
       <c r="I50" s="2" t="inlineStr">
         <is>
           <t>Internal</t>
@@ -3857,12 +3849,12 @@
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="M50" s="2" t="inlineStr">
@@ -3870,13 +3862,21 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="N50" s="2" t="inlineStr"/>
-      <c r="O50" s="2" t="inlineStr"/>
+      <c r="N50" s="2" t="inlineStr">
+        <is>
+          <t>Checked 2026-10-21 (CAS FD Oxygen): register addresses and fault codes match ATV600 EAV64332. Verify on the real drive at commissioning; program design/design basis still say ATV320.</t>
+        </is>
+      </c>
+      <c r="O50" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>OX-21</t>
+          <t>OX-19</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -3886,38 +3886,42 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Physical</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Missing hardware</t>
+          <t>Inconsistency</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Emergency stop to oxygen system</t>
+          <t>Side-stream pump head vs 4 bar setpoint</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>No E-stop input wired to the Heimdall PLC; oxygen stop on E-stop not possible.</t>
+          <t>Flygt NX 3153 datasheet: 10.2 m head at duty point, 18.3 m at shut-off (≈1-1.8 bar) — cannot give 4.0 bar after the pump. Simulator assumes 4.5 bar rise.</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Oxygen OI22; CAS FD Inlet OI13</t>
-        </is>
-      </c>
-      <c r="H51" s="2" t="inlineStr"/>
+          <t>CAS FD Oxygen OI18; NX 3153 datasheet; design_basis.toml</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>Confirm pump, injector inlet pressure and setpoint</t>
+        </is>
+      </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>Internal</t>
+          <t>Normex / Chucaotech</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>Project</t>
+          <t>Sigurd</t>
         </is>
       </c>
       <c r="K51" s="2" t="inlineStr">
@@ -3941,7 +3945,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>OX-22</t>
+          <t>OX-20</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -3951,32 +3955,32 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Missing info</t>
+          <t>Code bug</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>ATV650 comm-loss behaviour</t>
+          <t>Bad flow measurement causes over-dosing</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Factory default on lost PLC link is freewheel stop; FD wants hold at preset speed (fallback speed / speed maintain).</t>
+          <t>When a line's flow measurement is bad its flow counts as 0 in the sharing while its valve stays where it was — other lines add the same flow again.</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Oxygen OI19</t>
+          <t>CAS FD Oxygen OI15; FB.Inlet.InletSupervisor</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>Set ETHL fallback speed</t>
+          <t>Use last good flow or close the valve</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
@@ -3991,7 +3995,7 @@
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="L52" s="2" t="inlineStr">
@@ -4010,7 +4014,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>OX-23</t>
+          <t>OX-21</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -4020,27 +4024,27 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>PLC gap</t>
+          <t>Missing hardware</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Low pressure-drop alarm over injector</t>
+          <t>Emergency stop to oxygen system</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>OxynatorOutletPressure is read but unused; no low dP alarm.</t>
+          <t>No E-stop input wired to the Heimdall PLC; oxygen stop on E-stop not possible.</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Oxygen OI10</t>
+          <t>CAS FD Oxygen OI22; CAS FD Inlet OI13</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr"/>
@@ -4051,12 +4055,12 @@
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>Sigurd</t>
+          <t>Project</t>
         </is>
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="L53" s="2" t="inlineStr">
@@ -4075,7 +4079,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>OX-24</t>
+          <t>OX-22</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -4090,25 +4094,29 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>PLC gap</t>
+          <t>Missing info</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Pump leakage / temperature contacts unused</t>
+          <t>ATV650 comm-loss behaviour</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Side-stream pump leakage/temperature contacts exist on RIO1 only and are not used in the logic.</t>
+          <t>Factory default on lost PLC link is freewheel stop; FD wants hold at preset speed (fallback speed / speed maintain).</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Oxygen OI24</t>
-        </is>
-      </c>
-      <c r="H54" s="2" t="inlineStr"/>
+          <t>CAS FD Oxygen OI19</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>Set ETHL fallback speed</t>
+        </is>
+      </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
           <t>Internal</t>
@@ -4140,7 +4148,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>OX-25</t>
+          <t>OX-23</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -4150,33 +4158,33 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Physical</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Inconsistency</t>
+          <t>PLC gap</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>O2 supply pressure</t>
+          <t>Low pressure-drop alarm over injector</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Normex sketch '2.5 bar ?' vs Linde sheet 10 bar.</t>
+          <t>OxynatorOutletPressure is read but unused; no low dP alarm.</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Oxygen OI1; Normex sketch 15.10.26</t>
+          <t>CAS FD Oxygen OI10</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>Normex</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr">
@@ -4205,7 +4213,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>OX-26</t>
+          <t>OX-24</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -4215,27 +4223,27 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Physical</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>PLC gap</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Oxygen capacity with one inlet pump out</t>
+          <t>Pump leakage / temperature contacts unused</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Two lines must carry the full oxygen demand (~560-730 t biomass) when one inlet pump is out.</t>
+          <t>Side-stream pump leakage/temperature contacts exist on RIO1 only and are not used in the logic.</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Oxygen OI26; sizing sheet</t>
+          <t>CAS FD Oxygen OI24</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr"/>
@@ -4246,7 +4254,7 @@
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>Project</t>
+          <t>Sigurd</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr">
@@ -4270,7 +4278,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>OX-27</t>
+          <t>OX-25</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -4280,33 +4288,33 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Physical</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Code bug</t>
+          <t>Inconsistency</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>PT40 variable name</t>
+          <t>O2 supply pressure</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Supply pressure transmitter has the wrong variable name in the PLC vs P&amp;ID PT40.</t>
+          <t>Normex sketch '2.5 bar ?' vs Linde sheet 10 bar.</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Oxygen OI4</t>
+          <t>CAS FD Oxygen OI1; Normex sketch 15.10.26</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr"/>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>Internal</t>
+          <t>Normex</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr">
@@ -4316,7 +4324,7 @@
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L57" s="2" t="inlineStr">
@@ -4335,17 +4343,17 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>OUT-01</t>
+          <t>OX-26</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Outlet</t>
+          <t>Oxygen</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Physical</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -4355,24 +4363,20 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Outlet on power loss</t>
+          <t>Oxygen capacity with one inlet pump out</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Should the outlet close automatically on power loss (FD rev B) — accumulator, backup power for the pump, or manual?</t>
+          <t>Two lines must carry the full oxygen demand (~560-730 t biomass) when one inlet pump is out.</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>FD §3.2.3; Servi Q&amp;A; mail 'Automatisk stenging' 28.09</t>
-        </is>
-      </c>
-      <c r="H58" s="2" t="inlineStr">
-        <is>
-          <t>Accumulator / backup power / manual hand pump</t>
-        </is>
-      </c>
+          <t>CAS FD Oxygen OI26; sizing sheet</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr"/>
       <c r="I58" s="2" t="inlineStr">
         <is>
           <t>Internal</t>
@@ -4385,12 +4389,12 @@
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L58" s="2" t="inlineStr">
         <is>
-          <t>Decided</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="M58" s="2" t="inlineStr">
@@ -4398,71 +4402,59 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="N58" s="2" t="inlineStr">
-        <is>
-          <t>No automatic close. Dampers hold position; operator overrides with the HPU hand pump. Accumulator deferred — space for retrofit.</t>
-        </is>
-      </c>
-      <c r="O58" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
+      <c r="N58" s="2" t="inlineStr"/>
+      <c r="O58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>OUT-02</t>
+          <t>OX-27</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Outlet</t>
+          <t>Oxygen</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Missing hardware</t>
+          <t>Code bug</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Pressure transmitters per cylinder (8 → 4)</t>
+          <t>PT40 variable name</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Servi drawing A1 (2939238) has one PT per cylinder (1PT1-1PT4, 0-250 bar, A/plus line). FD PT61-68 and PLC (PressureOpen + PressureClose, 8 AIs) expect two. End position confirmable in one direction only.</t>
+          <t>Supply pressure transmitter has the wrong variable name in the PLC vs P&amp;ID PT40.</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Servi A1; FD §3.2.3; CylinderInputDUT; mail Bjørn 2026-10-19</t>
-        </is>
-      </c>
-      <c r="H59" s="2" t="inlineStr">
-        <is>
-          <t>Buy 2nd PT (Minimess point, Servi offer) / detect end-of-stroke by pulses stopping</t>
-        </is>
-      </c>
+          <t>CAS FD Oxygen OI4</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr"/>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>Servi</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>Bjørn</t>
+          <t>Sigurd</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="L59" s="2" t="inlineStr">
@@ -4481,7 +4473,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>OUT-03</t>
+          <t>OUT-01</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -4491,38 +4483,42 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Physical</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Missing info</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Plus stroke direction</t>
+          <t>Outlet on power loss</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Does plus stroke (A, extend) open or close the damper? Decides which end has the PT and the counter direction.</t>
+          <t>Should the outlet close automatically on power loss (FD rev B) — accumulator, backup power for the pump, or manual?</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Servi A1</t>
-        </is>
-      </c>
-      <c r="H60" s="2" t="inlineStr"/>
+          <t>FD §3.2.3; Servi Q&amp;A; mail 'Automatisk stenging' 28.09</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>Accumulator / backup power / manual hand pump</t>
+        </is>
+      </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>Østerbø / Servi</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>Bjørn</t>
+          <t>Project</t>
         </is>
       </c>
       <c r="K60" s="2" t="inlineStr">
@@ -4532,7 +4528,7 @@
       </c>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Decided</t>
         </is>
       </c>
       <c r="M60" s="2" t="inlineStr">
@@ -4540,13 +4536,21 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="N60" s="2" t="inlineStr"/>
-      <c r="O60" s="2" t="inlineStr"/>
+      <c r="N60" s="2" t="inlineStr">
+        <is>
+          <t>No automatic close. Dampers hold position; operator overrides with the HPU hand pump. Accumulator deferred — space for retrofit.</t>
+        </is>
+      </c>
+      <c r="O60" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>OUT-04</t>
+          <t>OUT-02</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -4561,25 +4565,29 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>PLC gap</t>
+          <t>Missing hardware</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Junction box signals not mapped</t>
+          <t>Pressure transmitters per cylinder (8 → 4)</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>JB 18068: pump on backup/normal power (K1/K2), filter clogged, E-stop loop, local Start/Stop panel ST-16183, motor running feedback, power-lost relay (action 82). PLC maps only StarterFault, HydraulicOilTankFault, EStop + Start/Reset.</t>
+          <t>Servi drawing A1 (2939238) has one PT per cylinder (1PT1-1PT4, 0-250 bar, A/plus line). FD PT61-68 and PLC (PressureOpen + PressureClose, 8 AIs) expect two. End position confirmable in one direction only.</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Servi JB 18068 A2/A3; FB.RIO.CommonRIO</t>
-        </is>
-      </c>
-      <c r="H61" s="2" t="inlineStr"/>
+          <t>Servi A1; FD §3.2.3; CylinderInputDUT; mail Bjørn 2026-10-19</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>Buy 2nd PT (Minimess point, Servi offer) / detect end-of-stroke by pulses stopping</t>
+        </is>
+      </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
           <t>Servi</t>
@@ -4611,7 +4619,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>OUT-05</t>
+          <t>OUT-03</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -4621,33 +4629,33 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Physical</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>PLC gap</t>
+          <t>Missing info</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Power-lost alarm to operator</t>
+          <t>Plus stroke direction</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>With manual override decided, operator must be alarmed on power loss. Needs the Servi power-lost / backup-power relay as a PLC input.</t>
+          <t>Does plus stroke (A, extend) open or close the damper? Decides which end has the PT and the counter direction.</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Decision 2026-10-21; action item 82</t>
+          <t>Servi A1</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr"/>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>Servi</t>
+          <t>Østerbø / Servi</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
@@ -4676,7 +4684,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>OUT-06</t>
+          <t>OUT-04</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -4691,28 +4699,28 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>PLC gap</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Hydraulic pump control authority</t>
+          <t>Junction box signals not mapped</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Pump is DOL (start/reset DO, StarterFault DI, no running feedback). Local start/stop panel offered by Servi but not ordered. Local vs PLC authority; hard-wired low-oil stop?</t>
+          <t>JB 18068: pump on backup/normal power (K1/K2), filter clogged, E-stop loop, local Start/Stop panel ST-16183, motor running feedback, power-lost relay (action 82). PLC maps only StarterFault, HydraulicOilTankFault, EStop + Start/Reset.</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Servi mail 2026-10-01; OutletControl.HydraulicPumpControl</t>
+          <t>Servi JB 18068 A2/A3; FB.RIO.CommonRIO</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr"/>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>Internal / Servi</t>
+          <t>Servi</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
@@ -4722,7 +4730,7 @@
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="L63" s="2" t="inlineStr">
@@ -4741,7 +4749,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>OUT-07</t>
+          <t>OUT-05</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -4751,33 +4759,33 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Code bug</t>
+          <t>PLC gap</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Pump not stopped on oil tank fault</t>
+          <t>Power-lost alarm to operator</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>PLC only alarms on HydraulicOilTankFault (low level / 70 °C); pump start not gated.</t>
+          <t>With manual override decided, operator must be alarmed on power loss. Needs the Servi power-lost / backup-power relay as a PLC input.</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>OutletControl.HydraulicPumpControl</t>
+          <t>Decision 2026-10-21; action item 82</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr"/>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>Internal</t>
+          <t>Servi</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -4787,7 +4795,7 @@
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="L64" s="2" t="inlineStr">
@@ -4806,7 +4814,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>OUT-08</t>
+          <t>OUT-06</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -4816,33 +4824,33 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>PLC gap</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>Outlet E-stop and other alarms</t>
+          <t>Hydraulic pump control authority</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>No E-stop alarm (ES61 in alarm list); no filter, pump overload or power-loss alarms.</t>
+          <t>Pump is DOL (start/reset DO, StarterFault DI, no running feedback). Local start/stop panel offered by Servi but not ordered. Local vs PLC authority; hard-wired low-oil stop?</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>FD-02 alarm list; OutletControl.AlarmHandling</t>
+          <t>Servi mail 2026-10-01; OutletControl.HydraulicPumpControl</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr"/>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>Internal</t>
+          <t>Internal / Servi</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
@@ -4871,7 +4879,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>OUT-09</t>
+          <t>OUT-07</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -4881,37 +4889,33 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Physical</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Inconsistency</t>
+          <t>Code bug</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Flow meter signal type</t>
+          <t>Pump not stopped on oil tank fault</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>JB overview sheet labels FT1-4 '24VDC 4-20MA'; sheet A2 says pulse. PLC assumes pulse (750-638).</t>
+          <t>PLC only alarms on HydraulicOilTankFault (low level / 70 °C); pump start not gated.</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Servi JB 18068</t>
-        </is>
-      </c>
-      <c r="H66" s="2" t="inlineStr">
-        <is>
-          <t>Servi to correct overview sheet</t>
-        </is>
-      </c>
+          <t>OutletControl.HydraulicPumpControl</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr"/>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>Servi</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
@@ -4940,7 +4944,7 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>OUT-10</t>
+          <t>OUT-08</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -4955,22 +4959,22 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Code bug</t>
+          <t>PLC gap</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Mode openings look reversed</t>
+          <t>Outlet E-stop and other alarms</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>OutletConfig.ModePosition default [20,30,40,50] % gives O-35 (34 000 m3/h) the smallest opening and S-75 the largest. FD column 'Spjeld-åpning %' empty.</t>
+          <t>No E-stop alarm (ES61 in alarm list); no filter, pump overload or power-loss alarms.</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>ConfigValues OutletConfig; FD Tabell 10</t>
+          <t>FD-02 alarm list; OutletControl.AlarmHandling</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr"/>
@@ -5005,7 +5009,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>OUT-11</t>
+          <t>OUT-09</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -5015,32 +5019,32 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Physical</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Missing info</t>
+          <t>Inconsistency</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Stroke time and travel limits</t>
+          <t>Flow meter signal type</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>MaxTravelTimeOpen/Close 30 s = assumed stroke time (no margin). Estimate: one cylinder 5-7 s, four sharing the pump 20-26 s. FD 'ca nn s'.</t>
+          <t>JB overview sheet labels FT1-4 '24VDC 4-20MA'; sheet A2 says pulse. PLC assumes pulse (750-638).</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>OutletConfig; design_basis.toml; Servi A1</t>
+          <t>Servi JB 18068</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>Fill in at FAT</t>
+          <t>Servi to correct overview sheet</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
@@ -5074,7 +5078,7 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>OUT-12</t>
+          <t>OUT-10</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -5084,33 +5088,33 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Physical</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Missing info</t>
+          <t>Code bug</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>PSL valves driven on/off</t>
+          <t>Mode openings look reversed</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>HAWE PSL are proportional; PLC drives them on/off via relays (750-1515). Confirm with Servi (min ~250 mA note, optional speed card) and relay rating.</t>
+          <t>OutletConfig.ModePosition default [20,30,40,50] % gives O-35 (34 000 m3/h) the smallest opening and S-75 the largest. FD column 'Spjeld-åpning %' empty.</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>Servi A1; CommonRIO output mapping</t>
+          <t>ConfigValues OutletConfig; FD Tabell 10</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr"/>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>Servi</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
@@ -5139,7 +5143,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>OUT-13</t>
+          <t>OUT-11</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -5159,23 +5163,27 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Outputs on remote I/O comm loss</t>
+          <t>Stroke time and travel limits</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>FD table empty; 750-1515 watchdog behaviour not set.</t>
+          <t>MaxTravelTimeOpen/Close 30 s = assumed stroke time (no margin). Estimate: one cylinder 5-7 s, four sharing the pump 20-26 s. FD 'ca nn s'.</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>FD §3.2.3</t>
-        </is>
-      </c>
-      <c r="H70" s="2" t="inlineStr"/>
+          <t>OutletConfig; design_basis.toml; Servi A1</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>Fill in at FAT</t>
+        </is>
+      </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>Internal</t>
+          <t>Servi</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -5204,7 +5212,7 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>OUT-14</t>
+          <t>OUT-12</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -5224,33 +5232,33 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Shut-off valve XV65</t>
+          <t>PSL valves driven on/off</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>In FD and PLS action list 6.3 ('Stopp-ventil') but not on Servi A1 or in the PLC. Deferred with the accumulator?</t>
+          <t>HAWE PSL are proportional; PLC drives them on/off via relays (750-1515). Confirm with Servi (min ~250 mA note, optional speed card) and relay rating.</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>FD §3.2.3; PLS aksjonsliste 6.3</t>
+          <t>Servi A1; CommonRIO output mapping</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr"/>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>Internal</t>
+          <t>Servi</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>Project</t>
+          <t>Bjørn</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L71" s="2" t="inlineStr">
@@ -5269,7 +5277,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>OUT-15</t>
+          <t>OUT-13</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -5279,33 +5287,33 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Physical</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Inconsistency</t>
+          <t>Missing info</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Motor and pressure data</t>
+          <t>Outputs on remote I/O comm loss</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Motor 1.5 kW 400 V (datasheet, A1) vs &lt;1 kW (Q&amp;A); cable W1M1 'Hydraulic motor 24Vdc'. Relief 150/130 bar (A1) vs 160 bar in simulator, 110 bar (T1). Tank 12 l (A1 part list) vs 10 l; cylinder HRC-N-D vs HCR-C-D; motor starter location (action 91).</t>
+          <t>FD table empty; 750-1515 watchdog behaviour not set.</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Servi A1, Q&amp;A, JB 18068; design_basis.toml</t>
+          <t>FD §3.2.3</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr"/>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>Servi</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -5315,7 +5323,7 @@
       </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L72" s="2" t="inlineStr">
@@ -5334,7 +5342,7 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>OUT-16</t>
+          <t>OUT-14</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -5354,24 +5362,20 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>Counter frequency</t>
+          <t>Shut-off valve XV65</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>~300 Hz at 3.5 l/min and ~5200 pulses/l; minus stroke of one cylinder pushes 4.7-5.4 l/min through its A-line meter (~410-470 Hz), near the QG100 top and the 750-638 500 Hz limit. Reverse-flow accuracy unknown.</t>
+          <t>In FD and PLS action list 6.3 ('Stopp-ventil') but not on Servi A1 or in the PLC. Deferred with the accumulator?</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>HySense QG datasheet; 750-638 manual; CAS FD Outlet OI11</t>
-        </is>
-      </c>
-      <c r="H73" s="2" t="inlineStr">
-        <is>
-          <t>Test at FAT</t>
-        </is>
-      </c>
+          <t>FD §3.2.3; PLS aksjonsliste 6.3</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr"/>
       <c r="I73" s="2" t="inlineStr">
         <is>
           <t>Internal</t>
@@ -5379,12 +5383,12 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>Bjørn</t>
+          <t>Project</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="L73" s="2" t="inlineStr">
@@ -5403,7 +5407,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>OUT-17</t>
+          <t>OUT-15</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -5418,38 +5422,38 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Inconsistency</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Integrated FAT at Østerbø</t>
+          <t>Motor and pressure data</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>Integrated test of our control cabinet with Servi's hydraulic cabinet, end of October: scope, hose lengths, fail-safe and hand pump test.</t>
+          <t>Motor 1.5 kW 400 V (datasheet, A1) vs &lt;1 kW (Q&amp;A); cable W1M1 'Hydraulic motor 24Vdc'. Relief 150/130 bar (A1) vs 160 bar in simulator, 110 bar (T1). Tank 12 l (A1 part list) vs 10 l; cylinder HRC-N-D vs HCR-C-D; motor starter location (action 91).</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Mail Fredrik 2026-10-07</t>
+          <t>Servi A1, Q&amp;A, JB 18068; design_basis.toml</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr"/>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>Østerbø / Servi</t>
+          <t>Servi</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>Project</t>
+          <t>Bjørn</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="L74" s="2" t="inlineStr">
@@ -5468,7 +5472,7 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>OUT-18</t>
+          <t>OUT-16</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -5478,32 +5482,32 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Physical</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Code bug</t>
+          <t>Missing info</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Close never confirmed without 2nd pressure transmitter</t>
+          <t>Counter frequency</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>With MaxPressureClose &gt; 0 on an unwired channel a 0 % setpoint never reaches Closed → travel timeout and fault; with 0 the end-position check is disabled. CalibrateOpen also needs Opened by pressure.</t>
+          <t>~300 Hz at 3.5 l/min and ~5200 pulses/l; minus stroke of one cylinder pushes 4.7-5.4 l/min through its A-line meter (~410-470 Hz), near the QG100 top and the 750-638 500 Hz limit. Reverse-flow accuracy unknown.</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>FB.Outlet.OutletControl; CylinderInputDUT</t>
+          <t>HySense QG datasheet; 750-638 manual; CAS FD Outlet OI11</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>Depends on OUT PT decision</t>
+          <t>Test at FAT</t>
         </is>
       </c>
       <c r="I75" s="2" t="inlineStr">
@@ -5518,7 +5522,7 @@
       </c>
       <c r="K75" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L75" s="2" t="inlineStr">
@@ -5537,7 +5541,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>OUT-19</t>
+          <t>OUT-17</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -5552,38 +5556,38 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Missing hardware</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Hydraulic pump running feedback</t>
+          <t>Integrated FAT at Østerbø</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>Pump is DOL; PLC has no running feedback (Status.Running = start command). Contactor auxiliary contact available in JB 18068?</t>
+          <t>Integrated test of our control cabinet with Servi's hydraulic cabinet, end of October: scope, hose lengths, fail-safe and hand pump test.</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>OutletControl.HydraulicPumpControl; Servi JB 18068</t>
+          <t>Mail Fredrik 2026-10-07</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>Servi</t>
+          <t>Østerbø / Servi</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>Bjørn</t>
+          <t>Project</t>
         </is>
       </c>
       <c r="K76" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="L76" s="2" t="inlineStr">
@@ -5602,7 +5606,7 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>OUT-20</t>
+          <t>OUT-18</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -5622,20 +5626,24 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>End-position pressure limit cannot trip</t>
+          <t>Close never confirmed without 2nd pressure transmitter</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Servi A1 port pressure limiters are 100 bar; PLC end-position limit is also 100 bar with strict '&gt;'. Set ~70-80 bar after FAT; align simulator (160 bar).</t>
+          <t>With MaxPressureClose &gt; 0 on an unwired channel a 0 % setpoint never reaches Closed → travel timeout and fault; with 0 the end-position check is disabled. CalibrateOpen also needs Opened by pressure.</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Outlet OI3; Servi A1; OutletConfig</t>
-        </is>
-      </c>
-      <c r="H77" s="2" t="inlineStr"/>
+          <t>FB.Outlet.OutletControl; CylinderInputDUT</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>Depends on OUT PT decision</t>
+        </is>
+      </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
           <t>Internal</t>
@@ -5667,7 +5675,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>OUT-21</t>
+          <t>OUT-19</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -5677,33 +5685,33 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Physical</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Code bug</t>
+          <t>Missing hardware</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Pressure scaling 0-250 bar</t>
+          <t>Hydraulic pump running feedback</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Production pressure scaling must be 0-250 bar; DUT default is 0-10.</t>
+          <t>Pump is DOL; PLC has no running feedback (Status.Running = start command). Contactor auxiliary contact available in JB 18068?</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Outlet OI4</t>
+          <t>OutletControl.HydraulicPumpControl; Servi JB 18068</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr"/>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>Internal</t>
+          <t>Servi</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
@@ -5732,7 +5740,7 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>OUT-22</t>
+          <t>OUT-20</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -5752,17 +5760,17 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Default span treated as calibrated</t>
+          <t>End-position pressure limit cannot trip</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>Default span 0-2000 counts counts as calibrated; calibration must be a commissioning step. FaultReset unused.</t>
+          <t>Servi A1 port pressure limiters are 100 bar; PLC end-position limit is also 100 bar with strict '&gt;'. Set ~70-80 bar after FAT; align simulator (160 bar).</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Outlet OI15</t>
+          <t>CAS FD Outlet OI3; Servi A1; OutletConfig</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr"/>
@@ -5778,7 +5786,7 @@
       </c>
       <c r="K79" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="L79" s="2" t="inlineStr">
@@ -5797,7 +5805,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>OUT-23</t>
+          <t>OUT-21</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -5807,33 +5815,33 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Inconsistency</t>
+          <t>Code bug</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>PLC Reset output has no JB counterpart</t>
+          <t>Pressure scaling 0-250 bar</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>PLC drives a pump Reset output; JB 18068 has no matching input. DI -R1-017 / DO -R1-020 wiring needed.</t>
+          <t>Production pressure scaling must be 0-250 bar; DUT default is 0-10.</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Outlet OI7; JB 18068</t>
+          <t>CAS FD Outlet OI4</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr"/>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>Servi</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
@@ -5862,7 +5870,7 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>OUT-24</t>
+          <t>OUT-22</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -5872,27 +5880,27 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Physical</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>Missing info</t>
+          <t>Code bug</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>Manual override procedure (O&amp;M)</t>
+          <t>Default span treated as calibrated</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>Hand pump and PSL manual levers, plus weekly end-position exercise, to be written into the O&amp;M manual.</t>
+          <t>Default span 0-2000 counts counts as calibrated; calibration must be a commissioning step. FaultReset unused.</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Outlet OI17; decision 2026-10-21</t>
+          <t>CAS FD Outlet OI15</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr"/>
@@ -5903,7 +5911,7 @@
       </c>
       <c r="J81" s="2" t="inlineStr">
         <is>
-          <t>Project</t>
+          <t>Bjørn</t>
         </is>
       </c>
       <c r="K81" s="2" t="inlineStr">
@@ -5927,7 +5935,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>OUT-25</t>
+          <t>OUT-23</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -5942,28 +5950,28 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Missing info</t>
+          <t>Inconsistency</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Position drift limit</t>
+          <t>PLC Reset output has no JB counterpart</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>Drift limit of 2 pulses (HOLD in FD) to be verified at FAT.</t>
+          <t>PLC drives a pump Reset output; JB 18068 has no matching input. DI -R1-017 / DO -R1-020 wiring needed.</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Outlet OI18</t>
+          <t>CAS FD Outlet OI7; JB 18068</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr"/>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>Internal</t>
+          <t>Servi</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr">
@@ -5973,7 +5981,7 @@
       </c>
       <c r="K82" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L82" s="2" t="inlineStr">
@@ -5989,8 +5997,138 @@
       <c r="N82" s="2" t="inlineStr"/>
       <c r="O82" s="2" t="inlineStr"/>
     </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>OUT-24</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>Outlet</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>Physical</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>Missing info</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>Manual override procedure (O&amp;M)</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>Hand pump and PSL manual levers, plus weekly end-position exercise, to be written into the O&amp;M manual.</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>CAS FD Outlet OI17; decision 2026-10-21</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr"/>
+      <c r="I83" s="2" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="K83" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L83" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M83" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="N83" s="2" t="inlineStr"/>
+      <c r="O83" s="2" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>OUT-25</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Outlet</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>Missing info</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>Position drift limit</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>Drift limit of 2 pulses (HOLD in FD) to be verified at FAT.</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>CAS FD Outlet OI18</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr"/>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>Bjørn</t>
+        </is>
+      </c>
+      <c r="K84" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L84" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M84" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="N84" s="2" t="inlineStr"/>
+      <c r="O84" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O82"/>
+  <autoFilter ref="A1:O84"/>
   <conditionalFormatting sqref="K2:K500">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"High"</formula>

</xml_diff>

<commit_message>
CAS: inlet Reset to Framo (FD Inlet rev A1, register IN-03/IN-29/IN-30)
FD Inlet A1: Reset held until the state change is seen, warning Failed to
reset after 2 x ResetExpectedTime (alarm, fault and parameter tables),
HOLD->REMOTE open issue reworded (the PLC follows the PCC either way),
OI24 HMI Reset button. Register: IN-03 updated; IN-29 PLC Reset handling
and IN-30 HMI Reset button (PR heimdall-cas-hmi#5), both in progress.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAS/Outstanding items.xlsx
+++ b/CAS/Outstanding items.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Outstanding items'!$A$1:$O$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Outstanding items'!$A$1:$O$86</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O84"/>
+  <dimension ref="A1:O86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -965,12 +965,12 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Framo rev B: HOLD returns to REMOTE automatically when heartbeat is back; LOCKDOWN exits on 'Sequence END'. FD Tabell 5 and PLC (D3) require operator Reset.</t>
+          <t>Framo rev B: HOLD returns to REMOTE automatically when heartbeat is back; LOCKDOWN exits on 'Sequence END'. FD Tabell 5 requires operator Reset. The PLC works either way: it follows the state the PCC reports (LIC01 frozen in HOLD, bumpless resume in REMOTE) and sends Reset only on the operator's command (since 2026-10-21 held until the state change is seen; warning FailedToReset after 2 x ResetExpectedTime). Open with Framo: which behaviour the PCC implements, edge or level on Reset, and whether the PCC panel has its own local Reset.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>FD Tabell 5; Framo spec rev B state diagram</t>
+          <t>FD Tabell 5; Framo spec rev B state diagram; FB.Inlet.InletControl; CAS FD Inlet rev A1 OI2/OI3</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -2674,37 +2674,37 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>OX-01</t>
+          <t>IN-29</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Oxygen</t>
+          <t>Inlet</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Physical</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>PLC gap</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Oxygen supplier</t>
+          <t>Reset to Framo held until state change</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Supplier for oxygen chosen.</t>
+          <t>HMI Reset was passed straight through as a level and never cleared by the PLC; a 1 s HMI pulse could be lost in the OPC UA data source.</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Project meeting 2026-10-21</t>
+          <t>FB.Inlet.InletControl; InletConfigDUT.ResetExpectedTime; InletPumpAlarmDUT.FailedToReset</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr"/>
@@ -2715,17 +2715,17 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>Project</t>
+          <t>Sigurd</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>Decided</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr">
@@ -2735,55 +2735,51 @@
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>Normex</t>
-        </is>
-      </c>
-      <c r="O33" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
+          <t>Implemented 2026-10-21 in CODESYS (not yet staged/compiled/tested): Command.Reset accepted in HOLD/LOCKDOWN, latched as ResetRequest, cleared when the state change is seen; no change within 2 x ResetExpectedTime (5 s) -&gt; Reset withdrawn and warning FailedToReset (auto-acknowledged).</t>
+        </is>
+      </c>
+      <c r="O33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>OX-02</t>
+          <t>IN-30</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Oxygen</t>
+          <t>Inlet</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Physical</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Missing info</t>
+          <t>PLC gap</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Oxygen supply and safety interface (Normex)</t>
+          <t>Reset button on the HMI</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Supply type (LOX / generator / valve panel), normal and minimum supply pressure, low-supply-pressure signal, PLC-controlled master shut-off valve, non-return protection (HAZID: water back into oxygenator and O2 tank). Supply pressure is display-only in the PLC.</t>
+          <t>No way for the operator to give Reset to the Framo controller (FD 3.2.1: Reset from the HMI).</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>HAZID oksygen; PenControl O2InjectionPressureSensor</t>
+          <t>heimdall-cas-hmi PR #5 (task/inlet-pump-reset-button); CAS FD Inlet OI24</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>Normex</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -2793,12 +2789,12 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr">
@@ -2806,13 +2802,17 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="N34" s="2" t="inlineStr"/>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>Test HMI: Reset button per inlet pump, enabled in HOLD/LOCKDOWN, with confirmation (PR #5, open). Production HMI needs the same.</t>
+        </is>
+      </c>
       <c r="O34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>OX-03</t>
+          <t>OX-01</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -2822,62 +2822,70 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Physical</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Inconsistency</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>O2 control valve type</t>
+          <t>Oxygen supplier</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>FD: PWM solenoid valve 'via 4-20 mA'. PLC: proportional valve 4-20 mA, 4 mA = closed, 2 s ramp. Linde photos show 'pwm_ventil'; Normex sketch (15.10.26) shows a motorised valve. Signal, stroke time, fail position, position feedback unknown.</t>
+          <t>Supplier for oxygen chosen.</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>FD §3.2.4; FB.OxySystem.OxyControl</t>
+          <t>Project meeting 2026-10-21</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr"/>
       <c r="I35" s="2" t="inlineStr">
         <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
           <t>Normex</t>
         </is>
       </c>
-      <c r="J35" s="2" t="inlineStr">
-        <is>
-          <t>Sigurd</t>
-        </is>
-      </c>
-      <c r="K35" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="L35" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M35" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="N35" s="2" t="inlineStr"/>
-      <c r="O35" s="2" t="inlineStr"/>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>OX-04</t>
+          <t>OX-02</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -2887,7 +2895,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Physical</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -2897,17 +2905,17 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>O2 flow meter</t>
+          <t>Oxygen supply and safety interface (Normex)</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Unit (kg/h or Nl/min), range and signal type. PLC and FIC work in kg/h; FD FIC in l/min.</t>
+          <t>Supply type (LOX / generator / valve panel), normal and minimum supply pressure, low-supply-pressure signal, PLC-controlled master shut-off valve, non-return protection (HAZID: water back into oxygenator and O2 tank). Supply pressure is display-only in the PLC.</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>FD Tabell 14; ConfigValues</t>
+          <t>HAZID oksygen; PenControl O2InjectionPressureSensor</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr"/>
@@ -2923,7 +2931,7 @@
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr">
@@ -2942,7 +2950,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>OX-05</t>
+          <t>OX-03</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -2952,33 +2960,33 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Physical</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Missing info</t>
+          <t>Inconsistency</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Injector model and gas ratio</t>
+          <t>O2 control valve type</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>FlowMax 104.2 kg/h = Chucaotech at 15 % v/v; same model 34.7 kg/h at 5 %. Confirm model, allowed ratio, valve and flow meter range.</t>
+          <t>FD: PWM solenoid valve 'via 4-20 mA'. PLC: proportional valve 4-20 mA, 4 mA = closed, 2 s ramp. Linde photos show 'pwm_ventil'; Normex sketch (15.10.26) shows a motorised valve. Signal, stroke time, fail position, position feedback unknown.</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Oppsett innløsere CT.xlsx; ConfigValues OxySystemConfig</t>
+          <t>FD §3.2.4; FB.OxySystem.OxyControl</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr"/>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>Normex / Chucaotech</t>
+          <t>Normex</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
@@ -2988,7 +2996,7 @@
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
@@ -3007,7 +3015,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>OX-06</t>
+          <t>OX-04</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -3017,37 +3025,33 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>PLC gap</t>
+          <t>Missing info</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>High-high O2 / supersaturation shut-off</t>
+          <t>O2 flow meter</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>FD (HOLD) asks oxygenation to close on high-high O2 near the inlet. No HH or TDGP shut-off in OxyControl/InletSupervisor.</t>
+          <t>Unit (kg/h or Nl/min), range and signal type. PLC and FIC work in kg/h; FD FIC in l/min.</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>FD §3.2.4</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>Decide limits, sensors, latching</t>
-        </is>
-      </c>
+          <t>FD Tabell 14; ConfigValues</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr"/>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>Internal</t>
+          <t>Normex</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -3057,7 +3061,7 @@
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
@@ -3076,7 +3080,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>OX-07</t>
+          <t>OX-05</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -3086,47 +3090,43 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Physical</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Missing info</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>O2 setpoint and unit</t>
+          <t>Injector model and gas ratio</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>8.0 mg/L is a placeholder. FD asks '% or g/l?'. Sizing sheet uses % saturation (≥80 %, 90 % at 16 °C).</t>
+          <t>FlowMax 104.2 kg/h = Chucaotech at 15 % v/v; same model 34.7 kg/h at 5 %. Confirm model, allowed ratio, valve and flow meter range.</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>FD §3.2.4; Beregningsark dimensjonering 17mars26.xlsx</t>
-        </is>
-      </c>
-      <c r="H39" s="2" t="inlineStr">
-        <is>
-          <t>mg/L vs % saturation (with temperature/salinity)</t>
-        </is>
-      </c>
+          <t>Oppsett innløsere CT.xlsx; ConfigValues OxySystemConfig</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr"/>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>Customer / biologist</t>
+          <t>Normex / Chucaotech</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>Project</t>
+          <t>Sigurd</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr">
@@ -3145,7 +3145,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>OX-08</t>
+          <t>OX-06</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -3160,27 +3160,27 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>PLC gap</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Loss of pen O2 measurement</t>
+          <t>High-high O2 / supersaturation shut-off</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>OIC01 holds its output indefinitely. FD sentence unfinished ('skal regulatoren…').</t>
+          <t>FD (HOLD) asks oxygenation to close on high-high O2 near the inlet. No HH or TDGP shut-off in OxyControl/InletSupervisor.</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>FD §3.2.4; FB.Inlet.InletSupervisor</t>
+          <t>FD §3.2.4</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Hold / fixed fallback flow / hold for limited time then alarm</t>
+          <t>Decide limits, sensors, latching</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>Project</t>
+          <t>Sigurd</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
@@ -3214,7 +3214,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>OX-09</t>
+          <t>OX-07</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -3234,27 +3234,27 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Loss of line flow measurement</t>
+          <t>O2 setpoint and unit</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Line leaves auto and holds its last valve position open-loop.</t>
+          <t>8.0 mg/L is a placeholder. FD asks '% or g/l?'. Sizing sheet uses % saturation (≥80 %, 90 % at 16 °C).</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>FB.OxySystem.OxyControl</t>
+          <t>FD §3.2.4; Beregningsark dimensjonering 17mars26.xlsx</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Hold vs close valve</t>
+          <t>mg/L vs % saturation (with temperature/salinity)</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>Internal</t>
+          <t>Customer / biologist</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
@@ -3264,7 +3264,7 @@
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="L41" s="2" t="inlineStr">
@@ -3283,7 +3283,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>OX-10</t>
+          <t>OX-08</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -3293,43 +3293,47 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Missing info</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Pressure transmitters absolute or gauge</t>
+          <t>Loss of pen O2 measurement</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>PressureSetpoint 4.0 bar assumes absolute; ValveOpenPressure 3.0 must change together with it. Range assumed 0-10 bar. Chucaotech required inlet pressure needed.</t>
+          <t>OIC01 holds its output indefinitely. FD sentence unfinished ('skal regulatoren…').</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>OxySystemConfigDUT; ConfigValues</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr"/>
+          <t>FD §3.2.4; FB.Inlet.InletSupervisor</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Hold / fixed fallback flow / hold for limited time then alarm</t>
+        </is>
+      </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>Normex / Chucaotech</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>Sigurd</t>
+          <t>Project</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr">
@@ -3348,7 +3352,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>OX-11</t>
+          <t>OX-09</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -3358,30 +3362,34 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Missing info</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>ATV650 settings</t>
+          <t>Loss of line flow measurement</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Unit id, comm-loss behaviour (FD expects hold at preset speed), 20-50 Hz and preset 40 Hz vs NX 3153 pump curve. Fault codes in PLC came from ATV320 list (NVE41316) — re-check for ATV650.</t>
+          <t>Line leaves auto and holds its last valve position open-loop.</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>ATV600-Communication-parameters-EAV64332; FB.OxySystem.OxyPumpATV650</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr"/>
+          <t>FB.OxySystem.OxyControl</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Hold vs close valve</t>
+        </is>
+      </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
           <t>Internal</t>
@@ -3389,7 +3397,7 @@
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>Sigurd</t>
+          <t>Project</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
@@ -3413,7 +3421,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>OX-12</t>
+          <t>OX-10</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -3423,7 +3431,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Physical</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -3433,33 +3441,33 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Ethernet to oxy pump drive cabinet</t>
+          <t>Pressure transmitters absolute or gauge</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Ethernet not drawn in 15169-874.004-DriveCabinet. DIN RJ45 socket (Bjørn) vs build into cabinets (JP).</t>
+          <t>PressureSetpoint 4.0 bar assumes absolute; ValveOpenPressure 3.0 must change together with it. Range assumed 0-10 bar. Chucaotech required inlet pressure needed.</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Mail 2026-10-16 'Drive cobinet for sideløpspumpen'</t>
+          <t>OxySystemConfigDUT; ConfigValues</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr"/>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>Internal</t>
+          <t>Normex / Chucaotech</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>Project</t>
+          <t>Sigurd</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr">
@@ -3478,7 +3486,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>OX-13</t>
+          <t>OX-11</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -3488,27 +3496,27 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>PLC gap</t>
+          <t>Missing info</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>OIC01 and O2 sensor alarms</t>
+          <t>ATV650 settings</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>FD Tabell 15: OIC01 deviation from setpoint and deviation between O2 sensors — not implemented.</t>
+          <t>Unit id, comm-loss behaviour (FD expects hold at preset speed), 20-50 Hz and preset 40 Hz vs NX 3153 pump curve. Fault codes in PLC came from ATV320 list (NVE41316) — re-check for ATV650.</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>FD Tabell 15</t>
+          <t>ATV600-Communication-parameters-EAV64332; FB.OxySystem.OxyPumpATV650</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr"/>
@@ -3524,7 +3532,7 @@
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L45" s="2" t="inlineStr">
@@ -3543,7 +3551,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>OX-14</t>
+          <t>OX-12</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -3553,27 +3561,27 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Physical</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Inconsistency</t>
+          <t>Missing info</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Controller units vs FD</t>
+          <t>Ethernet to oxy pump drive cabinet</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>FD: OIC01 0-100 %, three parameter sets; FIC in l/min. PLC: OIC01 total kg/h shared over lines, one set (Kp 50, Ti 1800). Deliberate — add to FD deviation list.</t>
+          <t>Ethernet not drawn in 15169-874.004-DriveCabinet. DIN RJ45 socket (Bjørn) vs build into cabinets (JP).</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>FD Tabell 13/14; FB.Inlet.InletSupervisor</t>
+          <t>Mail 2026-10-16 'Drive cobinet for sideløpspumpen'</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
@@ -3584,7 +3592,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>Sigurd</t>
+          <t>Project</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3608,7 +3616,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>OX-15</t>
+          <t>OX-13</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -3618,27 +3626,27 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Physical</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Missing info</t>
+          <t>PLC gap</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Orbit 864 Modbus noise / hub</t>
+          <t>OIC01 and O2 sensor alarms</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Mechatronic recommends a hub on the Orbit 864 RTU line. Hub ordered for Bergen lab?</t>
+          <t>FD Tabell 15: OIC01 deviation from setpoint and deviation between O2 sensors — not implemented.</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Mail 2026-09-21/30 'Bestilling av komponent til Lab i Bergen'</t>
+          <t>FD Tabell 15</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr"/>
@@ -3649,7 +3657,7 @@
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>Bjørn</t>
+          <t>Sigurd</t>
         </is>
       </c>
       <c r="K47" s="2" t="inlineStr">
@@ -3673,7 +3681,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>OX-16</t>
+          <t>OX-14</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -3688,22 +3696,22 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Code bug</t>
+          <t>Inconsistency</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Drive IP in ConfigValues</t>
+          <t>Controller units vs FD</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>InletRIOConfig DriveIP still 10.1.2.101; CAS simulator pod is at 10.1.2.150.</t>
+          <t>FD: OIC01 0-100 %, three parameter sets; FIC in l/min. PLC: OIC01 total kg/h shared over lines, one set (Kp 50, Ti 1800). Deliberate — add to FD deviation list.</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>PFC200_Sim ConfigValues</t>
+          <t>FD Tabell 13/14; FB.Inlet.InletSupervisor</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -3738,7 +3746,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>OX-17</t>
+          <t>OX-15</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -3753,38 +3761,38 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Missing hardware</t>
+          <t>Missing info</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Low O2 supply pressure switch / master shut-off valve</t>
+          <t>Orbit 864 Modbus noise / hub</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>No PLC input for low supply pressure and no PLC-controlled master shut-off valve on P&amp;ID or in PLC (HAZID backflow risk).</t>
+          <t>Mechatronic recommends a hub on the Orbit 864 RTU line. Hub ordered for Bergen lab?</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>HAZID oksygen; P&amp;ID rev A</t>
+          <t>Mail 2026-09-21/30 'Bestilling av komponent til Lab i Bergen'</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr"/>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>Normex</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>Sigurd</t>
+          <t>Bjørn</t>
         </is>
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="L49" s="2" t="inlineStr">
@@ -3803,7 +3811,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>OX-18</t>
+          <t>OX-16</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -3823,17 +3831,17 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>ATV650 fault codes from ATV320 list</t>
+          <t>Drive IP in ConfigValues</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>OxyPumpATV650 decodes LFT with ATV320 (NVE41316) codes (e.g. 16 OHF, 17 OLF, 22 USF). Verify against ATV600 list EAV64332.</t>
+          <t>InletRIOConfig DriveIP still 10.1.2.101; CAS simulator pod is at 10.1.2.150.</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>FB.OxySystem.OxyPumpATV650</t>
+          <t>PFC200_Sim ConfigValues</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
@@ -3849,12 +3857,12 @@
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="M50" s="2" t="inlineStr">
@@ -3862,21 +3870,13 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="N50" s="2" t="inlineStr">
-        <is>
-          <t>Checked 2026-10-21 (CAS FD Oxygen): register addresses and fault codes match ATV600 EAV64332. Verify on the real drive at commissioning; program design/design basis still say ATV320.</t>
-        </is>
-      </c>
-      <c r="O50" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
+      <c r="N50" s="2" t="inlineStr"/>
+      <c r="O50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>OX-19</t>
+          <t>OX-17</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -3891,32 +3891,28 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Inconsistency</t>
+          <t>Missing hardware</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Side-stream pump head vs 4 bar setpoint</t>
+          <t>Low O2 supply pressure switch / master shut-off valve</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Flygt NX 3153 datasheet: 10.2 m head at duty point, 18.3 m at shut-off (≈1-1.8 bar) — cannot give 4.0 bar after the pump. Simulator assumes 4.5 bar rise.</t>
+          <t>No PLC input for low supply pressure and no PLC-controlled master shut-off valve on P&amp;ID or in PLC (HAZID backflow risk).</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Oxygen OI18; NX 3153 datasheet; design_basis.toml</t>
-        </is>
-      </c>
-      <c r="H51" s="2" t="inlineStr">
-        <is>
-          <t>Confirm pump, injector inlet pressure and setpoint</t>
-        </is>
-      </c>
+          <t>HAZID oksygen; P&amp;ID rev A</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr"/>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>Normex / Chucaotech</t>
+          <t>Normex</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr">
@@ -3945,7 +3941,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>OX-20</t>
+          <t>OX-18</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -3965,24 +3961,20 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Bad flow measurement causes over-dosing</t>
+          <t>ATV650 fault codes from ATV320 list</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>When a line's flow measurement is bad its flow counts as 0 in the sharing while its valve stays where it was — other lines add the same flow again.</t>
+          <t>OxyPumpATV650 decodes LFT with ATV320 (NVE41316) codes (e.g. 16 OHF, 17 OLF, 22 USF). Verify against ATV600 list EAV64332.</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Oxygen OI15; FB.Inlet.InletSupervisor</t>
-        </is>
-      </c>
-      <c r="H52" s="2" t="inlineStr">
-        <is>
-          <t>Use last good flow or close the valve</t>
-        </is>
-      </c>
+          <t>FB.OxySystem.OxyPumpATV650</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr"/>
       <c r="I52" s="2" t="inlineStr">
         <is>
           <t>Internal</t>
@@ -3995,12 +3987,12 @@
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="M52" s="2" t="inlineStr">
@@ -4008,13 +4000,21 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="N52" s="2" t="inlineStr"/>
-      <c r="O52" s="2" t="inlineStr"/>
+      <c r="N52" s="2" t="inlineStr">
+        <is>
+          <t>Checked 2026-10-21 (CAS FD Oxygen): register addresses and fault codes match ATV600 EAV64332. Verify on the real drive at commissioning; program design/design basis still say ATV320.</t>
+        </is>
+      </c>
+      <c r="O52" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>OX-21</t>
+          <t>OX-19</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -4024,38 +4024,42 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Physical</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Missing hardware</t>
+          <t>Inconsistency</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Emergency stop to oxygen system</t>
+          <t>Side-stream pump head vs 4 bar setpoint</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>No E-stop input wired to the Heimdall PLC; oxygen stop on E-stop not possible.</t>
+          <t>Flygt NX 3153 datasheet: 10.2 m head at duty point, 18.3 m at shut-off (≈1-1.8 bar) — cannot give 4.0 bar after the pump. Simulator assumes 4.5 bar rise.</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Oxygen OI22; CAS FD Inlet OI13</t>
-        </is>
-      </c>
-      <c r="H53" s="2" t="inlineStr"/>
+          <t>CAS FD Oxygen OI18; NX 3153 datasheet; design_basis.toml</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>Confirm pump, injector inlet pressure and setpoint</t>
+        </is>
+      </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>Internal</t>
+          <t>Normex / Chucaotech</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>Project</t>
+          <t>Sigurd</t>
         </is>
       </c>
       <c r="K53" s="2" t="inlineStr">
@@ -4079,7 +4083,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>OX-22</t>
+          <t>OX-20</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -4089,32 +4093,32 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Missing info</t>
+          <t>Code bug</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>ATV650 comm-loss behaviour</t>
+          <t>Bad flow measurement causes over-dosing</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Factory default on lost PLC link is freewheel stop; FD wants hold at preset speed (fallback speed / speed maintain).</t>
+          <t>When a line's flow measurement is bad its flow counts as 0 in the sharing while its valve stays where it was — other lines add the same flow again.</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Oxygen OI19</t>
+          <t>CAS FD Oxygen OI15; FB.Inlet.InletSupervisor</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>Set ETHL fallback speed</t>
+          <t>Use last good flow or close the valve</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
@@ -4129,7 +4133,7 @@
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="L54" s="2" t="inlineStr">
@@ -4148,7 +4152,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>OX-23</t>
+          <t>OX-21</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -4158,27 +4162,27 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>PLC gap</t>
+          <t>Missing hardware</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Low pressure-drop alarm over injector</t>
+          <t>Emergency stop to oxygen system</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>OxynatorOutletPressure is read but unused; no low dP alarm.</t>
+          <t>No E-stop input wired to the Heimdall PLC; oxygen stop on E-stop not possible.</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Oxygen OI10</t>
+          <t>CAS FD Oxygen OI22; CAS FD Inlet OI13</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
@@ -4189,12 +4193,12 @@
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>Sigurd</t>
+          <t>Project</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="L55" s="2" t="inlineStr">
@@ -4213,7 +4217,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>OX-24</t>
+          <t>OX-22</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -4228,25 +4232,29 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>PLC gap</t>
+          <t>Missing info</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Pump leakage / temperature contacts unused</t>
+          <t>ATV650 comm-loss behaviour</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Side-stream pump leakage/temperature contacts exist on RIO1 only and are not used in the logic.</t>
+          <t>Factory default on lost PLC link is freewheel stop; FD wants hold at preset speed (fallback speed / speed maintain).</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Oxygen OI24</t>
-        </is>
-      </c>
-      <c r="H56" s="2" t="inlineStr"/>
+          <t>CAS FD Oxygen OI19</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Set ETHL fallback speed</t>
+        </is>
+      </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
           <t>Internal</t>
@@ -4278,7 +4286,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>OX-25</t>
+          <t>OX-23</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -4288,33 +4296,33 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Physical</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Inconsistency</t>
+          <t>PLC gap</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>O2 supply pressure</t>
+          <t>Low pressure-drop alarm over injector</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Normex sketch '2.5 bar ?' vs Linde sheet 10 bar.</t>
+          <t>OxynatorOutletPressure is read but unused; no low dP alarm.</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Oxygen OI1; Normex sketch 15.10.26</t>
+          <t>CAS FD Oxygen OI10</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr"/>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>Normex</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr">
@@ -4343,7 +4351,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>OX-26</t>
+          <t>OX-24</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -4353,27 +4361,27 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Physical</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>PLC gap</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Oxygen capacity with one inlet pump out</t>
+          <t>Pump leakage / temperature contacts unused</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Two lines must carry the full oxygen demand (~560-730 t biomass) when one inlet pump is out.</t>
+          <t>Side-stream pump leakage/temperature contacts exist on RIO1 only and are not used in the logic.</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Oxygen OI26; sizing sheet</t>
+          <t>CAS FD Oxygen OI24</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
@@ -4384,7 +4392,7 @@
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>Project</t>
+          <t>Sigurd</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr">
@@ -4408,7 +4416,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>OX-27</t>
+          <t>OX-25</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -4418,33 +4426,33 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Physical</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Code bug</t>
+          <t>Inconsistency</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>PT40 variable name</t>
+          <t>O2 supply pressure</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Supply pressure transmitter has the wrong variable name in the PLC vs P&amp;ID PT40.</t>
+          <t>Normex sketch '2.5 bar ?' vs Linde sheet 10 bar.</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Oxygen OI4</t>
+          <t>CAS FD Oxygen OI1; Normex sketch 15.10.26</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr"/>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>Internal</t>
+          <t>Normex</t>
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr">
@@ -4454,7 +4462,7 @@
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L59" s="2" t="inlineStr">
@@ -4473,17 +4481,17 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>OUT-01</t>
+          <t>OX-26</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Outlet</t>
+          <t>Oxygen</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Physical</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -4493,24 +4501,20 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Outlet on power loss</t>
+          <t>Oxygen capacity with one inlet pump out</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Should the outlet close automatically on power loss (FD rev B) — accumulator, backup power for the pump, or manual?</t>
+          <t>Two lines must carry the full oxygen demand (~560-730 t biomass) when one inlet pump is out.</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>FD §3.2.3; Servi Q&amp;A; mail 'Automatisk stenging' 28.09</t>
-        </is>
-      </c>
-      <c r="H60" s="2" t="inlineStr">
-        <is>
-          <t>Accumulator / backup power / manual hand pump</t>
-        </is>
-      </c>
+          <t>CAS FD Oxygen OI26; sizing sheet</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr"/>
       <c r="I60" s="2" t="inlineStr">
         <is>
           <t>Internal</t>
@@ -4523,12 +4527,12 @@
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>Decided</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="M60" s="2" t="inlineStr">
@@ -4536,71 +4540,59 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="N60" s="2" t="inlineStr">
-        <is>
-          <t>No automatic close. Dampers hold position; operator overrides with the HPU hand pump. Accumulator deferred — space for retrofit.</t>
-        </is>
-      </c>
-      <c r="O60" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
+      <c r="N60" s="2" t="inlineStr"/>
+      <c r="O60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>OUT-02</t>
+          <t>OX-27</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Outlet</t>
+          <t>Oxygen</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Missing hardware</t>
+          <t>Code bug</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Pressure transmitters per cylinder (8 → 4)</t>
+          <t>PT40 variable name</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Servi drawing A1 (2939238) has one PT per cylinder (1PT1-1PT4, 0-250 bar, A/plus line). FD PT61-68 and PLC (PressureOpen + PressureClose, 8 AIs) expect two. End position confirmable in one direction only.</t>
+          <t>Supply pressure transmitter has the wrong variable name in the PLC vs P&amp;ID PT40.</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Servi A1; FD §3.2.3; CylinderInputDUT; mail Bjørn 2026-10-19</t>
-        </is>
-      </c>
-      <c r="H61" s="2" t="inlineStr">
-        <is>
-          <t>Buy 2nd PT (Minimess point, Servi offer) / detect end-of-stroke by pulses stopping</t>
-        </is>
-      </c>
+          <t>CAS FD Oxygen OI4</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr"/>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>Servi</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>Bjørn</t>
+          <t>Sigurd</t>
         </is>
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="L61" s="2" t="inlineStr">
@@ -4619,7 +4611,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>OUT-03</t>
+          <t>OUT-01</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -4629,38 +4621,42 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Physical</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Missing info</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Plus stroke direction</t>
+          <t>Outlet on power loss</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Does plus stroke (A, extend) open or close the damper? Decides which end has the PT and the counter direction.</t>
+          <t>Should the outlet close automatically on power loss (FD rev B) — accumulator, backup power for the pump, or manual?</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Servi A1</t>
-        </is>
-      </c>
-      <c r="H62" s="2" t="inlineStr"/>
+          <t>FD §3.2.3; Servi Q&amp;A; mail 'Automatisk stenging' 28.09</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>Accumulator / backup power / manual hand pump</t>
+        </is>
+      </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>Østerbø / Servi</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>Bjørn</t>
+          <t>Project</t>
         </is>
       </c>
       <c r="K62" s="2" t="inlineStr">
@@ -4670,7 +4666,7 @@
       </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Decided</t>
         </is>
       </c>
       <c r="M62" s="2" t="inlineStr">
@@ -4678,13 +4674,21 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="N62" s="2" t="inlineStr"/>
-      <c r="O62" s="2" t="inlineStr"/>
+      <c r="N62" s="2" t="inlineStr">
+        <is>
+          <t>No automatic close. Dampers hold position; operator overrides with the HPU hand pump. Accumulator deferred — space for retrofit.</t>
+        </is>
+      </c>
+      <c r="O62" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>OUT-04</t>
+          <t>OUT-02</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -4699,25 +4703,29 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>PLC gap</t>
+          <t>Missing hardware</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Junction box signals not mapped</t>
+          <t>Pressure transmitters per cylinder (8 → 4)</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>JB 18068: pump on backup/normal power (K1/K2), filter clogged, E-stop loop, local Start/Stop panel ST-16183, motor running feedback, power-lost relay (action 82). PLC maps only StarterFault, HydraulicOilTankFault, EStop + Start/Reset.</t>
+          <t>Servi drawing A1 (2939238) has one PT per cylinder (1PT1-1PT4, 0-250 bar, A/plus line). FD PT61-68 and PLC (PressureOpen + PressureClose, 8 AIs) expect two. End position confirmable in one direction only.</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Servi JB 18068 A2/A3; FB.RIO.CommonRIO</t>
-        </is>
-      </c>
-      <c r="H63" s="2" t="inlineStr"/>
+          <t>Servi A1; FD §3.2.3; CylinderInputDUT; mail Bjørn 2026-10-19</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>Buy 2nd PT (Minimess point, Servi offer) / detect end-of-stroke by pulses stopping</t>
+        </is>
+      </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
           <t>Servi</t>
@@ -4749,7 +4757,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>OUT-05</t>
+          <t>OUT-03</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -4759,33 +4767,33 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Physical</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>PLC gap</t>
+          <t>Missing info</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Power-lost alarm to operator</t>
+          <t>Plus stroke direction</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>With manual override decided, operator must be alarmed on power loss. Needs the Servi power-lost / backup-power relay as a PLC input.</t>
+          <t>Does plus stroke (A, extend) open or close the damper? Decides which end has the PT and the counter direction.</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Decision 2026-10-21; action item 82</t>
+          <t>Servi A1</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr"/>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>Servi</t>
+          <t>Østerbø / Servi</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -4814,7 +4822,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>OUT-06</t>
+          <t>OUT-04</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -4829,28 +4837,28 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>PLC gap</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>Hydraulic pump control authority</t>
+          <t>Junction box signals not mapped</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Pump is DOL (start/reset DO, StarterFault DI, no running feedback). Local start/stop panel offered by Servi but not ordered. Local vs PLC authority; hard-wired low-oil stop?</t>
+          <t>JB 18068: pump on backup/normal power (K1/K2), filter clogged, E-stop loop, local Start/Stop panel ST-16183, motor running feedback, power-lost relay (action 82). PLC maps only StarterFault, HydraulicOilTankFault, EStop + Start/Reset.</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Servi mail 2026-10-01; OutletControl.HydraulicPumpControl</t>
+          <t>Servi JB 18068 A2/A3; FB.RIO.CommonRIO</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr"/>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>Internal / Servi</t>
+          <t>Servi</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
@@ -4860,7 +4868,7 @@
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="L65" s="2" t="inlineStr">
@@ -4879,7 +4887,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>OUT-07</t>
+          <t>OUT-05</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -4889,33 +4897,33 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Code bug</t>
+          <t>PLC gap</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Pump not stopped on oil tank fault</t>
+          <t>Power-lost alarm to operator</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>PLC only alarms on HydraulicOilTankFault (low level / 70 °C); pump start not gated.</t>
+          <t>With manual override decided, operator must be alarmed on power loss. Needs the Servi power-lost / backup-power relay as a PLC input.</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>OutletControl.HydraulicPumpControl</t>
+          <t>Decision 2026-10-21; action item 82</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>Internal</t>
+          <t>Servi</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
@@ -4925,7 +4933,7 @@
       </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="L66" s="2" t="inlineStr">
@@ -4944,7 +4952,7 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>OUT-08</t>
+          <t>OUT-06</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -4954,33 +4962,33 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>PLC gap</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Outlet E-stop and other alarms</t>
+          <t>Hydraulic pump control authority</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>No E-stop alarm (ES61 in alarm list); no filter, pump overload or power-loss alarms.</t>
+          <t>Pump is DOL (start/reset DO, StarterFault DI, no running feedback). Local start/stop panel offered by Servi but not ordered. Local vs PLC authority; hard-wired low-oil stop?</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>FD-02 alarm list; OutletControl.AlarmHandling</t>
+          <t>Servi mail 2026-10-01; OutletControl.HydraulicPumpControl</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr"/>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>Internal</t>
+          <t>Internal / Servi</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
@@ -5009,7 +5017,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>OUT-09</t>
+          <t>OUT-07</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -5019,37 +5027,33 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Physical</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Inconsistency</t>
+          <t>Code bug</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Flow meter signal type</t>
+          <t>Pump not stopped on oil tank fault</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>JB overview sheet labels FT1-4 '24VDC 4-20MA'; sheet A2 says pulse. PLC assumes pulse (750-638).</t>
+          <t>PLC only alarms on HydraulicOilTankFault (low level / 70 °C); pump start not gated.</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Servi JB 18068</t>
-        </is>
-      </c>
-      <c r="H68" s="2" t="inlineStr">
-        <is>
-          <t>Servi to correct overview sheet</t>
-        </is>
-      </c>
+          <t>OutletControl.HydraulicPumpControl</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr"/>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>Servi</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
@@ -5078,7 +5082,7 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>OUT-10</t>
+          <t>OUT-08</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -5093,22 +5097,22 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Code bug</t>
+          <t>PLC gap</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Mode openings look reversed</t>
+          <t>Outlet E-stop and other alarms</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>OutletConfig.ModePosition default [20,30,40,50] % gives O-35 (34 000 m3/h) the smallest opening and S-75 the largest. FD column 'Spjeld-åpning %' empty.</t>
+          <t>No E-stop alarm (ES61 in alarm list); no filter, pump overload or power-loss alarms.</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>ConfigValues OutletConfig; FD Tabell 10</t>
+          <t>FD-02 alarm list; OutletControl.AlarmHandling</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr"/>
@@ -5143,7 +5147,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>OUT-11</t>
+          <t>OUT-09</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -5153,32 +5157,32 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Physical</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Missing info</t>
+          <t>Inconsistency</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Stroke time and travel limits</t>
+          <t>Flow meter signal type</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>MaxTravelTimeOpen/Close 30 s = assumed stroke time (no margin). Estimate: one cylinder 5-7 s, four sharing the pump 20-26 s. FD 'ca nn s'.</t>
+          <t>JB overview sheet labels FT1-4 '24VDC 4-20MA'; sheet A2 says pulse. PLC assumes pulse (750-638).</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>OutletConfig; design_basis.toml; Servi A1</t>
+          <t>Servi JB 18068</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>Fill in at FAT</t>
+          <t>Servi to correct overview sheet</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
@@ -5212,7 +5216,7 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>OUT-12</t>
+          <t>OUT-10</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -5222,33 +5226,33 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Physical</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Missing info</t>
+          <t>Code bug</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>PSL valves driven on/off</t>
+          <t>Mode openings look reversed</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>HAWE PSL are proportional; PLC drives them on/off via relays (750-1515). Confirm with Servi (min ~250 mA note, optional speed card) and relay rating.</t>
+          <t>OutletConfig.ModePosition default [20,30,40,50] % gives O-35 (34 000 m3/h) the smallest opening and S-75 the largest. FD column 'Spjeld-åpning %' empty.</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>Servi A1; CommonRIO output mapping</t>
+          <t>ConfigValues OutletConfig; FD Tabell 10</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr"/>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>Servi</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
@@ -5277,7 +5281,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>OUT-13</t>
+          <t>OUT-11</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -5297,23 +5301,27 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Outputs on remote I/O comm loss</t>
+          <t>Stroke time and travel limits</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>FD table empty; 750-1515 watchdog behaviour not set.</t>
+          <t>MaxTravelTimeOpen/Close 30 s = assumed stroke time (no margin). Estimate: one cylinder 5-7 s, four sharing the pump 20-26 s. FD 'ca nn s'.</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>FD §3.2.3</t>
-        </is>
-      </c>
-      <c r="H72" s="2" t="inlineStr"/>
+          <t>OutletConfig; design_basis.toml; Servi A1</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>Fill in at FAT</t>
+        </is>
+      </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>Internal</t>
+          <t>Servi</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -5342,7 +5350,7 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>OUT-14</t>
+          <t>OUT-12</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -5362,33 +5370,33 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>Shut-off valve XV65</t>
+          <t>PSL valves driven on/off</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>In FD and PLS action list 6.3 ('Stopp-ventil') but not on Servi A1 or in the PLC. Deferred with the accumulator?</t>
+          <t>HAWE PSL are proportional; PLC drives them on/off via relays (750-1515). Confirm with Servi (min ~250 mA note, optional speed card) and relay rating.</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>FD §3.2.3; PLS aksjonsliste 6.3</t>
+          <t>Servi A1; CommonRIO output mapping</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr"/>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>Internal</t>
+          <t>Servi</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>Project</t>
+          <t>Bjørn</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L73" s="2" t="inlineStr">
@@ -5407,7 +5415,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>OUT-15</t>
+          <t>OUT-13</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -5417,33 +5425,33 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Physical</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Inconsistency</t>
+          <t>Missing info</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Motor and pressure data</t>
+          <t>Outputs on remote I/O comm loss</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>Motor 1.5 kW 400 V (datasheet, A1) vs &lt;1 kW (Q&amp;A); cable W1M1 'Hydraulic motor 24Vdc'. Relief 150/130 bar (A1) vs 160 bar in simulator, 110 bar (T1). Tank 12 l (A1 part list) vs 10 l; cylinder HRC-N-D vs HCR-C-D; motor starter location (action 91).</t>
+          <t>FD table empty; 750-1515 watchdog behaviour not set.</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Servi A1, Q&amp;A, JB 18068; design_basis.toml</t>
+          <t>FD §3.2.3</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr"/>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>Servi</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
@@ -5453,7 +5461,7 @@
       </c>
       <c r="K74" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L74" s="2" t="inlineStr">
@@ -5472,7 +5480,7 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>OUT-16</t>
+          <t>OUT-14</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -5492,24 +5500,20 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Counter frequency</t>
+          <t>Shut-off valve XV65</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>~300 Hz at 3.5 l/min and ~5200 pulses/l; minus stroke of one cylinder pushes 4.7-5.4 l/min through its A-line meter (~410-470 Hz), near the QG100 top and the 750-638 500 Hz limit. Reverse-flow accuracy unknown.</t>
+          <t>In FD and PLS action list 6.3 ('Stopp-ventil') but not on Servi A1 or in the PLC. Deferred with the accumulator?</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>HySense QG datasheet; 750-638 manual; CAS FD Outlet OI11</t>
-        </is>
-      </c>
-      <c r="H75" s="2" t="inlineStr">
-        <is>
-          <t>Test at FAT</t>
-        </is>
-      </c>
+          <t>FD §3.2.3; PLS aksjonsliste 6.3</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr"/>
       <c r="I75" s="2" t="inlineStr">
         <is>
           <t>Internal</t>
@@ -5517,12 +5521,12 @@
       </c>
       <c r="J75" s="2" t="inlineStr">
         <is>
-          <t>Bjørn</t>
+          <t>Project</t>
         </is>
       </c>
       <c r="K75" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="L75" s="2" t="inlineStr">
@@ -5541,7 +5545,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>OUT-17</t>
+          <t>OUT-15</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -5556,38 +5560,38 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Inconsistency</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Integrated FAT at Østerbø</t>
+          <t>Motor and pressure data</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>Integrated test of our control cabinet with Servi's hydraulic cabinet, end of October: scope, hose lengths, fail-safe and hand pump test.</t>
+          <t>Motor 1.5 kW 400 V (datasheet, A1) vs &lt;1 kW (Q&amp;A); cable W1M1 'Hydraulic motor 24Vdc'. Relief 150/130 bar (A1) vs 160 bar in simulator, 110 bar (T1). Tank 12 l (A1 part list) vs 10 l; cylinder HRC-N-D vs HCR-C-D; motor starter location (action 91).</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Mail Fredrik 2026-10-07</t>
+          <t>Servi A1, Q&amp;A, JB 18068; design_basis.toml</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>Østerbø / Servi</t>
+          <t>Servi</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>Project</t>
+          <t>Bjørn</t>
         </is>
       </c>
       <c r="K76" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="L76" s="2" t="inlineStr">
@@ -5606,7 +5610,7 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>OUT-18</t>
+          <t>OUT-16</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -5616,32 +5620,32 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Physical</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>Code bug</t>
+          <t>Missing info</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Close never confirmed without 2nd pressure transmitter</t>
+          <t>Counter frequency</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>With MaxPressureClose &gt; 0 on an unwired channel a 0 % setpoint never reaches Closed → travel timeout and fault; with 0 the end-position check is disabled. CalibrateOpen also needs Opened by pressure.</t>
+          <t>~300 Hz at 3.5 l/min and ~5200 pulses/l; minus stroke of one cylinder pushes 4.7-5.4 l/min through its A-line meter (~410-470 Hz), near the QG100 top and the 750-638 500 Hz limit. Reverse-flow accuracy unknown.</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>FB.Outlet.OutletControl; CylinderInputDUT</t>
+          <t>HySense QG datasheet; 750-638 manual; CAS FD Outlet OI11</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>Depends on OUT PT decision</t>
+          <t>Test at FAT</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
@@ -5656,7 +5660,7 @@
       </c>
       <c r="K77" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L77" s="2" t="inlineStr">
@@ -5675,7 +5679,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>OUT-19</t>
+          <t>OUT-17</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -5690,38 +5694,38 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Missing hardware</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Hydraulic pump running feedback</t>
+          <t>Integrated FAT at Østerbø</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Pump is DOL; PLC has no running feedback (Status.Running = start command). Contactor auxiliary contact available in JB 18068?</t>
+          <t>Integrated test of our control cabinet with Servi's hydraulic cabinet, end of October: scope, hose lengths, fail-safe and hand pump test.</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>OutletControl.HydraulicPumpControl; Servi JB 18068</t>
+          <t>Mail Fredrik 2026-10-07</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr"/>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>Servi</t>
+          <t>Østerbø / Servi</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t>Bjørn</t>
+          <t>Project</t>
         </is>
       </c>
       <c r="K78" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="L78" s="2" t="inlineStr">
@@ -5740,7 +5744,7 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>OUT-20</t>
+          <t>OUT-18</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -5760,20 +5764,24 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>End-position pressure limit cannot trip</t>
+          <t>Close never confirmed without 2nd pressure transmitter</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>Servi A1 port pressure limiters are 100 bar; PLC end-position limit is also 100 bar with strict '&gt;'. Set ~70-80 bar after FAT; align simulator (160 bar).</t>
+          <t>With MaxPressureClose &gt; 0 on an unwired channel a 0 % setpoint never reaches Closed → travel timeout and fault; with 0 the end-position check is disabled. CalibrateOpen also needs Opened by pressure.</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Outlet OI3; Servi A1; OutletConfig</t>
-        </is>
-      </c>
-      <c r="H79" s="2" t="inlineStr"/>
+          <t>FB.Outlet.OutletControl; CylinderInputDUT</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>Depends on OUT PT decision</t>
+        </is>
+      </c>
       <c r="I79" s="2" t="inlineStr">
         <is>
           <t>Internal</t>
@@ -5805,7 +5813,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>OUT-21</t>
+          <t>OUT-19</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -5815,33 +5823,33 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Physical</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Code bug</t>
+          <t>Missing hardware</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Pressure scaling 0-250 bar</t>
+          <t>Hydraulic pump running feedback</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Production pressure scaling must be 0-250 bar; DUT default is 0-10.</t>
+          <t>Pump is DOL; PLC has no running feedback (Status.Running = start command). Contactor auxiliary contact available in JB 18068?</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Outlet OI4</t>
+          <t>OutletControl.HydraulicPumpControl; Servi JB 18068</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr"/>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>Internal</t>
+          <t>Servi</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
@@ -5870,7 +5878,7 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>OUT-22</t>
+          <t>OUT-20</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -5890,17 +5898,17 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>Default span treated as calibrated</t>
+          <t>End-position pressure limit cannot trip</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>Default span 0-2000 counts counts as calibrated; calibration must be a commissioning step. FaultReset unused.</t>
+          <t>Servi A1 port pressure limiters are 100 bar; PLC end-position limit is also 100 bar with strict '&gt;'. Set ~70-80 bar after FAT; align simulator (160 bar).</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Outlet OI15</t>
+          <t>CAS FD Outlet OI3; Servi A1; OutletConfig</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr"/>
@@ -5916,7 +5924,7 @@
       </c>
       <c r="K81" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="L81" s="2" t="inlineStr">
@@ -5935,7 +5943,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>OUT-23</t>
+          <t>OUT-21</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -5945,33 +5953,33 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Inconsistency</t>
+          <t>Code bug</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>PLC Reset output has no JB counterpart</t>
+          <t>Pressure scaling 0-250 bar</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>PLC drives a pump Reset output; JB 18068 has no matching input. DI -R1-017 / DO -R1-020 wiring needed.</t>
+          <t>Production pressure scaling must be 0-250 bar; DUT default is 0-10.</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Outlet OI7; JB 18068</t>
+          <t>CAS FD Outlet OI4</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr"/>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>Servi</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr">
@@ -6000,7 +6008,7 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>OUT-24</t>
+          <t>OUT-22</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
@@ -6010,27 +6018,27 @@
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>Physical</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>Missing info</t>
+          <t>Code bug</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Manual override procedure (O&amp;M)</t>
+          <t>Default span treated as calibrated</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>Hand pump and PSL manual levers, plus weekly end-position exercise, to be written into the O&amp;M manual.</t>
+          <t>Default span 0-2000 counts counts as calibrated; calibration must be a commissioning step. FaultReset unused.</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Outlet OI17; decision 2026-10-21</t>
+          <t>CAS FD Outlet OI15</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr"/>
@@ -6041,7 +6049,7 @@
       </c>
       <c r="J83" s="2" t="inlineStr">
         <is>
-          <t>Project</t>
+          <t>Bjørn</t>
         </is>
       </c>
       <c r="K83" s="2" t="inlineStr">
@@ -6065,7 +6073,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>OUT-25</t>
+          <t>OUT-23</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -6080,28 +6088,28 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Missing info</t>
+          <t>Inconsistency</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Position drift limit</t>
+          <t>PLC Reset output has no JB counterpart</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>Drift limit of 2 pulses (HOLD in FD) to be verified at FAT.</t>
+          <t>PLC drives a pump Reset output; JB 18068 has no matching input. DI -R1-017 / DO -R1-020 wiring needed.</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>CAS FD Outlet OI18</t>
+          <t>CAS FD Outlet OI7; JB 18068</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr"/>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>Internal</t>
+          <t>Servi</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
@@ -6111,7 +6119,7 @@
       </c>
       <c r="K84" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L84" s="2" t="inlineStr">
@@ -6127,8 +6135,138 @@
       <c r="N84" s="2" t="inlineStr"/>
       <c r="O84" s="2" t="inlineStr"/>
     </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>OUT-24</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>Outlet</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>Physical</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>Missing info</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>Manual override procedure (O&amp;M)</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>Hand pump and PSL manual levers, plus weekly end-position exercise, to be written into the O&amp;M manual.</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>CAS FD Outlet OI17; decision 2026-10-21</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr"/>
+      <c r="I85" s="2" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="J85" s="2" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="K85" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L85" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M85" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="N85" s="2" t="inlineStr"/>
+      <c r="O85" s="2" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>OUT-25</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Outlet</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>Missing info</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>Position drift limit</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>Drift limit of 2 pulses (HOLD in FD) to be verified at FAT.</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>CAS FD Outlet OI18</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr"/>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>Bjørn</t>
+        </is>
+      </c>
+      <c r="K86" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L86" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M86" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="N86" s="2" t="inlineStr"/>
+      <c r="O86" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O84"/>
+  <autoFilter ref="A1:O86"/>
   <conditionalFormatting sqref="K2:K500">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"High"</formula>

</xml_diff>

<commit_message>
CAS outstanding items: status Fixed (green row), IN-29 fixed in CODESYS
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAS/Outstanding items.xlsx
+++ b/CAS/Outstanding items.xlsx
@@ -113,6 +113,13 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="00C6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="00F8CBAD"/>
         </patternFill>
       </fill>
@@ -128,13 +135,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00E2EFDA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00C6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2725,7 +2725,7 @@
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr">
@@ -2735,10 +2735,14 @@
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>Implemented 2026-10-21 in CODESYS (not yet staged/compiled/tested): Command.Reset accepted in HOLD/LOCKDOWN, latched as ResetRequest, cleared when the state change is seen; no change within 2 x ResetExpectedTime (5 s) -&gt; Reset withdrawn and warning FailedToReset (auto-acknowledged).</t>
-        </is>
-      </c>
-      <c r="O33" s="2" t="inlineStr"/>
+          <t>Fixed in CODESYS 2026-10-21 (FB.Inlet.InletControl): Command.Reset accepted in HOLD/LOCKDOWN, latched as ResetRequest and cleared when the state change is seen; no change within 2 x InletConfig.ResetExpectedTime (default 5 s) -&gt; Reset withdrawn and warning Alarm.FailedToReset (AutoAcknowledge). Command.Reset is exported read/write over OPC UA (checked on 10.1.2.41). Pre-compile clean; full compile and sim test pending.</t>
+        </is>
+      </c>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -6267,22 +6271,27 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:O86"/>
+  <conditionalFormatting sqref="A2:O500">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
+      <formula>$L2="Fixed"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="K2:K500">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
       <formula>"High"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
       <formula>"Medium"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"Low"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L2:L500">
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="0">
       <formula>"Decided"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="4">
       <formula>"Closed"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6300,7 +6309,7 @@
       <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
     <dataValidation sqref="L2:L500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Open,In progress,Decided,Closed"</formula1>
+      <formula1>"Open,In progress,Decided,Fixed,Closed"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6313,7 +6322,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6323,6 +6332,7 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6365,6 +6375,11 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
           <t>All items</t>
         </is>
       </c>
@@ -6396,6 +6411,10 @@
         <v/>
       </c>
       <c r="G4" s="5">
+        <f>COUNTIFS('Outstanding items'!$B:$B,$A4,'Outstanding items'!$L:$L,"Fixed")</f>
+        <v/>
+      </c>
+      <c r="H4" s="5">
         <f>COUNTIFS('Outstanding items'!$B:$B,$A4)</f>
         <v/>
       </c>
@@ -6427,6 +6446,10 @@
         <v/>
       </c>
       <c r="G5" s="5">
+        <f>COUNTIFS('Outstanding items'!$B:$B,$A5,'Outstanding items'!$L:$L,"Fixed")</f>
+        <v/>
+      </c>
+      <c r="H5" s="5">
         <f>COUNTIFS('Outstanding items'!$B:$B,$A5)</f>
         <v/>
       </c>
@@ -6458,6 +6481,10 @@
         <v/>
       </c>
       <c r="G6" s="5">
+        <f>COUNTIFS('Outstanding items'!$B:$B,$A6,'Outstanding items'!$L:$L,"Fixed")</f>
+        <v/>
+      </c>
+      <c r="H6" s="5">
         <f>COUNTIFS('Outstanding items'!$B:$B,$A6)</f>
         <v/>
       </c>
@@ -6489,6 +6516,10 @@
         <v/>
       </c>
       <c r="G7" s="5">
+        <f>COUNTIFS('Outstanding items'!$B:$B,$A7,'Outstanding items'!$L:$L,"Fixed")</f>
+        <v/>
+      </c>
+      <c r="H7" s="5">
         <f>COUNTIFS('Outstanding items'!$B:$B,$A7)</f>
         <v/>
       </c>
@@ -6521,6 +6552,10 @@
       </c>
       <c r="G8" s="5">
         <f>SUM(G4:G7)</f>
+        <v/>
+      </c>
+      <c r="H8" s="5">
+        <f>SUM(H4:H7)</f>
         <v/>
       </c>
     </row>
@@ -6618,7 +6653,7 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Open → In progress → Decided (fill Decision/answer and Decided date) → Closed (implemented in docs/PLC).</t>
+          <t>Open → In progress → Decided (fill Decision/answer and Decided date) → Fixed (changed in CODESYS / code: whole row green, Decision/answer says what was done and how it was tested) → Closed (verified, docs updated).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CAS outstanding items: conditional fills visible in Excel (set bgColor)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAS/Outstanding items.xlsx
+++ b/CAS/Outstanding items.xlsx
@@ -114,6 +114,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00C6EFCE"/>
+          <bgColor rgb="00C6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -121,6 +122,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00F8CBAD"/>
+          <bgColor rgb="00F8CBAD"/>
         </patternFill>
       </fill>
     </dxf>
@@ -128,6 +130,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00FFE699"/>
+          <bgColor rgb="00FFE699"/>
         </patternFill>
       </fill>
     </dxf>
@@ -135,6 +138,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00E2EFDA"/>
+          <bgColor rgb="00E2EFDA"/>
         </patternFill>
       </fill>
     </dxf>
@@ -142,6 +146,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00D9D9D9"/>
+          <bgColor rgb="00D9D9D9"/>
         </patternFill>
       </fill>
     </dxf>

</xml_diff>

<commit_message>
CAS FD Inlet rev B, FD Oxygen rev A1, outstanding items
Inlet rev B: LIC01 total output shared by the pumps in REMOTE (IN-05, IN-07),
InletRIO link loss drops the pair (IN-19), level deviation alarms (IN-09),
automatic pump count and rotation (IN-15). Oxygen rev A1: RIO link loss freeze
(OX-28); a line restarts by itself when its inlet pump is back in REMOTE.
Register: IN-09 and IN-15 in progress.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAS/Outstanding items.xlsx
+++ b/CAS/Outstanding items.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Outstanding items'!$A$1:$O$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Outstanding items'!$A$1:$O$87</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O86"/>
+  <dimension ref="A1:O87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1134,7 +1134,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
@@ -1142,8 +1142,12 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr"/>
-      <c r="O9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>Baseline sim 2026-10-22: pump 3 out -&gt; level 6.0 -&gt; 3.0 cm, 4 min back; pump 3 restart -&gt; 9.1 cm, mostly during its START (own preset speed while the others still ran fast). Implemented in CODESYS 2026-10-22 (not yet downloaded/tested): LIC01 output = TOTAL speed of the pumps in level control; pumps in REMOTE share (total - actual speed of the pumps starting/stopping) / N, limited 40-130 rpm, in PenInletSupervisor.AutoSpeedSetpoint. A trip or a start is compensated in the same cycle; Kp 450 -&gt; 1350 (total). Retained Kp must be set to 1350 after download. HMI: heimdall-cas-hmi PR #6. Sim test pending (PLC busy).</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1272,7 +1276,7 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
@@ -1280,8 +1284,12 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr"/>
-      <c r="O11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>With the shared total output (IN-05) the loop gain no longer depends on the number of pumps: one parameter set (Kp 1350 total rpm/m, Ti 60 s) replaces FD Tabell 8's three. Update FD to rev C after the sim test.</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1402,7 +1410,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
@@ -1410,7 +1418,11 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>Control deviation implemented in CODESYS 2026-10-22 (not yet downloaded/tested): Pen.Alarm.LevelDeviationHigh / LevelDeviationLow when LIC01 is in auto and the over-height is more than PenConfig.LevelDeviationLimit (0.02 m) above / below the setpoint for LevelDeviationDelay (5 min); not during start-up, manual, SafeOutput or HOLD freeze. Fault per level sensor already covered by the transmitters' Quality alarms. Still open: absolute low / high level alarms (alarm list rows 31-32). HMI: heimdall-cas-hmi PR #8.</t>
+        </is>
+      </c>
       <c r="O13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
@@ -1796,7 +1808,7 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
@@ -1804,7 +1816,11 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="N19" s="2" t="inlineStr"/>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>Automatic pump start/stop and rotation implemented in CODESYS 2026-10-22 (not yet downloaded/tested), InletSupervisor.PumpCount: candidates = InletConfig[i].InletPump.Enable AND auto AND not UNAVAILABLE/LOCKDOWN. Pen Start starts all candidates; with LIC01 in auto and no pump changing: stop the pump with most running days when the others would run &lt;= PumpTargetSpeed (85 rpm) for PumpRemoveDelay (15 min); start the standby with fewest running days when the share &gt;= PumpAddSpeed (115 rpm) for PumpAddDelay (2 min); rotation after PumpCycleTime (24 h) in REMOTE, make-before-break. Settings retained in PenConfig (Reset Origin on next download). Still open from the HOLD list: manual level setpoint, auto outlet close on pump stop, E-stop alarm.</t>
+        </is>
+      </c>
       <c r="O19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
@@ -1995,7 +2011,7 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
@@ -2003,8 +2019,16 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="N22" s="2" t="inlineStr"/>
-      <c r="O22" s="2" t="inlineStr"/>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>Not a bug. Util.PID adapts the integral while the output is limited (anti-windup). Sim test 2026-10-22: one of three pumps out, LIC01 output rose 74 -&gt; 107 rpm and never reached 130 (LimitsActive FALSE). The dip/overshoot is the missing compensation of the pump count, see IN-05.</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2064,7 +2088,7 @@
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
@@ -2072,8 +2096,16 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="N23" s="2" t="inlineStr"/>
-      <c r="O23" s="2" t="inlineStr"/>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>Fixed in CODESYS 2026-10-22: InletControl / InletSensors get RIOCommOK = GVLIO.InletRIO[i].Status.CommOK; without it both transmitters of that inlet count as BadQuality, so only that pair drops out of LIC01's PV (all three lost -&gt; LevelMeasurementLost, SafeOutput). Sim test 2026-10-22 (PFC200 vs CAS plant 10.1.2.150): pair 1 out for 60 s with 3 pumps in REMOTE, PV continued on pairs 2-3, LIC01 output 74.1-74.3 rpm, pair back without a jump. Realistic link-down test (5 s socket timeout) with the simulator fault of heimdall-cas-simulation PR #17.</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -3871,7 +3903,7 @@
       </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M50" s="2" t="inlineStr">
@@ -3879,8 +3911,16 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="N50" s="2" t="inlineStr"/>
-      <c r="O50" s="2" t="inlineStr"/>
+      <c r="N50" s="2" t="inlineStr">
+        <is>
+          <t>ConfigValues 2026-10-22: CommonRIO, InletRIO 1-3 and the drives point at the CAS plant 10.1.2.150 (simulator-manager, southshore-bergen); also written into the running PLC's retain.</t>
+        </is>
+      </c>
+      <c r="O50" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -6274,8 +6314,77 @@
       <c r="N86" s="2" t="inlineStr"/>
       <c r="O86" s="2" t="inlineStr"/>
     </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>OX-28</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>Oxygen</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>Code bug</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>RIO link loss freezes oxygen line sensors</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>Same as IN-19 on the oxygen side: PT41-43 / PT44-46 (InletRIO) and FT41-43, PT40 (CommonRIO) keep their last value and good quality when the RIO link is lost, so PIC4n, the valve permit I4 and FIC4n run on frozen values.</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>IN-19; FB.RIO.InletRIO / CommonRIO InputMapping; FB.OxySystem.OxyControl</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>Mark the line's sensors BadQuality on RIO comm loss (as IN-19): PIC on preset speed, valve closed, line out of auto</t>
+        </is>
+      </c>
+      <c r="I87" s="2" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K87" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L87" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M87" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="N87" s="2" t="n"/>
+      <c r="O87" s="2" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O86"/>
+  <autoFilter ref="A1:O87"/>
   <conditionalFormatting sqref="A2:O500">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>$L2="Fixed"</formula>
@@ -6588,7 +6697,6 @@
           <t>How to use</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" s="7" t="inlineStr">

</xml_diff>

<commit_message>
CAS: speed deviation alarm (IN-10), LowPower/HighPower notification only (IN-11)
FD Inlet rev B: alarm and fault tables, parameters, OI9/OI10; register updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAS/Outstanding items.xlsx
+++ b/CAS/Outstanding items.xlsx
@@ -1479,7 +1479,7 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
@@ -1487,7 +1487,11 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>Implemented in CODESYS 2026-10-22 (not yet downloaded/tested): Inlet[i].InletPump.Alarm.SpeedDeviation (operator ack) when the pump is in REMOTE and |VelocitySetpoint - MotorVelocity| &gt; InletConfig[i].SpeedDeviationLimit (10 rpm) for SpeedDeviationDelay (30 s); limit 0 = off. Retained in InletConfigDUT (Reset Origin with IN-15). Duplicate alarm-list row removed in FD-01 rev C.</t>
+        </is>
+      </c>
       <c r="O14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
@@ -1548,7 +1552,7 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
@@ -1556,7 +1560,11 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>Implemented in CODESYS 2026-10-22 (not yet downloaded): LowPower / HighPower removed from PumpCommonError; their own alarms are notifications (AutoAcknowledge), as FD Tabell 7.</t>
+        </is>
+      </c>
       <c r="O15" s="2" t="inlineStr"/>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
CAS: no upstream O2 shut-off valves (budget decision), OX-17 / FD Oxygen OI5
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAS/Outstanding items.xlsx
+++ b/CAS/Outstanding items.xlsx
@@ -3984,7 +3984,7 @@
       </c>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Decided</t>
         </is>
       </c>
       <c r="M51" s="2" t="inlineStr">
@@ -3992,8 +3992,16 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="N51" s="2" t="inlineStr"/>
-      <c r="O51" s="2" t="inlineStr"/>
+      <c r="N51" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22 (Sigurd): no on/off solenoid or master shut-off valves upstream of the O2 control valves (budget decision). The control valve is the only shut-off: the PLC holds it at 4 mA (closed) without the valve permit (oxy pump running, PT after the pump good and above ValveOpenPressure, default 3.0 bar), before RunDelay, without the inlet permit and on emergency stop. A low-supply-pressure input is still not available. Consequences: O2 HH shut-off (OX-06) can only close the control valves; backflow protection (HAZID) relies on the non-return valves.</t>
+        </is>
+      </c>
+      <c r="O51" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">

</xml_diff>

<commit_message>
CAS: live test 2026-10-22 in register and FDs; O2 valve output bug OX-29; IN-31 rotation swing
Register: IN-05/07/15 test results (start, pump count, rotation), IN-09/10/11
not yet tested, new OX-29 (valve AO mapping, fixed) and IN-31 (level swing
during rotation). FD Inlet rev B: live test results, OI15. FD Oxygen rev A1:
valve output mapping corrected, no upstream shut-off valves.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAS/Outstanding items.xlsx
+++ b/CAS/Outstanding items.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Outstanding items'!$A$1:$O$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Outstanding items'!$A$1:$O$89</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O87"/>
+  <dimension ref="A1:O89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1144,7 +1144,7 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>Baseline sim 2026-10-22: pump 3 out -&gt; level 6.0 -&gt; 3.0 cm, 4 min back; pump 3 restart -&gt; 9.1 cm, mostly during its START (own preset speed while the others still ran fast). Implemented in CODESYS 2026-10-22 (not yet downloaded/tested): LIC01 output = TOTAL speed of the pumps in level control; pumps in REMOTE share (total - actual speed of the pumps starting/stopping) / N, limited 40-130 rpm, in PenInletSupervisor.AutoSpeedSetpoint. A trip or a start is compensated in the same cycle; Kp 450 -&gt; 1350 (total). Retained Kp must be set to 1350 after download. HMI: heimdall-cas-hmi PR #6. Sim test pending (PLC busy).</t>
+          <t>Baseline sim 2026-10-22: pump 3 out -&gt; level 6.0 -&gt; 3.0 cm, 4 min back; pump 3 restart -&gt; 9.1 cm, mostly during its START (own preset speed while the others still ran fast). Implemented in CODESYS 2026-10-22 (not yet downloaded/tested): LIC01 output = TOTAL speed of the pumps in level control; pumps in REMOTE share (total - actual speed of the pumps starting/stopping) / N, limited 40-130 rpm, in PenInletSupervisor.AutoSpeedSetpoint. A trip or a start is compensated in the same cycle; Kp 450 -&gt; 1350 (total). Retained Kp must be set to 1350 after download. HMI: heimdall-cas-hmi PR #6. Sim test pending (PLC busy). | Live test 2026-10-22 (PFC200 10.1.2.41, main 1a427c0, CAS plant 10.1.2.150, after Reset Origin): Pen Start from drained (-3.4 cm): pumps tracked to 260 rpm total, REMOTE at 85.5 rpm share (bumpless), level 6.6 cm peak (0.6 cm overshoot), settled 6.1 cm in ~2.5 min with 3 x 74 rpm. Pump stopped by the pump count: the other two took its share in the same cycle, level dip 6.0 -&gt; 5.2 cm, back to 6.3 cm. Pump trip test still to do.</t>
         </is>
       </c>
       <c r="O9" s="2" t="n"/>
@@ -1286,7 +1286,7 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>With the shared total output (IN-05) the loop gain no longer depends on the number of pumps: one parameter set (Kp 1350 total rpm/m, Ti 60 s) replaces FD Tabell 8's three. Update FD to rev C after the sim test.</t>
+          <t>With the shared total output (IN-05) the loop gain no longer depends on the number of pumps: one parameter set (Kp 1350 total rpm/m, Ti 60 s) replaces FD Tabell 8's three. Update FD to rev C after the sim test. | Live test 2026-10-22 (PFC200 10.1.2.41, main 1a427c0, CAS plant 10.1.2.150, after Reset Origin): one parameter set Kp 1350 / Ti 60 s works for 3 and 2 pumps (start-up and pump stop above).</t>
         </is>
       </c>
       <c r="O11" s="2" t="n"/>
@@ -1420,7 +1420,7 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>Control deviation implemented in CODESYS 2026-10-22 (not yet downloaded/tested): Pen.Alarm.LevelDeviationHigh / LevelDeviationLow when LIC01 is in auto and the over-height is more than PenConfig.LevelDeviationLimit (0.02 m) above / below the setpoint for LevelDeviationDelay (5 min); not during start-up, manual, SafeOutput or HOLD freeze. Fault per level sensor already covered by the transmitters' Quality alarms. Still open: absolute low / high level alarms (alarm list rows 31-32). HMI: heimdall-cas-hmi PR #8.</t>
+          <t>Control deviation implemented in CODESYS 2026-10-22 (not yet downloaded/tested): Pen.Alarm.LevelDeviationHigh / LevelDeviationLow when LIC01 is in auto and the over-height is more than PenConfig.LevelDeviationLimit (0.02 m) above / below the setpoint for LevelDeviationDelay (5 min); not during start-up, manual, SafeOutput or HOLD freeze. Fault per level sensor already covered by the transmitters' Quality alarms. Still open: absolute low / high level alarms (alarm list rows 31-32). HMI: heimdall-cas-hmi PR #8. | Live test 2026-10-22 (PFC200 10.1.2.41, main 1a427c0, CAS plant 10.1.2.150, after Reset Origin): not tested yet.</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr"/>
@@ -1489,7 +1489,7 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>Implemented in CODESYS 2026-10-22 (not yet downloaded/tested): Inlet[i].InletPump.Alarm.SpeedDeviation (operator ack) when the pump is in REMOTE and |VelocitySetpoint - MotorVelocity| &gt; InletConfig[i].SpeedDeviationLimit (10 rpm) for SpeedDeviationDelay (30 s); limit 0 = off. Retained in InletConfigDUT (Reset Origin with IN-15). Duplicate alarm-list row removed in FD-01 rev C.</t>
+          <t>Implemented in CODESYS 2026-10-22 (not yet downloaded/tested): Inlet[i].InletPump.Alarm.SpeedDeviation (operator ack) when the pump is in REMOTE and |VelocitySetpoint - MotorVelocity| &gt; InletConfig[i].SpeedDeviationLimit (10 rpm) for SpeedDeviationDelay (30 s); limit 0 = off. Retained in InletConfigDUT (Reset Origin with IN-15). Duplicate alarm-list row removed in FD-01 rev C. | Live test 2026-10-22 (PFC200 10.1.2.41, main 1a427c0, CAS plant 10.1.2.150, after Reset Origin): not tested yet.</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr"/>
@@ -1562,7 +1562,7 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>Implemented in CODESYS 2026-10-22 (not yet downloaded): LowPower / HighPower removed from PumpCommonError; their own alarms are notifications (AutoAcknowledge), as FD Tabell 7.</t>
+          <t>Implemented in CODESYS 2026-10-22 (not yet downloaded): LowPower / HighPower removed from PumpCommonError; their own alarms are notifications (AutoAcknowledge), as FD Tabell 7. | Live test 2026-10-22 (PFC200 10.1.2.41, main 1a427c0, CAS plant 10.1.2.150, after Reset Origin): not tested yet.</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr"/>
@@ -1826,7 +1826,7 @@
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>Automatic pump start/stop and rotation implemented in CODESYS 2026-10-22 (not yet downloaded/tested), InletSupervisor.PumpCount: candidates = InletConfig[i].InletPump.Enable AND auto AND not UNAVAILABLE/LOCKDOWN. Pen Start starts all candidates; with LIC01 in auto and no pump changing: stop the pump with most running days when the others would run &lt;= PumpTargetSpeed (85 rpm) for PumpRemoveDelay (15 min); start the standby with fewest running days when the share &gt;= PumpAddSpeed (115 rpm) for PumpAddDelay (2 min); rotation after PumpCycleTime (24 h) in REMOTE, make-before-break. Settings retained in PenConfig (Reset Origin on next download). Still open from the HOLD list: manual level setpoint, auto outlet close on pump stop, E-stop alarm.</t>
+          <t>Automatic pump start/stop and rotation implemented in CODESYS 2026-10-22 (not yet downloaded/tested), InletSupervisor.PumpCount: candidates = InletConfig[i].InletPump.Enable AND auto AND not UNAVAILABLE/LOCKDOWN. Pen Start starts all candidates; with LIC01 in auto and no pump changing: stop the pump with most running days when the others would run &lt;= PumpTargetSpeed (85 rpm) for PumpRemoveDelay (15 min); start the standby with fewest running days when the share &gt;= PumpAddSpeed (115 rpm) for PumpAddDelay (2 min); rotation after PumpCycleTime (24 h) in REMOTE, make-before-break. Settings retained in PenConfig (Reset Origin on next download). Still open from the HOLD list: manual level setpoint, auto outlet close on pump stop, E-stop alarm. | Live test 2026-10-22 (PFC200 10.1.2.41, main 1a427c0, CAS plant 10.1.2.150, after Reset Origin): pump count: with PumpTargetSpeed 115 / delay 60 s (test values) the pump with most running days stopped, 2 pumps at ~112 rpm, no flapping (PumpAddSpeed 125). Rotation (PumpCycleTime 2 min, test value): standby started first, old pump stopped once the new one was in REMOTE, level 5.1-7.1 cm during the handover (IN-31). All defaults restored afterwards (85 / 115 rpm, 15 / 2 min, 24 h).</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
@@ -6399,8 +6399,154 @@
       <c r="N87" s="2" t="n"/>
       <c r="O87" s="2" t="n"/>
     </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>OX-29</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>Oxygen</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>Code bug</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>O2 control valve outputs always 0 (CommonRIO mapping)</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>CommonRIO.OutputMapping wrote OutputData[20..22] (750-563, valves OV41-43) from OxySystem[i].Output.OxyControlValve.Output.RawPosition, which nothing writes; OxyControl writes OxySystem[i].OxyValve. The valves stayed at 4 mA (closed) whatever FIC asked; found in the live test 2026-10-22 (simulator valve_pct 0 while FIC opened 63 %, flow 0).</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>FB.RIO.CommonRIO.OutputMapping</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>Map words 20-22 from OxySystem[i].OxyValve.Output.RawPosition</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K88" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L88" s="2" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="M88" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="N88" s="2" t="inlineStr">
+        <is>
+          <t>Fixed in CODESYS 2026-10-22 (online change, to be pushed): OutputData[20..22] := OxySystem[i].OxyValve.Output.RawPosition. Unused OxySystemOutputDUT removed. Oxygen live test (flow per line, OIC01) still to repeat.</t>
+        </is>
+      </c>
+      <c r="O88" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>IN-31</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>Inlet</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>Observation</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>Level swing during pump rotation</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>Live test 2026-10-22: during a rotation handover the over-height moved 5.1-7.1 cm (setpoint 6 cm). The starting pump runs at its own START preset speed (~87 rpm) while the others give way, and the stopping pump's ramp-down follows.</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>InletSupervisor.PumpCount; CAS FD Inlet sec. 3.4</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>Accept; or soften: start the standby only when the share is near the START preset speed, or wait until the stopping pump has left level control</t>
+        </is>
+      </c>
+      <c r="I89" s="2" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K89" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L89" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M89" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="N89" s="2" t="n"/>
+      <c r="O89" s="2" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O87"/>
+  <autoFilter ref="A1:O89"/>
   <conditionalFormatting sqref="A2:O500">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>$L2="Fixed"</formula>

</xml_diff>

<commit_message>
CAS: LIC01 auto->manual bumpless (IN-32), FD Inlet rev. B1
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAS/Outstanding items.xlsx
+++ b/CAS/Outstanding items.xlsx
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O89"/>
+  <dimension ref="A1:O90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6544,6 +6544,83 @@
       </c>
       <c r="N89" s="2" t="n"/>
       <c r="O89" s="2" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>IN-32</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Inlet</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>Code bug</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>LIC01 auto -&gt; manual not bumpless</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>Seen on the HMI Inlet control page 2026-10-23: putting LIC01 in manual made the pumps jump to 40 rpm. In manual the output is LevelController.Command.ManualOutput x N, and ManualOutput is only written by the operator (0 if never set, limited to MinOutput 40 rpm). PIDController copies Output to ManualOutput on the manual edge, but only into its own input for that one scan.</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>FB.Inlet.InletSupervisor; FB.Components.PIDController; CAS FD Inlet sec. 3.3</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>Set ManualOutput to the current output per pump on the auto -&gt; manual edge</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K90" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L90" s="2" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="M90" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="N90" s="2" t="inlineStr">
+        <is>
+          <t>Fixed in CODESYS 2026-10-23 (FB.Inlet.InletSupervisor): on the rising edge of LevelController.Status.Manual, Command.ManualOutput := LIMIT(MinOutput, Output.OUT / N, MaxOutput), the current output per pump (bumpless, as the user asked). LevelManualLast starts TRUE so a download in manual keeps ManualOutput. Pre-compile clean; download and test on the rig pending. CAS FD Inlet rev. B1.</t>
+        </is>
+      </c>
+      <c r="O90" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:O89"/>

</xml_diff>

<commit_message>
CAS: LIC01 bumpless both ways, SP = PV on manual->auto (IN-32); OX-30 OIC01; FD Inlet B1
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAS/Outstanding items.xlsx
+++ b/CAS/Outstanding items.xlsx
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O90"/>
+  <dimension ref="A1:O91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6568,7 +6568,7 @@
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>LIC01 auto -&gt; manual not bumpless</t>
+          <t>LIC01 operator auto/manual not bumpless</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
@@ -6583,7 +6583,7 @@
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>Set ManualOutput to the current output per pump on the auto -&gt; manual edge</t>
+          <t>Auto -&gt; manual: ManualOutput := current output per pump. Manual -&gt; auto: setpoint := PV, PID restart with cleared integral (user, 2026-10-23)</t>
         </is>
       </c>
       <c r="I90" s="2" t="inlineStr">
@@ -6613,7 +6613,7 @@
       </c>
       <c r="N90" s="2" t="inlineStr">
         <is>
-          <t>Fixed in CODESYS 2026-10-23 (FB.Inlet.InletSupervisor): on the rising edge of LevelController.Status.Manual, Command.ManualOutput := LIMIT(MinOutput, Output.OUT / N, MaxOutput), the current output per pump (bumpless, as the user asked). LevelManualLast starts TRUE so a download in manual keeps ManualOutput. Pre-compile clean; download and test on the rig pending. CAS FD Inlet rev. B1.</t>
+          <t>Fixed in CODESYS 2026-10-23 (FB.Inlet.InletSupervisor), on the operator edge of LevelController.Status.Manual, only while the pen is started with pumps in level control and not on the first scan after a download: auto -&gt; manual sets Command.ManualOutput := LIMIT(MinOutput, Output.OUT / N, MaxOutput), the current output per pump; manual -&gt; auto sets Pen.Command.LevelSetpoint := PenStatus.OverHeight (if LevelControlOK), before the LevelControl call, so PIDController restarts Util.PID with RESET (integral cleared) and Y_OFFSET = the manual output (e = 0). Dead lines removed in FB.Components.PIDController (ManualOutput := Output on the manual edge wrote its own input for one scan). Checked against the Util.PID documentation. Pre-compile of PFC200_Sim clean; download and test on the rig pending. CAS FD Inlet rev. B1.</t>
         </is>
       </c>
       <c r="O90" s="2" t="inlineStr">
@@ -6621,6 +6621,75 @@
           <t>2026-10-23</t>
         </is>
       </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>OX-30</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>Oxygen</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>Code bug</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>OIC01 auto -&gt; manual not bumpless</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>Same as IN-32 on the oxygen side: in manual OIC01 outputs OxyController.Command.ManualOutput [kg/h total], written only by the operator. If never set it is 0: switching OIC01 to manual stops the O2 flow to the pen.</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>FB.Inlet.InletSupervisor (OIC01); IN-32</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>On the auto -&gt; manual edge set ManualOutput := current output (and SP := PV on manual -&gt; auto, as LIC01)</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="J91" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K91" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L91" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M91" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="N91" s="2" t="n"/>
+      <c r="O91" s="2" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:O89"/>

</xml_diff>

<commit_message>
CAS: OIC01 bumpless both ways, SP = PV on manual->auto (OX-30); FD Oxygen A2
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAS/Outstanding items.xlsx
+++ b/CAS/Outstanding items.xlsx
@@ -6680,7 +6680,7 @@
       </c>
       <c r="L91" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M91" s="2" t="inlineStr">
@@ -6688,8 +6688,16 @@
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="N91" s="2" t="n"/>
-      <c r="O91" s="2" t="n"/>
+      <c r="N91" s="2" t="inlineStr">
+        <is>
+          <t>Fixed in CODESYS 2026-10-23 (FB.Inlet.InletSupervisor), as LIC01 (IN-32), on the operator edge of OxyController.Status.Manual, only while the pen is started with lines in auto and not on the first scan after a download: auto -&gt; manual sets Command.ManualOutput := MAX(0, Output.OUT), the current total O2 flow; manual -&gt; auto sets PenConfig.OxySetpoint := PenStatus.PenOxygenLevel (if OxyControlOK), before the OxyControl call, so PIDController restarts with RESET (integral cleared) and Y_OFFSET = the manual output. Pre-compile of PFC200_Sim clean; download and test on the rig pending. CAS FD Oxygen rev. A2.</t>
+        </is>
+      </c>
+      <c r="O91" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:O89"/>

</xml_diff>

<commit_message>
CAS register: live test of the bumpless LIC01 / OIC01 transfers passed (IN-32, OX-30)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAS/Outstanding items.xlsx
+++ b/CAS/Outstanding items.xlsx
@@ -6613,7 +6613,7 @@
       </c>
       <c r="N90" s="2" t="inlineStr">
         <is>
-          <t>Fixed in CODESYS 2026-10-23 (FB.Inlet.InletSupervisor), on the operator edge of LevelController.Status.Manual, only while the pen is started with pumps in level control and not on the first scan after a download: auto -&gt; manual sets Command.ManualOutput := LIMIT(MinOutput, Output.OUT / N, MaxOutput), the current output per pump; manual -&gt; auto sets Pen.Command.LevelSetpoint := PenStatus.OverHeight (if LevelControlOK), before the LevelControl call, so PIDController restarts Util.PID with RESET (integral cleared) and Y_OFFSET = the manual output (e = 0). Dead lines removed in FB.Components.PIDController (ManualOutput := Output on the manual edge wrote its own input for one scan). Checked against Util 3.5.22.0 PID documentation; PIDController now limits Y_MANUAL to OutputMin..OutputMax (Util.PID does not limit Y in manual; live test 2026-10-23 on the old build showed OUT = 0 in manual). Live test 2026-10-23 before the download of this change: rig ran the old build (auto -&gt; manual gave OUT 0, pumps to 40 rpm; SP unchanged on manual -&gt; auto). Pre-compile of PFC200_Sim clean; download and test on the rig pending. CAS FD Inlet rev. B1.</t>
+          <t>Fixed in CODESYS 2026-10-23 (FB.Inlet.InletSupervisor), on the operator edge of LevelController.Status.Manual, only while the pen is started with pumps in level control and not on the first scan after a download: auto -&gt; manual sets Command.ManualOutput := LIMIT(MinOutput, Output.OUT / N, MaxOutput), the current output per pump; manual -&gt; auto sets Pen.Command.LevelSetpoint := PenStatus.OverHeight (if LevelControlOK), before the LevelControl call, so PIDController restarts Util.PID with RESET (integral cleared) and Y_OFFSET = the manual output (e = 0). Dead lines removed in FB.Components.PIDController (ManualOutput := Output on the manual edge wrote its own input for one scan). Checked against Util 3.5.22.0 PID documentation; PIDController now limits Y_MANUAL to OutputMin..OutputMax (Util.PID does not limit Y in manual; live test 2026-10-23 on the old build showed OUT = 0 in manual). Live test 2026-10-23 before the download of this change: rig ran the old build (auto -&gt; manual gave OUT 0, pumps to 40 rpm; SP unchanged on manual -&gt; auto). Pre-compile of PFC200_Sim clean; download and test on the rig pending. CAS FD Inlet rev. B1. | Live test 2026-10-23 on the new build (PFC200 10.1.2.41, inletControl, CAS plant 2.4.8 at 10.1.2.150): auto -&gt; manual at 6.08 cm: ManualOutput set to 73.90 rpm (= 221.69 total / 3), pumps 74.01 -&gt; 73.90 rpm, no step, level held 6.0 cm. Manual 80 rpm raised the level to 7.58 cm; manual -&gt; auto: SP 6.00 -&gt; 7.59 cm (= PV), total 240.00 -&gt; 239.93 rpm, held 7.57-7.64 cm. Passed.</t>
         </is>
       </c>
       <c r="O90" s="2" t="inlineStr">
@@ -6690,7 +6690,7 @@
       </c>
       <c r="N91" s="2" t="inlineStr">
         <is>
-          <t>Fixed in CODESYS 2026-10-23 (FB.Inlet.InletSupervisor), as LIC01 (IN-32), on the operator edge of OxyController.Status.Manual, only while the pen is started with lines in auto and not on the first scan after a download: auto -&gt; manual sets Command.ManualOutput := MAX(0, Output.OUT), the current total O2 flow; manual -&gt; auto sets PenConfig.OxySetpoint := PenStatus.PenOxygenLevel (if OxyControlOK), before the OxyControl call, so PIDController restarts with RESET (integral cleared) and Y_OFFSET = the manual output. Pre-compile of PFC200_Sim clean; download and test on the rig pending. CAS FD Oxygen rev. A2.</t>
+          <t>Fixed in CODESYS 2026-10-23 (FB.Inlet.InletSupervisor), as LIC01 (IN-32), on the operator edge of OxyController.Status.Manual, only while the pen is started with lines in auto and not on the first scan after a download: auto -&gt; manual sets Command.ManualOutput := MAX(0, Output.OUT), the current total O2 flow; manual -&gt; auto sets PenConfig.OxySetpoint := PenStatus.PenOxygenLevel (if OxyControlOK), before the OxyControl call, so PIDController restarts with RESET (integral cleared) and Y_OFFSET = the manual output. Pre-compile of PFC200_Sim clean; download and test on the rig pending. CAS FD Oxygen rev. A2. | Live test 2026-10-23 (same rig): auto -&gt; manual while OIC01 ramped: ManualOutput 26.00 kg/h = output at the edge, line flows continued 7.6 -&gt; 8.6 kg/h without a step. Manual -&gt; auto: O2 setpoint 8.00 -&gt; 2.26 mg/L (= pen O2), output continued from 26.00 kg/h. Passed; setpoint set back to 8.0. Seen: after the PLC download the three ATV650 drives were in EtHF (LFT 150, comm interrupt while enabled) and needed a fault reset before oxygenation could start.</t>
         </is>
       </c>
       <c r="O91" s="2" t="inlineStr">

</xml_diff>

<commit_message>
CAS register: IN-33 LIC01 resume after HOLD drops the returning pump
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAS/Outstanding items.xlsx
+++ b/CAS/Outstanding items.xlsx
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O91"/>
+  <dimension ref="A1:O92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6698,6 +6698,75 @@
           <t>2026-10-23</t>
         </is>
       </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>IN-33</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>Inlet</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>Code bug</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>LIC01 resume after HOLD drops the returning pump</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>Live test 2026-10-23 (sim update to 2.4.9 restarted the Framo servers: heartbeat lost, all pumps HOLD). Pumps 1-2 back in REMOTE, then pump 3 reset HOLD -&gt; REMOTE: all three pumps fell to the low 40s rpm and the over-height dropped (6 -&gt; about 3.3 cm) before LIC01 recovered. Cause: the resume cycle sums the speed of the pumps with Status.EnableLevelControl, but InletSupervisor runs before InletControl in Main, so the pump just back in REMOTE is not in level control yet; the resume total is that of the other two (about 2 x 74 rpm), and on the next scan it is shared by three (about 49 rpm each).</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>FB.Inlet.InletSupervisor (LevelResume, LevelResumeSpeed); PRG.Main call order</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>Include pumps in auto and REMOTE (they count for level control from the next scan) in the resume sum and its limits</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="J92" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K92" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L92" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M92" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="N92" s="2" t="n"/>
+      <c r="O92" s="2" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:O89"/>

</xml_diff>

<commit_message>
CAS: LIC01 resume after HOLD counts the returning pump (IN-33), FD Inlet B1
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAS/Outstanding items.xlsx
+++ b/CAS/Outstanding items.xlsx
@@ -6757,7 +6757,7 @@
       </c>
       <c r="L92" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M92" s="2" t="inlineStr">
@@ -6765,8 +6765,16 @@
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="N92" s="2" t="n"/>
-      <c r="O92" s="2" t="n"/>
+      <c r="N92" s="2" t="inlineStr">
+        <is>
+          <t>Fixed in CODESYS 2026-10-23 (FB.Inlet.InletSupervisor): the resume sum and the sharing loop (LevelPumps, RemotePumps, FixedSpeed, so also LevelN and the output limits) count a pump that is in auto and in REMOTE even before InletControl sets its EnableLevelControl (NOT Status.Manual AND State = Remote). Only differs in the scan a pump comes HOLD -&gt; REMOTE. Pre-compile of PFC200_Sim clean; download and test on the rig pending (reset one pump from HOLD while the others are in REMOTE). CAS FD Inlet rev. B1.</t>
+        </is>
+      </c>
+      <c r="O92" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:O89"/>

</xml_diff>

<commit_message>
CAS: IN-33 live test, second fix (resume when a pump joins in REMOTE); FD Inlet B1
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAS/Outstanding items.xlsx
+++ b/CAS/Outstanding items.xlsx
@@ -6757,7 +6757,7 @@
       </c>
       <c r="L92" s="2" t="inlineStr">
         <is>
-          <t>Fixed</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="M92" s="2" t="inlineStr">
@@ -6767,7 +6767,7 @@
       </c>
       <c r="N92" s="2" t="inlineStr">
         <is>
-          <t>Fixed in CODESYS 2026-10-23 (FB.Inlet.InletSupervisor): the resume sum and the sharing loop (LevelPumps, RemotePumps, FixedSpeed, so also LevelN and the output limits) count a pump that is in auto and in REMOTE even before InletControl sets its EnableLevelControl (NOT Status.Manual AND State = Remote). Only differs in the scan a pump comes HOLD -&gt; REMOTE. Pre-compile of PFC200_Sim clean; download and test on the rig pending (reset one pump from HOLD while the others are in REMOTE). CAS FD Inlet rev. B1.</t>
+          <t>Fixed in CODESYS 2026-10-23 (FB.Inlet.InletSupervisor): the resume sum and the sharing loop (LevelPumps, RemotePumps, FixedSpeed, so also LevelN and the output limits) count a pump that is in auto and in REMOTE even before InletControl sets its EnableLevelControl (NOT Status.Manual AND State = Remote). Only differs in the scan a pump comes HOLD -&gt; REMOTE. Pre-compile of PFC200_Sim clean; download and test on the rig pending (reset one pump from HOLD while the others are in REMOTE). CAS FD Inlet rev. B1. | Live test 2026-10-23 of the first fix: heartbeat of pump 3 lost (simulator fault): PLC UNAVAILABLE, PCC HOLD at 88 rpm, LIC01 frozen at 221.95 total (pumps 1-2 at 73.98 rpm), as designed. Link back: the freeze ended at once (state read other than HOLD for a cycle), LIC01 ran on pumps 1-2 (2 x 69 rpm) with pump 3 still in HOLD. Reset of pump 3 then dropped the share 67.9 -&gt; 45.3 rpm (all pumps to about 51 rpm, level 6.4 -&gt; 4.6 cm): first fix incomplete. Second fix (CODESYS 2026-10-23): a pump in auto that joins level control straight in REMOTE (NOT EnableLevelControl, auto, REMOTE, pen started, no freeze) triggers LevelResume, so LIC01 restarts from the summed actual speed including it. Pre-compile clean; load and retest pending.</t>
         </is>
       </c>
       <c r="O92" s="2" t="inlineStr">

</xml_diff>

<commit_message>
CAS: InletSupervisor split into FBs, LIC01 rules R1/R2 (DEC9: no freeze on HOLD); FDs, program design, register GEN-04 / IN-33
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAS/Outstanding items.xlsx
+++ b/CAS/Outstanding items.xlsx
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O92"/>
+  <dimension ref="A1:O93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6757,7 +6757,7 @@
       </c>
       <c r="L92" s="2" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M92" s="2" t="inlineStr">
@@ -6767,10 +6767,87 @@
       </c>
       <c r="N92" s="2" t="inlineStr">
         <is>
-          <t>Fixed in CODESYS 2026-10-23 (FB.Inlet.InletSupervisor): the resume sum and the sharing loop (LevelPumps, RemotePumps, FixedSpeed, so also LevelN and the output limits) count a pump that is in auto and in REMOTE even before InletControl sets its EnableLevelControl (NOT Status.Manual AND State = Remote). Only differs in the scan a pump comes HOLD -&gt; REMOTE. Pre-compile of PFC200_Sim clean; download and test on the rig pending (reset one pump from HOLD while the others are in REMOTE). CAS FD Inlet rev. B1. | Live test 2026-10-23 of the first fix: heartbeat of pump 3 lost (simulator fault): PLC UNAVAILABLE, PCC HOLD at 88 rpm, LIC01 frozen at 221.95 total (pumps 1-2 at 73.98 rpm), as designed. Link back: the freeze ended at once (state read other than HOLD for a cycle), LIC01 ran on pumps 1-2 (2 x 69 rpm) with pump 3 still in HOLD. Reset of pump 3 then dropped the share 67.9 -&gt; 45.3 rpm (all pumps to about 51 rpm, level 6.4 -&gt; 4.6 cm): first fix incomplete. Second fix (CODESYS 2026-10-23): a pump in auto that joins level control straight in REMOTE (NOT EnableLevelControl, auto, REMOTE, pen started, no freeze) triggers LevelResume, so LIC01 restarts from the summed actual speed including it. Pre-compile clean; load and retest pending.</t>
+          <t>Fixed in CODESYS 2026-10-23 (FB.Inlet.InletSupervisor): the resume sum and the sharing loop (LevelPumps, RemotePumps, FixedSpeed, so also LevelN and the output limits) count a pump that is in auto and in REMOTE even before InletControl sets its EnableLevelControl (NOT Status.Manual AND State = Remote). Only differs in the scan a pump comes HOLD -&gt; REMOTE. Pre-compile of PFC200_Sim clean; download and test on the rig pending (reset one pump from HOLD while the others are in REMOTE). CAS FD Inlet rev. B1. | Live test 2026-10-23 of the first fix: heartbeat of pump 3 lost (simulator fault): PLC UNAVAILABLE, PCC HOLD at 88 rpm, LIC01 frozen at 221.95 total (pumps 1-2 at 73.98 rpm), as designed. Link back: the freeze ended at once (state read other than HOLD for a cycle), LIC01 ran on pumps 1-2 (2 x 69 rpm) with pump 3 still in HOLD. Reset of pump 3 then dropped the share 67.9 -&gt; 45.3 rpm (all pumps to about 51 rpm, level 6.4 -&gt; 4.6 cm): first fix incomplete. Second fix (CODESYS 2026-10-23): a pump in auto that joins level control straight in REMOTE (NOT EnableLevelControl, auto, REMOTE, pen started, no freeze) triggers LevelResume, so LIC01 restarts from the summed actual speed including it. Pre-compile clean; load and retest pending. | Replaced 2026-10-23 by the split of InletSupervisor (GEN-04): rules R1/R2 instead of tracking, freeze and resume. A pump in HOLD or with its link lost counts in LIC01's total at its own (last) speed and the pumps in REMOTE keep controlling (user decision: the three PCCs do not know each other's state, DEC9 in CAS FD Inlet); a reset from HOLD only evens out the speeds. Pump states read directly in InletPumpSet, so no one-scan lag. Pre-compile of PFC200_Sim clean; load and live test pending.</t>
         </is>
       </c>
       <c r="O92" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>GEN-04</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>InletSupervisor split into function blocks</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>InletSupervisor had grown to about 700 lines with five jobs and many state flags. Split after Cooling, Software Engineering for Real-Time Systems (2020) sec. 4.2 and 7.3.7 (one function per module, data coupling by value, explicit states, fixed execution order).</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>FB.Inlet.InletSupervisor, InletPumpSet, PenLevelControl, PumpCount, PenOxygenControl, PenSequence; FB.Components.ControllerMode; ENUM.LevelControlMode; CAS FD Inlet B1, CAS FD Oxygen A2, CAS program design</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>Split the FB; keep the interface</t>
+        </is>
+      </c>
+      <c r="I93" s="2" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="J93" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K93" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L93" s="2" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="M93" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="N93" s="2" t="inlineStr">
+        <is>
+          <t>Done in CODESYS 2026-10-23: InletSupervisor (about 80 lines) calls InletPumpSet (pumps counted / controlled), PenLevelControl (LIC01, mode enum Idle/Manual/SafeOutput/Tracking/Auto), PumpCount (unchanged logic), PenOxygenControl (OIC01, unchanged), PenSequence (pen statechart, called last: one-cycle delay for the others) in a fixed order; ControllerMode (one instance per loop) does the bumpless operator transfers. Same interface: Main, GVLMain and the HMI unchanged. Manual output of LIC01 is now per pump in REMOTE. IN-nn and FD references removed from code comments. Pre-compile of PFC200_Sim clean; load and live tests pending (start from drained, operator auto/manual, one pump HOLD and back, all links lost, trip, rotation, OIC01).</t>
+        </is>
+      </c>
+      <c r="O93" s="2" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>

</xml_diff>

<commit_message>
CAS register: Framo SCD 7664-017-1 findings (IN-01/02/03/12/13, new IN-34)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAS/Outstanding items.xlsx
+++ b/CAS/Outstanding items.xlsx
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O93"/>
+  <dimension ref="A1:O94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -870,7 +870,11 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr"/>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>Framo SCD 7664-017-1 (received 2026-10-23): logic only, no OPC UA node names or data types (addresses "TBA"). CAS signals: HMI START (M01-U04), HMI STOP (M01-U05), HMI RESET (M01-U11), REMOTE CONTROL (UY-012), SPEED SETPOINT (M01-U56), INHIBIT START (M01-Q03) from CAS; STARTING SEQU ACTIVE (UI-010), FAILED TO START (UA-011) to CAS. No pump state (UNAVAILABLE/AVAILABLE/START/REMOTE/HOLD/LOCKDOWN) as the PLC expects. See IN-34.</t>
+        </is>
+      </c>
       <c r="O5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
@@ -939,7 +943,11 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr"/>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>Framo SCD 7664-017-1 (received 2026-10-23): heartbeat is a Framo standard FB #HRTB (UI-100); its fault output is ORed with HMI STOP: heartbeat loss resets the start latch and STOPS the pump. No HOLD at preset speed. Interval/timeout not given.</t>
+        </is>
+      </c>
       <c r="O6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
@@ -1008,7 +1016,11 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr"/>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>Framo SCD 7664-017-1 (received 2026-10-23): no HOLD or LOCKDOWN state in the SCD. Heartbeat loss = stop; drive trip / FSL trip -&gt; pump block YF, cleared by HMI RESET (also resets the drive). Ask Framo whether HOLD (rev B spec) still exists.</t>
+        </is>
+      </c>
       <c r="O7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
@@ -1629,7 +1641,11 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>Framo SCD 7664-017-1 (received 2026-10-23): air evacuation: start latch AND no stop AND release valve UY-004A closed opens comp. air valve UY-003A (ejector) until LSH-002A; pump start only when LSL-001A is wet; NOT LSL or sensor deviation (LSH AND NOT LSL, UA-001A) trips the pump (FSL). HMI STOP opens the release valve.</t>
+        </is>
+      </c>
       <c r="O16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
@@ -1694,7 +1710,11 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="N17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>Framo SCD 7664-017-1 (received 2026-10-23): start: drive runs at a fixed 40 rpm start setpoint ("adjust while commissioning"); READY TO REMOTE CNTRL (UI-013) 30 s after DRIVE RUNNING; speed from CAS only when CAS gives REMOTE CONTROL (UY-012) and ready to remote. FAILED TO START (UA-011) when the start sequence stays active for "time" (not given).</t>
+        </is>
+      </c>
       <c r="O17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
@@ -6852,6 +6872,75 @@
           <t>2026-10-23</t>
         </is>
       </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>IN-34</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>Inlet</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>Inconsistency</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>Framo SCD 7664-017-1 vs the PLC interface</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>First official Framo document (SCD 7664-017-1, IEC PAS 63131, drawn 24.07.2026, checked 05.08.2026, rev -). Differs from what the PLC implements (Framo spec rev B): 1) no pump state machine, only status bits (drive ready / running / in remote / tripped / start inhibit, starting sequence active, ready to remote); 2) heartbeat loss stops the pump (no HOLD); 3) a separate REMOTE CONTROL command (UY-012) from CAS is needed before CAS sets the speed, else 40 rpm; 4) a new INHIBIT START (M01-Q03) from CAS; 5) start at 40 rpm for 30 s (PLC and simulator assume about 87 rpm and a short START); 6) alarm set differs (earth leakage, short circuit, STO, stall, power unit loss, overspeed, phase loss, comm fault; no E-stop, motor temperature, UPS, emergency run, low/high power, pump stopped); 7) no OPC UA node list (TBA).</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>Framo 7664-017-1 SCD; 7664-021-1 P&amp;ID; PRG.FramoDataProcessing; FB.Inlet.InletControl; CAS FD Inlet sec. 3.5</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>Ask Framo for the OPC UA signal list and the state model; decide HOLD vs stop on heartbeat loss; add REMOTE CONTROL and INHIBIT START to the PLC</t>
+        </is>
+      </c>
+      <c r="I94" s="2" t="inlineStr">
+        <is>
+          <t>Framo</t>
+        </is>
+      </c>
+      <c r="J94" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K94" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L94" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M94" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="N94" s="2" t="n"/>
+      <c r="O94" s="2" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:O89"/>

</xml_diff>

<commit_message>
CAS register: Framo P&ID 7664-021-1 findings (IN-12, IN-16, IN-34)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAS/Outstanding items.xlsx
+++ b/CAS/Outstanding items.xlsx
@@ -1643,7 +1643,7 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>Framo SCD 7664-017-1 (received 2026-10-23): air evacuation: start latch AND no stop AND release valve UY-004A closed opens comp. air valve UY-003A (ejector) until LSH-002A; pump start only when LSL-001A is wet; NOT LSL or sensor deviation (LSH AND NOT LSL, UA-001A) trips the pump (FSL). HMI STOP opens the release valve.</t>
+          <t>Framo SCD 7664-017-1 (received 2026-10-23): air evacuation: start latch AND no stop AND release valve UY-004A closed opens comp. air valve UY-003A (ejector) until LSH-002A; pump start only when LSL-001A is wet; NOT LSL or sensor deviation (LSH AND NOT LSL, UA-001A) trips the pump (FSL). HMI STOP opens the release valve. | Framo P&amp;ID 7664-021-1 (08.09.26, received 2026-10-23): per inlet one vacuum chamber with ejector: compressed-air valve UY-003x (ZSO/ZSC-003x), release valve UY-004x (ZSO/ZSC-004x), LSH-002x, LSL-001x; all their signals go to the Framo UCP only (none to the client system). No compressed-air pressure transmitter, although the PLC reads Framo_n.PressureCompressedAir; the PLC has one status bit per valve (StatusV001/V002), the P&amp;ID two limit switches per valve. Compressed air supply comes from client scope (one line to all three units). Drafting error: the release valve of unit A is tagged UY-004B (B, C correct).</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr"/>
@@ -1913,7 +1913,11 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="N20" s="2" t="inlineStr"/>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>Framo P&amp;ID 7664-021-1 (08.09.26, received 2026-10-23): Framo tags: pumps P-01A/B/C, level switches LSL-001A..C / LSH-002A..C, valves UY-003A..C / UY-004A..C (SCD uses the A tags). FD uses PM31..33 / PU41..43, LSL31 / LSH32, XV31 / XV32; PLC uses LSL01 / LSH02, V001 / V002.</t>
+        </is>
+      </c>
       <c r="O20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
@@ -6939,7 +6943,11 @@
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="N94" s="2" t="n"/>
+      <c r="N94" s="2" t="inlineStr">
+        <is>
+          <t>Framo P&amp;ID 7664-021-1 (08.09.26, received 2026-10-23): P&amp;ID: no instruments on the pumps (only VSD per pump over Ethernet); no E-stop shown. The P&amp;ID draws a client datalink from PDIC-01 straight to the three VSDs, while the SCD sends the speed setpoint through the Framo UCP (M01-U56): to clear with Framo. Client-scope parts of the P&amp;ID (oxygen, outlet, level measurement) are out of date and not used.</t>
+        </is>
+      </c>
       <c r="O94" s="2" t="n"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
CAS register: Framo SCD / P&ID inconsistencies IN-35..IN-38
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAS/Outstanding items.xlsx
+++ b/CAS/Outstanding items.xlsx
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O94"/>
+  <dimension ref="A1:O98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6945,10 +6945,286 @@
       </c>
       <c r="N94" s="2" t="inlineStr">
         <is>
-          <t>Framo P&amp;ID 7664-021-1 (08.09.26, received 2026-10-23): P&amp;ID: no instruments on the pumps (only VSD per pump over Ethernet); no E-stop shown. The P&amp;ID draws a client datalink from PDIC-01 straight to the three VSDs, while the SCD sends the speed setpoint through the Framo UCP (M01-U56): to clear with Framo. Client-scope parts of the P&amp;ID (oxygen, outlet, level measurement) are out of date and not used.</t>
+          <t>Framo P&amp;ID 7664-021-1 (08.09.26, received 2026-10-23): P&amp;ID: no instruments on the pumps (only VSD per pump over Ethernet); no E-stop shown. The P&amp;ID draws a client datalink from PDIC-01 straight to the three VSDs, while the SCD sends the speed setpoint through the Framo UCP (M01-U56): to clear with Framo. Client-scope parts of the P&amp;ID (oxygen, outlet, level measurement) are out of date and not used. | Details split out 2026-10-23: IN-35 (Remote control / speed setpoint mode), IN-36 (start/stop pulse or level, restart after heartbeat loss), IN-37 (speed setpoint path P&amp;ID vs SCD), IN-38 (tags and evacuation signals).</t>
         </is>
       </c>
       <c r="O94" s="2" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>IN-35</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>Inlet</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>Inconsistency</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>SCD: speed setpoint mode (Remote control, LA / LM)</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>SCD 7664-017-1 sheet 3: SPEED SETPOINT TO DRIVE (M01-U56, CAS/HA) has X = 40 rpm start setpoint, LA = REMOTE CONTROL (UY-012, CAS/HB command from CAS) and LM = NOT READY TO REMOTE CNTRL (UI-013, TRUE until 30 s after drive running). In the HA template Auto = follow X, Manual = operator (CAS) value; read that way, Remote control gives 40 rpm and "not ready" gives the CAS setpoint, the opposite of the intent (rev B spec: fixed speed during start, CAS speed in remote). The PLC does not send a Remote control command today.</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>Framo 7664-017-1 sheet 3; PRG.FramoDataProcessing</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>Framo to confirm: is UY-012 a command from CAS or set by their logic; which mode gives 40 rpm and which the CAS setpoint (LA / LM swapped?); level or pulse; what happens if Remote control drops while running</t>
+        </is>
+      </c>
+      <c r="I95" s="2" t="inlineStr">
+        <is>
+          <t>Framo</t>
+        </is>
+      </c>
+      <c r="J95" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K95" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L95" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M95" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="N95" s="2" t="n"/>
+      <c r="O95" s="2" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>IN-36</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>Inlet</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>Missing info</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>SCD: start / stop pulse or level, restart after heartbeat loss</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>SCD sheet 2: HMI START sets a memory (SR, reset dominant), HMI STOP or heartbeat fault resets it; pump block M01 (SBE) has XH = start, XL = stop and latches. So a pulse is enough. The PLC writes Framo_n.Start.Active / Stop.Active as levels (Start held while the PLC wants the pump started and it is AVAILABLE). Consequence: after a heartbeat loss Framo stops the pump; when the link is back the PLC sees AVAILABLE with its start request still active and sends Start again, so the pump restarts by itself.</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>Framo 7664-017-1 sheets 2-3; FB.Inlet.InletControl; PRG.FramoDataProcessing; IN-28</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>Framo to confirm edge or level on XH / XL and what they expect from CAS; decide whether a pump stopped by heartbeat loss may restart automatically when the link is back</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="inlineStr">
+        <is>
+          <t>Framo / Internal</t>
+        </is>
+      </c>
+      <c r="J96" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K96" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L96" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M96" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="N96" s="2" t="n"/>
+      <c r="O96" s="2" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>IN-37</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>Inlet</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>Inconsistency</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>Speed setpoint path: P&amp;ID vs SCD</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>P&amp;ID 7664-021-1 draws a client datalink (Ethernet) from PDIC-01 straight to the three VSDs; SCD 7664-017-1 sends the speed setpoint through the Framo UCP (M01-U56) with Remote control and start setpoint logic. The PLC writes Framo_n.SpeedSetpoint over OPC UA to the Framo controller.</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>Framo 7664-021-1; Framo 7664-017-1 sheet 3; PRG.FramoDataProcessing</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>Framo to confirm the speed setpoint goes CAS -&gt; Framo UCP -&gt; VSD (as the SCD), and correct the P&amp;ID</t>
+        </is>
+      </c>
+      <c r="I97" s="2" t="inlineStr">
+        <is>
+          <t>Framo</t>
+        </is>
+      </c>
+      <c r="J97" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K97" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L97" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M97" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="N97" s="2" t="n"/>
+      <c r="O97" s="2" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>IN-38</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>Inlet</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>Physical</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>Inconsistency</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>Framo P&amp;ID / SCD tags and evacuation signals</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>P&amp;ID 7664-021-1: release valve of unit A tagged UY-004B (unit B and C: UY-004B, UY-004C; SCD: UY-004A). Valve position switches ZSO / ZSC on the P&amp;ID, ZSL / ZSH on the SCD. No compressed-air pressure transmitter on the P&amp;ID or SCD, but the PLC reads Framo_n.PressureCompressedAir. Two limit switches per valve on the P&amp;ID, one status bit per valve in the PLC (StatusV001 / V002). All evacuation signals go to the Framo UCP only. No E-stop on either document.</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>Framo 7664-021-1; Framo 7664-017-1 sheet 2; PRG.FramoDataProcessing; IN-12, IN-16</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>Framo to correct the tag of unit A and give the OPC UA signals for the evacuation (valve positions, level switches, any air pressure); adapt the PLC to the final list</t>
+        </is>
+      </c>
+      <c r="I98" s="2" t="inlineStr">
+        <is>
+          <t>Framo</t>
+        </is>
+      </c>
+      <c r="J98" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K98" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L98" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M98" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="N98" s="2" t="n"/>
+      <c r="O98" s="2" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:O89"/>

</xml_diff>

<commit_message>
CAS register: CPU and task monitor measurements in IN-21
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAS/Outstanding items.xlsx
+++ b/CAS/Outstanding items.xlsx
@@ -2270,7 +2270,11 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="N25" s="2" t="inlineStr"/>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23 measured on the PFC200 (10.1.2.41): htop CPU 86 %, load average 2.6 (single core); task monitor: Task 20 ms avg 3.0 / max 5.0 ms (about 15 %), OPC_Processing 50 ms avg 0.11 / max 0.68 ms, DatasourcesTask 50 ms avg 3.4 / max 154 ms, jitter up to 104 ms. IEC tasks about 22 %: the rest is runtime threads (OPC UA server for the HMI / 7 sessions, OPC UA client of the data sources). Next: thread names, HMI-off test, data source update rate; then a task split (20 ms outlet + CommonRIO, 100 ms control incl. FramoDataProcessing, data sources lowest) and watchdogs per task. Task config kept as is for now.</t>
+        </is>
+      </c>
       <c r="O25" s="2" t="inlineStr"/>
     </row>
     <row r="26">

</xml_diff>

<commit_message>
CAS register: IN-32 level transmitter span for Hs 2.0 m, IN-33 frozen RIO link with CommOK TRUE; OX-29 confirmed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAS/Outstanding items.xlsx
+++ b/CAS/Outstanding items.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Outstanding items'!$A$1:$O$89</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Outstanding items'!$A$1:$O$100</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O98"/>
+  <dimension ref="A1:O100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6495,7 +6495,7 @@
       </c>
       <c r="N88" s="2" t="inlineStr">
         <is>
-          <t>Fixed in CODESYS 2026-10-22 (online change, to be pushed): OutputData[20..22] := OxySystem[i].OxyValve.Output.RawPosition. Unused OxySystemOutputDUT removed. Oxygen live test (flow per line, OIC01) still to repeat.</t>
+          <t>Fixed in CODESYS 2026-10-22 (online change, to be pushed): OutputData[20..22] := OxySystem[i].OxyValve.Output.RawPosition. Unused OxySystemOutputDUT removed. Confirmed 2026-10-26: lines 2 and 3 deliver 103.6 kg/h with the valves at 99 %, pen O2 rising (5.0 mg/L); line 1 after the IN-33 recovery 41 kg/h and rising.</t>
         </is>
       </c>
       <c r="O88" s="2" t="inlineStr">
@@ -7230,8 +7230,146 @@
       <c r="N98" s="2" t="n"/>
       <c r="O98" s="2" t="n"/>
     </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>IN-32</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>Inlet</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>Physical</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>Inconsistency</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>Level transmitter span too small for Hs 2.0 m</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>The 750-455 level signals span 0-2 m. The transmitters hang on the floater, so each reading moves with the wave minus the heave: at Hs 2.0 m / Tp 4.5 s (design basis wave model) sigma 53.5 cm inside (LT0x) and 40.5 cm outside (LT2x), about +-2.1 m / +-1.6 m in a 3 h storm (4 sigma). Clipped crests bias the mean: sim 2026-10-26 at Hs 2.0 m the PLC read over-height -3 cm while the true value was +20-23 cm, LIC01 ran the pumps to max and the pen overfilled.</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>design_basis.toml [waves], [instruments.level_span]; casdesign.waves WaveField.hs(); IN-24</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t>Span 0-5 m inside (normal level ~2.5 m), 0-4 m outside (normal ~2.0 m); minimum 4.3 / 3.3 m (4 sigma). 750-455 resolution 2.4 / 2.0 mm per step (quantization dithered by the waves, filtered PV much finer); or a 16-bit AI module; or a stilling well. PLC: treat readings at the span limits as suspect (drop the pair). Heave / slosh parameters are assumptions: measure on the prototype.</t>
+        </is>
+      </c>
+      <c r="I99" s="2" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="J99" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K99" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L99" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M99" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="N99" s="2" t="n"/>
+      <c r="O99" s="2" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>IN-33</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>Inlet</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>Code bug</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>RIO / drive link frozen while CommOK stays TRUE</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>Sim 2026-10-26: InletRIO 1 and its oxy pump drive stopped updating (raw level and PT words constant for minutes while the simulator's words moved with the waves) but SCL.sModbusMasterTCP.comOk stayed TRUE, so InletRIO.Status.CommOK and OxyPump.Status.CommunicationOK were TRUE and InputMapping kept the last values. Effects: level pair 1 frozen at -38 cm (wrong LIC01 PV, IN-19 fix not triggered), oxy pump 1 shown running at 40.9 Hz / 4 bar while the drive had tripped on EtHF (comm interrupt), no O2 on line 1, no alarm. Probably since the simulator pod restart. Recovered by toggling InletRIOConfig[0].Enabled / DriveEnabled, then OxyPump Reset.</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>FB.RIO.InletRIO (Status.CommOK := RioMaster.comOk); SCL.sModbusMasterTCP; OX-28, IN-19</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>Data-freshness watchdog per master: the library's request/response counter or last-response time if it has one, else a value that must change (e.g. 750-362 / ATV status or a counter) -&gt; CommOK FALSE + alarm after a timeout, and restart the master (enable FALSE/TRUE). Check the same for CommonRIO. Ask ScaleAQ library owner how comOk is defined.</t>
+        </is>
+      </c>
+      <c r="I100" s="2" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="J100" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K100" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L100" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M100" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="N100" s="2" t="n"/>
+      <c r="O100" s="2" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O89"/>
+  <autoFilter ref="A1:O100"/>
   <conditionalFormatting sqref="A2:O500">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>$L2="Fixed"</formula>

</xml_diff>

<commit_message>
CAS: drive fault reset by acknowledging the DriveError alarm (OX-30, FD Oxygen)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAS/Outstanding items.xlsx
+++ b/CAS/Outstanding items.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Outstanding items'!$A$1:$O$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Outstanding items'!$A$1:$O$101</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O100"/>
+  <dimension ref="A1:O101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7368,8 +7368,81 @@
       <c r="N100" s="2" t="n"/>
       <c r="O100" s="2" t="n"/>
     </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>OX-30</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>Oxygen</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>Drive fault reset by acknowledging the alarm</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>Live test 2026-10-26: oxy pump 1's ATV650 had tripped on EtHF (Ethernet comm. interrupt) and the operator had no way to reset it from the overview. Wanted flow: VSD trips -&gt; PLC alarm -&gt; the operator acknowledges it like any alarm -&gt; the PLC sends the fault reset -&gt; the alarm clears when the drive reads healthy.</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>FB.OxySystem.OxyControl (Drive Reset), OxyPumpATV650, heimdall-cas-hmi PR #13</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr"/>
+      <c r="I101" s="2" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="J101" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K101" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L101" s="2" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="M101" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="N101" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26: OxyControl Drive(Reset := OxyPump.Command.Reset OR OxyPump.AlarmAck.DriveError): the HMI's Reset oxy pump or acknowledging the DriveError alarm (also Acknowledge all) sends 0x0080 for 0.5 s; the alarm clears once ETA has no fault. HMI overview shows the drive fault (LFT) and a Reset oxy pump button (PR #13). To be tested in the sim.</t>
+        </is>
+      </c>
+      <c r="O101" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O100"/>
+  <autoFilter ref="A1:O101"/>
   <conditionalFormatting sqref="A2:O500">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>$L2="Fixed"</formula>

</xml_diff>

<commit_message>
CAS register: Framo SCD follow-ups IN-41..45, OX-32/33, GEN-05; unique IDs
- IN-41 heartbeat loss stops the pump (SCD) while LIC01 counts it; local mode asked from Framo
- IN-42 pump state derived from Framo status bits (state machine removed, meeting 2026-10-28)
- IN-43 start sequence timing / duplicate Start failed, IN-44 Reset handshake without states
- IN-45 vacuum chamber gas build-up trips the pump (PUMP FSL), release valve questions
- OX-32 oxygenation permit without REMOTE, OX-33 oxygenation not restored after PLC restart
- GEN-05 Framo data sources lost after the PLC security change
- Duplicates renumbered: IN-32 (span) -> IN-39, IN-33 (frozen link) -> IN-40, OX-30 (drive fault) -> OX-31
- Notes on IN-11, IN-13, IN-34 from the SCD review and the Framo meeting

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAS/Outstanding items.xlsx
+++ b/CAS/Outstanding items.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Outstanding items'!$A$1:$O$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Outstanding items'!$A$1:$O$109</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O101"/>
+  <dimension ref="A1:O109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>Implemented in CODESYS 2026-10-22 (not yet downloaded): LowPower / HighPower removed from PumpCommonError; their own alarms are notifications (AutoAcknowledge), as FD Tabell 7. | Live test 2026-10-22 (PFC200 10.1.2.41, main 1a427c0, CAS plant 10.1.2.150, after Reset Origin): not tested yet.</t>
+          <t>Implemented in CODESYS 2026-10-22 (not yet downloaded): LowPower / HighPower removed from PumpCommonError; their own alarms are notifications (AutoAcknowledge), as FD Tabell 7. | Live test 2026-10-22 (PFC200 10.1.2.41, main 1a427c0, CAS plant 10.1.2.150, after Reset Origin): not tested yet. | SCD review 2026-10-28: SCD 7664-017-1 sheet 4 has no LowPower / HighPower alarms; the change may be moot once the final alarm list is known.</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr"/>
@@ -1712,7 +1712,7 @@
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>Framo SCD 7664-017-1 (received 2026-10-23): start: drive runs at a fixed 40 rpm start setpoint ("adjust while commissioning"); READY TO REMOTE CNTRL (UI-013) 30 s after DRIVE RUNNING; speed from CAS only when CAS gives REMOTE CONTROL (UY-012) and ready to remote. FAILED TO START (UA-011) when the start sequence stays active for "time" (not given).</t>
+          <t>Framo SCD 7664-017-1 (received 2026-10-23): start: drive runs at a fixed 40 rpm start setpoint ("adjust while commissioning"); READY TO REMOTE CNTRL (UI-013) 30 s after DRIVE RUNNING; speed from CAS only when CAS gives REMOTE CONTROL (UY-012) and ready to remote. FAILED TO START (UA-011) when the start sequence stays active for "time" (not given). | SCD review 2026-10-28: the start setpoint is given as 40 rpm, so the speed setpoint is most likely in rpm (to confirm in the OPC UA list). MOTOR RUNNING DAYS is on SCD sheet 4, so run-time rotation (IN-15) has its source.</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr"/>
@@ -6495,7 +6495,7 @@
       </c>
       <c r="N88" s="2" t="inlineStr">
         <is>
-          <t>Fixed in CODESYS 2026-10-22 (online change, to be pushed): OutputData[20..22] := OxySystem[i].OxyValve.Output.RawPosition. Unused OxySystemOutputDUT removed. Confirmed 2026-10-26: lines 2 and 3 deliver 103.6 kg/h with the valves at 99 %, pen O2 rising (5.0 mg/L); line 1 after the IN-33 recovery 41 kg/h and rising.</t>
+          <t>Fixed in CODESYS 2026-10-22 (online change, to be pushed): OutputData[20..22] := OxySystem[i].OxyValve.Output.RawPosition. Unused OxySystemOutputDUT removed. Confirmed 2026-10-26: lines 2 and 3 deliver 103.6 kg/h with the valves at 99 %, pen O2 rising (5.0 mg/L); line 1 after the IN-40 recovery 41 kg/h and rising.</t>
         </is>
       </c>
       <c r="O88" s="2" t="inlineStr">
@@ -6949,7 +6949,7 @@
       </c>
       <c r="N94" s="2" t="inlineStr">
         <is>
-          <t>Framo P&amp;ID 7664-021-1 (08.09.26, received 2026-10-23): P&amp;ID: no instruments on the pumps (only VSD per pump over Ethernet); no E-stop shown. The P&amp;ID draws a client datalink from PDIC-01 straight to the three VSDs, while the SCD sends the speed setpoint through the Framo UCP (M01-U56): to clear with Framo. Client-scope parts of the P&amp;ID (oxygen, outlet, level measurement) are out of date and not used. | Details split out 2026-10-23: IN-35 (Remote control / speed setpoint mode), IN-36 (start/stop pulse or level, restart after heartbeat loss), IN-37 (speed setpoint path P&amp;ID vs SCD), IN-38 (tags and evacuation signals).</t>
+          <t>Framo P&amp;ID 7664-021-1 (08.09.26, received 2026-10-23): P&amp;ID: no instruments on the pumps (only VSD per pump over Ethernet); no E-stop shown. The P&amp;ID draws a client datalink from PDIC-01 straight to the three VSDs, while the SCD sends the speed setpoint through the Framo UCP (M01-U56): to clear with Framo. Client-scope parts of the P&amp;ID (oxygen, outlet, level measurement) are out of date and not used. | Details split out 2026-10-23: IN-35 (Remote control / speed setpoint mode), IN-36 (start/stop pulse or level, restart after heartbeat loss), IN-37 (speed setpoint path P&amp;ID vs SCD), IN-38 (tags and evacuation signals). | Framo meeting 2026-10-28: Framo confirmed the pump state machine (UNAVAILABLE ... LOCKDOWN) is removed; the PCC publishes status bits only. The PLC must derive the pump state itself (IN-42). ScaleAQ asked for a local mode on heartbeat loss (IN-41).</t>
         </is>
       </c>
       <c r="O94" s="2" t="n"/>
@@ -7233,7 +7233,7 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>IN-32</t>
+          <t>IN-39</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
@@ -7296,13 +7296,17 @@
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="N99" s="2" t="n"/>
+      <c r="N99" s="2" t="inlineStr">
+        <is>
+          <t>Renumbered IN-32 -&gt; IN-39 on 2026-10-28: IN-32 was used twice.</t>
+        </is>
+      </c>
       <c r="O99" s="2" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>IN-33</t>
+          <t>IN-40</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -7365,13 +7369,17 @@
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="N100" s="2" t="n"/>
+      <c r="N100" s="2" t="inlineStr">
+        <is>
+          <t>Renumbered IN-33 -&gt; IN-40 on 2026-10-28: IN-33 was used twice.</t>
+        </is>
+      </c>
       <c r="O100" s="2" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>OX-30</t>
+          <t>OX-31</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
@@ -7432,7 +7440,7 @@
       </c>
       <c r="N101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26: OxyControl Drive(Reset := OxyPump.Command.Reset OR OxyPump.AlarmAck.DriveError): the HMI's Reset oxy pump or acknowledging the DriveError alarm (also Acknowledge all) sends 0x0080 for 0.5 s; the alarm clears once ETA has no fault. HMI overview shows the drive fault (LFT) and a Reset oxy pump button (PR #13). To be tested in the sim.</t>
+          <t>2026-10-26: OxyControl Drive(Reset := OxyPump.Command.Reset OR OxyPump.AlarmAck.DriveError): the HMI's Reset oxy pump or acknowledging the DriveError alarm (also Acknowledge all) sends 0x0080 for 0.5 s; the alarm clears once ETA has no fault. HMI overview shows the drive fault (LFT) and a Reset oxy pump button (PR #13). To be tested in the sim. | Renumbered OX-30 -&gt; OX-31 on 2026-10-28: OX-30 was used twice.</t>
         </is>
       </c>
       <c r="O101" s="2" t="inlineStr">
@@ -7441,8 +7449,560 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>IN-41</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>Inlet</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>Inconsistency</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>Heartbeat loss stops the pump: LIC01 counts a stopped pump</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>SCD 7664-017-1 sheet 2: the #HRTB fault (UI-100) is ORed with HMI STOP and resets the start latch, so the pump STOPS on heartbeat loss (no HOLD). The PLC and CAS FD Inlet (DEC9, fault table) assume HOLD at a preset speed: a pump without link stays in LIC01's total at its last speed and the pumps in REMOTE do not compensate. With the SCD behaviour the PLC overestimates the total by one pump (about 74 rpm) and the level falls uncompensated, like an undetected trip; with all links lost all three pumps stop and the pen loses its over-height within minutes. CasFramoSim models HOLD at 88 rpm, so the simulator hides it.</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>Framo 7664-017-1 sheet 2; CAS FD Inlet DEC9, fault table; FB.Inlet.InletPumpSet, PenLevelControl; CasFramoSim; IN-02, IN-36</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t>Preferred (asked Framo 2026-10-28): local mode in the PCC: on heartbeat fault keep running on the last good CAS setpoint (sample-and-hold, limited 40-130 rpm, A-selector before M01-U56), remove the HRTB fault from the stop OR, new status bit LOCAL MODE ACTIVE, optional time limit T_local, automatic return to the CAS setpoint when the link is back; no release valve opening or re-evacuation on heartbeat loss. Fallback: count a pump without link as 0 rpm in LIC01 and make CasFramoSim stop the pump on heartbeat loss.</t>
+        </is>
+      </c>
+      <c r="I102" s="2" t="inlineStr">
+        <is>
+          <t>Framo / Internal</t>
+        </is>
+      </c>
+      <c r="J102" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K102" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L102" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M102" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="N102" s="2" t="n"/>
+      <c r="O102" s="2" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>IN-42</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>Inlet</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>PLC gap</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>Pump state derived from Framo status bits</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>Framo has removed the pump state machine (meeting 2026-10-28). PLC functions built on InletPump.State need a state the PLC derives itself: PRG.FramoDataProcessing (reads the PumpState* flags), InletControl (start/stop/reset timers), InletPumpSet / PenLevelControl (R1/R2: counted / controlled), PumpCount (candidates: not UNAVAILABLE / LOCKDOWN), oxygenation permit I1 (OX-32), HMI ENUM.InletPumpState, CasFramoSim. Proposed mapping (to confirm with the OPC UA list): UNAVAILABLE = no link OR NOT DRIVE IN REMOTE (Q27) OR DRIVE START INHIBIT (U03); LOCKDOWN = DRIVE TRIPPED (Q10) OR FAILED TO START (UA-011) OR an A alarm of sheet 4; AVAILABLE = DRIVE READY (Q65) AND NOT DRIVE RUNNING (Q02) AND NOT STARTING SEQU ACTIVE (UI-010); START = UI-010 OR (Q02 AND NOT READY TO REMOTE CNTRL (UI-013)); REMOTE = Q02 AND UI-013 AND REMOTE CONTROL (UY-012) given by CAS; STOP = Stop sent AND Q02; HOLD = none (or LOCAL MODE ACTIVE if IN-41 is accepted).</t>
+        </is>
+      </c>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>Framo 7664-017-1 sheets 2-4; PRG.FramoDataProcessing; FB.Inlet.InletControl, InletPumpSet, PumpCount; ENUM.InletPumpState; heimdall-cas-hmi tags.py; CasFramoSim; IN-34</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
+          <t>Keep ENUM.InletPumpState in the PLC and the HMI, derive it in FramoDataProcessing from the bits; add the REMOTE CONTROL output (UY-012). Ask Framo: which bits come over OPC UA, whether UI-013 needs UY-012 first, which faults need Reset, whether DRIVE READY is FALSE while running.</t>
+        </is>
+      </c>
+      <c r="I103" s="2" t="inlineStr">
+        <is>
+          <t>Framo / Internal</t>
+        </is>
+      </c>
+      <c r="J103" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K103" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L103" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M103" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="N103" s="2" t="n"/>
+      <c r="O103" s="2" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>IN-43</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>Inlet</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>Inconsistency</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>Start sequence timing and duplicate Start failed alarm</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>SCD: a start runs air evacuation until LSH-002A, then the drive starts at 40 rpm and READY TO REMOTE CNTRL comes 30 s after DRIVE RUNNING; Framo raises FAILED TO START (UA-011) after a time not given. The PLC raises its own 'Start failed' when the pump is still AVAILABLE 30 s after Start (a state that no longer exists) and tracks the starting pumps in LIC01 with about 87 rpm START speed (simulator the same). Two alarms for one fault with different times; PLC timers may trip before Framo's sequence is done.</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>Framo 7664-017-1 sheets 2-3; CAS FD Inlet fault table 'Start not acknowledged'; FB.Inlet.InletControl; CasFramoSim; IN-13</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>Use Framo's UA-011 as the start failure (drop or lengthen the PLC timer); ask Framo for the normal start duration and the UA-011 time; update CasFramoSim (evacuation time, 40 rpm, 30 s).</t>
+        </is>
+      </c>
+      <c r="I104" s="2" t="inlineStr">
+        <is>
+          <t>Framo / Internal</t>
+        </is>
+      </c>
+      <c r="J104" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K104" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L104" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M104" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="N104" s="2" t="n"/>
+      <c r="O104" s="2" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>IN-44</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>Inlet</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>PLC gap</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>Reset handshake without pump states</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>IN-29: the PLC holds Reset to the PCC until it sees HOLD / LOCKDOWN change, else warning FailedToReset after 2 x ResetExpectedTime. Without pump states there is no state change to wait for. SCD sheet 3: HMI RESET (M01-U11) clears the pump block YF and also sends a reset to the drive (Q11 'REST COMMAND TO DRIVE').</t>
+        </is>
+      </c>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>Framo 7664-017-1 sheet 3; FB.Inlet.InletControl; InletPumpAlarmDUT.FailedToReset; IN-29, IN-42</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="inlineStr">
+        <is>
+          <t>Hold Reset until the fault bits (drive tripped, failed to start, A alarms) clear, with the same timeout; ask Framo edge or level on U11 and what it resets.</t>
+        </is>
+      </c>
+      <c r="I105" s="2" t="inlineStr">
+        <is>
+          <t>Framo / Internal</t>
+        </is>
+      </c>
+      <c r="J105" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K105" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L105" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M105" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="N105" s="2" t="n"/>
+      <c r="O105" s="2" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>IN-45</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>Inlet</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>Missing info</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>Vacuum chamber: gas build-up trips the pump (PUMP FSL)</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>SCD sheet 2: LSL-001A dry (after a delay) or sensor deviation UA-001A (LSH wet, LSL dry) gives PUMP FSL (signal 100) to the FSL terminal of pump block M01: the pump trips, probably latched (YF, needs HMI RESET). The P&amp;ID appears to show the client oxygenators feeding the inlet lines, so undissolved O2 can collect in the vacuum chamber at the high point and trip a running pump; the ejector would also vent O2-rich gas. Release valve UY-004A (SBV, terminals XH/XL/XGH/XGL/FSL/BCL) opens on HMI STOP; the meaning of its FSL and BCL, the fail positions of UY-003 / UY-004 and whether the heartbeat fault also opens it are not given.</t>
+        </is>
+      </c>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>Framo 7664-017-1 sheet 2; Framo 7664-021-1; IN-12, IN-38, IN-41; HAZID oksygen</t>
+        </is>
+      </c>
+      <c r="H106" s="2" t="inlineStr">
+        <is>
+          <t>Ask Framo: automatic re-evacuation while running (UY-003 on LSL dry, warning, trip only if LSL stays dry) instead of a trip; FSL delay and latching; gas volume between LSH and LSL; ejector exhaust location (O2); FSL / BCL on the release valve; fail positions; does the pen drain back through the pump when the siphon is broken; compressed air pressure, consumption and simultaneous evacuation of three units; valve and switch signals over OPC UA.</t>
+        </is>
+      </c>
+      <c r="I106" s="2" t="inlineStr">
+        <is>
+          <t>Framo</t>
+        </is>
+      </c>
+      <c r="J106" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K106" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L106" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M106" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="N106" s="2" t="n"/>
+      <c r="O106" s="2" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>OX-32</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>Oxygen</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>PLC gap</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>Oxygenation permit I1 without a REMOTE state</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>PLC and CAS FD Oxygen: a line may add oxygen only while its inlet pump is in REMOTE with a live heartbeat (Inlet[i].InletPump.Status.OxyPermit, I1; FD Oxygen OI23). Framo has removed the pump states (IN-42), so REMOTE must be redefined from the status bits, and with a local mode (IN-41) it must be decided whether oxygenation may continue while the link is down.</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>CAS FD Oxygen I1, OI23; FB.Inlet.InletControl (OxyPermit); IN-41, IN-42</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="inlineStr">
+        <is>
+          <t>Permit = DRIVE RUNNING AND READY TO REMOTE CNTRL AND DRIVE IN REMOTE AND link OK (as IN-42's REMOTE); decide oxygenation in local mode (proposal: stop, as today on link loss).</t>
+        </is>
+      </c>
+      <c r="I107" s="2" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="J107" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K107" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L107" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M107" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="N107" s="2" t="n"/>
+      <c r="O107" s="2" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>OX-33</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>Oxygen</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>Oxygenation not restored after a PLC restart</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>Seen 2026-10-28: after the PLC restart around the password change the pen and inlet pumps ran again but oxygenation stayed off (Pen.Status.OxygenOn FALSE, OIC01 output 0, pen O2 7.45 mg/L under the 8.0 setpoint and falling) until Oxygen Start was given. By design (FD Oxygen S1): OxygenOn is not retained and Oxygen Start is an operator pulse. [FD] table 2.2 asks auto-restart, sequence 3 after the inlet pumps (FD Oxygen OI23).</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>CAS FD Oxygen S1, S3, OI23; FB.Inlet.PenOxygenControl / PenSequence; heimdall-cas-hmi commands.py (Pen.Command.OxygenStart)</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>A: as today (operator always gives Oxygen Start); B (recommended): retain OxygenOn, restart oxygenation after the inlet pumps when it was on before the restart; C: oxygenation follows Pen Start.</t>
+        </is>
+      </c>
+      <c r="I108" s="2" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="J108" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K108" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L108" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M108" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="N108" s="2" t="n"/>
+      <c r="O108" s="2" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>GEN-05</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>Code bug</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>Framo OPC UA data sources lost after the PLC security change</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28, after the PLC user passwords were changed and anonymous OPC UA access to the PLC was disabled: the PLC's data sources Framo_1..3 did not connect to the simulated Framo servers. The simulator side was fine: opc.tcp://10.1.2.150:4841-4843 answered, SecurityPolicy None, Anonymous and UserName offered, servers up since 2026-10-27 12:11 UTC (no restart). The outgoing client does not use the changed passwords, so the trigger was probably the restart around the change (client not reconnecting, as IN-40) or a security / certificate setting. Later the same day the data sources were connected again; the oxygen pump drives then showed a latched drive fault (last fault 150 EtHF), cleared by acknowledging. Root cause not found; the data source status and the device log were not read.</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>PFC200_Sim Data Sources Framo_1..3; CODESYS device log (CmpOPCUAClient); IN-40</t>
+        </is>
+      </c>
+      <c r="H109" s="2" t="inlineStr">
+        <is>
+          <t>Next time: read the data source communication status and the device log before restarting anything; consider a data-source freshness watchdog with reconnect, like IN-40 for the Modbus masters.</t>
+        </is>
+      </c>
+      <c r="I109" s="2" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="J109" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K109" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L109" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M109" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="N109" s="2" t="n"/>
+      <c r="O109" s="2" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O101"/>
+  <autoFilter ref="A1:O109"/>
   <conditionalFormatting sqref="A2:O500">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>$L2="Fixed"</formula>

</xml_diff>

<commit_message>
CAS register: IN-46 Framo OPC UA endpoints from config, GEN-06 PLC CPU load and state in GVLMain
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAS/Outstanding items.xlsx
+++ b/CAS/Outstanding items.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Outstanding items'!$A$1:$O$109</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Outstanding items'!$A$1:$O$111</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O109"/>
+  <dimension ref="A1:O111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8001,8 +8001,146 @@
       <c r="N109" s="2" t="n"/>
       <c r="O109" s="2" t="n"/>
     </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>IN-46</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>Inlet</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>PLC gap</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>Framo OPC UA server addresses from config variables</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>The OPC UA endpoints of the Framo controllers are fixed in the Data Sources Framo_1..3 (opc.tcp://&lt;ip&gt;:4841-4843 for the CAS plant simulator). Moving between the simulator and the real Framo PCCs, or a new simulator address, needs a project edit and a download. Sigurd wants the IP (and port) per pump as config variables that can be changed at runtime, like CommonRIOConfig / InletRIOConfig for the Modbus devices. Sigurd has done this in another project, to be used as the template.</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>PFC200_Sim Data Sources Framo_1..3; GVL ConfigValues; simulation docs (point the PLC at a CAS plant)</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="inlineStr">
+        <is>
+          <t>Look at Sigurd's other project for the method (runtime change of the data source endpoint, or an own OPC UA client FB fed from config); add e.g. FramoConfig[0..2].IP / Port in ConfigValues; reconnect when the value changes; HMI / docs to show the active endpoint. Data Sources are edited by Sigurd, not via MCP.</t>
+        </is>
+      </c>
+      <c r="I110" s="2" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="J110" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K110" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L110" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M110" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="N110" s="2" t="n"/>
+      <c r="O110" s="2" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>GEN-06</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>PLC gap</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>PLC CPU load and state in GVLMain (OPC UA)</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd wants to see the PLC's CPU load and its state over the OPC UA interface (HMI, monitoring). Today only the CODESYS task monitor / htop show load (IN-21: CPU 86 %, load average 2.6 on 2026-10-23), and nothing in GVLMain tells whether the application runs, has been restarted or is overloaded.</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>IN-21; GVLMain; heimdall-cas-hmi</t>
+        </is>
+      </c>
+      <c r="H111" s="2" t="inlineStr">
+        <is>
+          <t>Add e.g. GVLMain.PlcStatus: CpuLoad [%] (runtime CPU load function, check the library on the PFC200), per-task cycle time avg / max and jitter (IEC task info), application state (run / stop / exception), uptime since start, first-cycle / restart counter, PLC time; HMI tile and trend later.</t>
+        </is>
+      </c>
+      <c r="I111" s="2" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="J111" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K111" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L111" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M111" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="N111" s="2" t="n"/>
+      <c r="O111" s="2" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O109"/>
+  <autoFilter ref="A1:O111"/>
   <conditionalFormatting sqref="A2:O500">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>$L2="Fixed"</formula>

</xml_diff>

<commit_message>
CAS register: IN-47 pump count / rotation / auto start timers and next pump to GVLMain and HMI
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAS/Outstanding items.xlsx
+++ b/CAS/Outstanding items.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Outstanding items'!$A$1:$O$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Outstanding items'!$A$1:$O$112</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O111"/>
+  <dimension ref="A1:O112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8139,8 +8139,77 @@
       <c r="N111" s="2" t="n"/>
       <c r="O111" s="2" t="n"/>
     </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>IN-47</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>Inlet</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>PLC gap</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>Pump count / rotation / auto start not visible: timers and next pump</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>Operator request 2026-10-28: when LIC01's share reaches the pump-count limits it is unclear how long until a pump is stopped or started, and which one; the same for the automatic start of pumps and for rotation. FB.Inlet.PumpCount keeps all of it internal: RemoveTimer (IN: count active AND Total / (LevelPumps - 1) &lt;= PumpTargetSpeed, PT PumpRemoveDelay), AddTimer (IN: count active AND an idle candidate AND Share &gt;= PumpAddSpeed, PT PumpAddDelay), RunTimer[i] (time in REMOTE, PT PumpCycleTime, rotation), StartFailTimer[i] (PT StartupTime + 10 s), the choice by Sequence (stop: most running days among the wanted pumps in REMOTE; start: fewest among the idle candidates in AVAILABLE), and CountActive (PenStart AND LevelInAuto AND Settled AND NOT Rotating). Only PumpsWanted and PumpRotationActive reach PenInletSupervisorDUT, so the HMI cannot show a countdown without copying the logic (it would drift from the PLC).</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>FB.Inlet.PumpCount; DUT PenInletSupervisorDUT; GVLMain.PenInletSupervisor; heimdall-cas-hmi; IN-15, IN-31; CAS FD Inlet sec. pump count</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>PLC first (next CODESYS batch), then the HMI card. PumpCount writes to PenInletSupervisorDUT (status only, no retain): CountActive : BOOL and CountBlocked : WORD (bits: pen not started, LIC01 not in auto, pumps changing / not settled, rotation running); per action StopPending / StartPending : BOOL (timer IN), StopIn / StartIn : TIME (PT - ET while pending), StopNext / StartNext : UINT (inlet 1..3 that would be chosen now, 0 = none), StopCondition / StartCondition : REAL (Total / (LevelPumps - 1) and Share, to show against PumpTargetSpeed / PumpAddSpeed); rotation: RotationIn : TIME (shortest PumpCycleTime - RunTimer[i].ET of the wanted pumps in REMOTE), RotationOut / RotationIn pump numbers, standby available : BOOL; auto start per pump: StartWanted[i], StartTimeout[i] : TIME (StartupTime + 10 s - StartFailTimer[i].ET while AVAILABLE and wanted), StartFailed[i]. HMI: a 'Pump supervisor' card on the overview and inlet page, e.g. 'Stop pump 2 in 12:40 (others would run 81 &lt; 85 rpm)', 'Start pump 3 in 1:15 (share 117 &gt;= 115 rpm)', 'Rotation: pump 1 -&gt; pump 3 in 18 h', 'Auto start pump 2: waiting for REMOTE, start failure in 0:45', or why the count is paused. FD Inlet pump-count section to describe the new status.</t>
+        </is>
+      </c>
+      <c r="I112" s="2" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="J112" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K112" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L112" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M112" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="N112" s="2" t="n"/>
+      <c r="O112" s="2" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O111"/>
+  <autoFilter ref="A1:O112"/>
   <conditionalFormatting sqref="A2:O500">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>$L2="Fixed"</formula>

</xml_diff>

<commit_message>
CAS register: items from Lekang, Aquaculture Engineering (3rd ed. 2020)
New: OX-34 emergency oxygenation independent of the inlet pumps, IN-48 minimum exchange set
by CO2, OX-35 O2 per line vs water flow, OX-36 total gas pressure / N2, OX-37 injection point,
OUT-26 outlet velocity at low exchange. Literature notes on IN-23, IN-09, OX-06, OX-13.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAS/Outstanding items.xlsx
+++ b/CAS/Outstanding items.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Outstanding items'!$A$1:$O$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Outstanding items'!$A$1:$O$118</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O112"/>
+  <dimension ref="A1:O118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1404,7 +1404,11 @@
           <t>FD Tabell 7; FD-02 alarm list</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>[Lekang] O.-I. Lekang, Aquaculture Engineering, 3rd ed., Wiley 2020 (file 'Odd-ivar Lekang - Aquaculture Engineering-Blackwell Pub (2013).pdf' in Dokumenter\Litteratur) p. 443: level by pressure or ultrasound / radar with separate high and low alarms against overflow and water shortage; p. 476-477: gas at a siphon crest blocks the flow - supervise the vacuum chambers (level / vacuum) as well (IN-45).</t>
+        </is>
+      </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Internal</t>
@@ -2378,7 +2382,11 @@
           <t>FD rev B 'Motor-Forrigling', Tabell T3/T4; CAS FD Inlet OI16; FB.Inlet.InletSupervisor (PenStart)</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>[Lekang] O.-I. Lekang, Aquaculture Engineering, 3rd ed., Wiley 2020 (file 'Odd-ivar Lekang - Aquaculture Engineering-Blackwell Pub (2013).pdf' in Dokumenter\Litteratur) p. 449-451: generator start on power failure, battery backup (UPS) for the control and monitoring system, automatic restart, weekly test of the alarm chain and periodic test of emergency O2 and generator. Add UPS for PLC / HMI / alarm path to the scope check.</t>
+        </is>
+      </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
           <t>Internal</t>
@@ -3257,7 +3265,7 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Decide limits, sensors, latching</t>
+          <t>Decide limits, sensors, latching | [Lekang] O.-I. Lekang, Aquaculture Engineering, 3rd ed., Wiley 2020 (file 'Odd-ivar Lekang - Aquaculture Engineering-Blackwell Pub (2013).pdf' in Dokumenter\Litteratur) p. 225: inlet water to the fish volume not above about 150-200 % saturation; see OX-35 for the per-line limit against the water flow.</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -3726,7 +3734,11 @@
           <t>FD Tabell 15</t>
         </is>
       </c>
-      <c r="H47" s="2" t="inlineStr"/>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>[Lekang] O.-I. Lekang, Aquaculture Engineering, 3rd ed., Wiley 2020 (file 'Odd-ivar Lekang - Aquaculture Engineering-Blackwell Pub (2013).pdf' in Dokumenter\Litteratur) p. 226, 231, 304, 431, 434: one O2 meter is not representative (use several), control on a representative low point / the outlet (about 7 mg/L in tanks), wrong readings are worse than none, fouling makes optical O2 read low; define cleaning / calibration intervals and flag drifting sensors.</t>
+        </is>
+      </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
           <t>Internal</t>
@@ -8208,8 +8220,422 @@
       <c r="N112" s="2" t="n"/>
       <c r="O112" s="2" t="n"/>
     </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>OX-34</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>Oxygen</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>Missing hardware</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="inlineStr">
+        <is>
+          <t>Emergency oxygenation independent of the inlet pumps</t>
+        </is>
+      </c>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>All oxygenation in CAS depends on the inlet pumps (oxygenators in the inlet lines, permit I1). If all pumps stop, pen O2 falls about 10 mg/L per hour at full biomass (196 kg/h consumption in 20 000 m3), so about 15-20 min from setpoint to a critical level. Literature: the standard design has emergency diffusers in the production unit fed directly from the O2 supply for when the water supply stops, opened automatically by the PLC on low O2, with siren / phone alarm, and tested at fixed intervals.</t>
+        </is>
+      </c>
+      <c r="G113" s="2" t="inlineStr">
+        <is>
+          <t>[Lekang] O.-I. Lekang, Aquaculture Engineering, 3rd ed., Wiley 2020 (file 'Odd-ivar Lekang - Aquaculture Engineering-Blackwell Pub (2013).pdf' in Dokumenter\Litteratur) p. 229, 450-451, 492; FD Oxygen (emergency oxygenation [FD] 3.2.5 out of scope); OX-26, IN-41</t>
+        </is>
+      </c>
+      <c r="H113" s="2" t="inlineStr">
+        <is>
+          <t>Emergency diffusers (or another pump-independent O2 path) fed from the Normex supply through a fail-open / PLC valve; PLC opens it on pen O2 low-low or when no inlet pump runs; alarm to siren and phone; periodic test. Needs a decision on hardware and scope (Normex / Project).</t>
+        </is>
+      </c>
+      <c r="I113" s="2" t="inlineStr">
+        <is>
+          <t>Project / Normex</t>
+        </is>
+      </c>
+      <c r="J113" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K113" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L113" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M113" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="N113" s="2" t="n"/>
+      <c r="O113" s="2" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>IN-48</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>Inlet</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t>Minimum water exchange set by CO2 at high biomass</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>Literature: once pure O2 is added, CO2, solids and NH3 rather than O2 set the water need; CO2 above 10-15 mg/L is suboptimal for salmonids; CO2 stripping needs 3-10 volumes of air per volume of water, not realistic at CAS flows, so the exchange rate is the only CO2 control. Estimate (ratio 1.375 g CO2 per g O2, a common figure NOT from the book; seawater buffering makes it an overestimate): 196 kg/h O2 at 1000 t gives about 270 kg/h CO2, i.e. a rise of about 8 mg/L at 34 000 m3/h (O-35), 13.5 mg/L at 20 000 (O-60) and 17 mg/L at 16 000 (S-75), on top of the intake CO2. O-60 and S-75 may give too little water at full biomass. CAS sets the exchange by operating mode and level only; no CO2 measurement in use (a CO2 word exists in CommonRIO).</t>
+        </is>
+      </c>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>[Lekang] O.-I. Lekang, Aquaculture Engineering, 3rd ed., Wiley 2020 (file 'Odd-ivar Lekang - Aquaculture Engineering-Blackwell Pub (2013).pdf' in Dokumenter\Litteratur) p. 204, 218, 221, 261-262, 303-304; FD-01 Tabell 10 (modes); design basis</t>
+        </is>
+      </c>
+      <c r="H114" s="2" t="inlineStr">
+        <is>
+          <t>Measure CO2 (and TGP) in the pen; define a minimum exchange per biomass (block or warn on O-60 / S-75 above a biomass limit); verify the CO2 figure with a seawater carbonate calculation.</t>
+        </is>
+      </c>
+      <c r="I114" s="2" t="inlineStr">
+        <is>
+          <t>Project / Customer</t>
+        </is>
+      </c>
+      <c r="J114" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K114" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L114" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M114" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="N114" s="2" t="n"/>
+      <c r="O114" s="2" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>OX-35</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>Oxygen</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>PLC gap</t>
+        </is>
+      </c>
+      <c r="E115" s="2" t="inlineStr">
+        <is>
+          <t>O2 added per line not limited against the line's water flow</t>
+        </is>
+      </c>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>Literature: water entering the fish volume should not be above about 150-200 % O2 saturation. OxyControl limits each line to FlowMax 104.2 kg/h gas regardless of the inlet pump's speed. At 40 rpm (about 6 000 m3/h if flow scales with speed) a full line gives about 83 kg/h dissolved, about +13.5 mg/L, i.e. about 230 % saturation in that inlet stream.</t>
+        </is>
+      </c>
+      <c r="G115" s="2" t="inlineStr">
+        <is>
+          <t>[Lekang] O.-I. Lekang, Aquaculture Engineering, 3rd ed., Wiley 2020 (file 'Odd-ivar Lekang - Aquaculture Engineering-Blackwell Pub (2013).pdf' in Dokumenter\Litteratur) p. 225; FB.OxySystem.OxyControl (FlowMax); OIC01 sharing; OX-06</t>
+        </is>
+      </c>
+      <c r="H115" s="2" t="inlineStr">
+        <is>
+          <t>Limit each line's O2 flow to k x its inlet water flow (from MotorVelocity, e.g. so the inlet stays &lt;= 150 % saturation) and give the excess to the other lines; together with the high-high O2 shut-off (OX-06).</t>
+        </is>
+      </c>
+      <c r="I115" s="2" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="J115" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K115" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L115" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M115" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="N115" s="2" t="n"/>
+      <c r="O115" s="2" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>OX-36</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>Oxygen</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>Missing hardware</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t>Total gas pressure / N2 supersaturation not monitored</t>
+        </is>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>Literature: N2 should stay below about 100.5 % saturation, problems in salmonids from about 102 %; total gas pressure above 100 % may be harmful. Pure O2 raises TGP but not N2; N2 supersaturation comes from air drawn into the suction side of a pump ('false air', also cavitation), air added deeper than 1-2 m, and low-purity O2 from an ageing PSA generator (80-85 %) injected under pressure. CAS has a TotalGasPressure word in CommonRIO but no TGP alarm or shut-off; the O2 supply type (LOX / PSA) is open (OX-02).</t>
+        </is>
+      </c>
+      <c r="G116" s="2" t="inlineStr">
+        <is>
+          <t>[Lekang] O.-I. Lekang, Aquaculture Engineering, 3rd ed., Wiley 2020 (file 'Odd-ivar Lekang - Aquaculture Engineering-Blackwell Pub (2013).pdf' in Dokumenter\Litteratur) p. 32, 42, 212, 221, 224, 235, 435; CommonRIO TotalGasPressure; OX-02, OX-06</t>
+        </is>
+      </c>
+      <c r="H116" s="2" t="inlineStr">
+        <is>
+          <t>TGP sensor in the pen (and ideally after an oxygenator) with alarm at about 100.5-102 % N2-equivalent; if the supply is PSA, an O2 purity signal with alarm; check the ejector / vacuum chamber cannot draw air into the pump suction.</t>
+        </is>
+      </c>
+      <c r="I116" s="2" t="inlineStr">
+        <is>
+          <t>Project / Normex</t>
+        </is>
+      </c>
+      <c r="J116" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K116" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L116" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M116" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="N116" s="2" t="n"/>
+      <c r="O116" s="2" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>OX-37</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>Oxygen</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>Physical</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>Missing info</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t>Oxygen injection point vs vacuum chamber and inlet pump</t>
+        </is>
+      </c>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>Literature: after supersaturating, avoid free surfaces and bends and keep the pipe to the fish short; O2 bubbles into a pump cause cavitation. In CAS the side-stream oxygenator returns into the inlet line; the Framo P&amp;ID 7664-021-1 shows the vacuum chamber at the high point of each inlet line. If the O2-rich stream enters upstream of the vacuum chamber or a pump, gas comes out at the free surface in the chamber (lost O2, O2-rich vent, PUMP FSL trips, IN-45).</t>
+        </is>
+      </c>
+      <c r="G117" s="2" t="inlineStr">
+        <is>
+          <t>[Lekang] O.-I. Lekang, Aquaculture Engineering, 3rd ed., Wiley 2020 (file 'Odd-ivar Lekang - Aquaculture Engineering-Blackwell Pub (2013).pdf' in Dokumenter\Litteratur) p. 224, 230; Framo 7664-021-1; IN-45</t>
+        </is>
+      </c>
+      <c r="H117" s="2" t="inlineStr">
+        <is>
+          <t>Confirm with Framo / Normex / Chucaotech where the oxygenator outlet joins the inlet line: it must be downstream of the inlet pump and of the vacuum chamber, with no free surface after it.</t>
+        </is>
+      </c>
+      <c r="I117" s="2" t="inlineStr">
+        <is>
+          <t>Framo / Normex</t>
+        </is>
+      </c>
+      <c r="J117" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K117" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L117" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M117" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="N117" s="2" t="n"/>
+      <c r="O117" s="2" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>OUT-26</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>Outlet</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>Physical</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>Outlet velocity too low at low exchange (sedimentation, fouling)</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>Literature: velocity in outlet pipes above 0.3 m/s to avoid settling (below 1.5 m/s to avoid breaking particles), and above 0.3-0.4 m/s through screen openings against fouling. With D_out 5.5 m (A 23.8 m2) the mean velocity is about 0.40 m/s at 34 000 m3/h (O-35) but about 0.19 m/s at 16 000 m3/h (S-75) and 0.23 m/s at 20 000 (O-60) with the damper fully open. The damper openings per mode (OUT-10, sim 2.4.11: 100/44/28/22 %) raise the velocity in the damper opening, but not in the pipe and screen upstream.</t>
+        </is>
+      </c>
+      <c r="G118" s="2" t="inlineStr">
+        <is>
+          <t>[Lekang] O.-I. Lekang, Aquaculture Engineering, 3rd ed., Wiley 2020 (file 'Odd-ivar Lekang - Aquaculture Engineering-Blackwell Pub (2013).pdf' in Dokumenter\Litteratur) p. 312-313; design basis [pen.D_out]; OUT-10</t>
+        </is>
+      </c>
+      <c r="H118" s="2" t="inlineStr">
+        <is>
+          <t>Check the velocity at the fish screen and in the outlet pipe per mode with Servi / Østerbø; consider screen area / cleaning interval for the low-flow modes.</t>
+        </is>
+      </c>
+      <c r="I118" s="2" t="inlineStr">
+        <is>
+          <t>Servi / Østerbø</t>
+        </is>
+      </c>
+      <c r="J118" s="2" t="inlineStr">
+        <is>
+          <t>Sigurd</t>
+        </is>
+      </c>
+      <c r="K118" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L118" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M118" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="N118" s="2" t="n"/>
+      <c r="O118" s="2" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O112"/>
+  <autoFilter ref="A1:O118"/>
   <conditionalFormatting sqref="A2:O500">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>$L2="Fixed"</formula>

</xml_diff>